<commit_message>
Update dashboard data 2026-04-13 17:07:04
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkCode\AI_Digest\data\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AEA4AB-9FF3-4C82-A2C0-DC5A1D0CAF91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0CABA7-8CDB-4305-9E52-F4B6D7A71D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4F6CCF54-37E5-4816-9B51-3E2CFD892ED8}"/>
   </bookViews>
@@ -371,31 +371,7 @@
     <t/>
   </si>
   <si>
-    <t>【整体来店】
-ICE+NEV累计来店 49,254；当日来店 6,584
-① ICE累计来店 19,154；当日来店 2,391
-② NEV累计来店 30,100；当日来店 4,193</t>
-  </si>
-  <si>
     <t>请查收4月1-12日的来店业绩：</t>
-  </si>
-  <si>
-    <t>1、ICE+NEV合计来店：12日来店量6,584，1-12日来店总量42,640，同比4.8%，环比2.7%</t>
-  </si>
-  <si>
-    <t>2、ICE（油车）来店：管控目标：12日来店目标0，来店量2,068，达成率-；月累来店目标0，来店量16,742，达成率-；月度目标0，达成率-；同比-58.1%，环比-36.2%；必达目标，达成率-</t>
-  </si>
-  <si>
-    <t>3、NEV来店：12日来店量4,193，1-12日来店总量25,898，环比69.6%</t>
-  </si>
-  <si>
-    <t>—自然来店9,518，达成率-，同比-51.9%，环比-33.9%；</t>
-  </si>
-  <si>
-    <t>—开拓渠道来店6,130，达成率-，同比-65.8%，环比-40.9%；</t>
-  </si>
-  <si>
-    <t>—保有客户来店1,094，达成率-，同比-51.2%，环比-26.3%</t>
   </si>
   <si>
     <t>累计实绩：49254（累计同比9%）</t>
@@ -435,6 +411,30 @@
   </si>
   <si>
     <t>统计周期4.1-4.12</t>
+  </si>
+  <si>
+    <t>【整体来店】
+ICE+NEV累计来店 49,254；当日来店 6,583
+① ICE累计来店 19,154；当日来店 2,382
+② NEV累计来店 30,100；当日来店 4,201</t>
+  </si>
+  <si>
+    <t>1、ICE+NEV合计来店：12日来店量6,583，1-12日来店总量49,252，同比8.7%，环比10.8%</t>
+  </si>
+  <si>
+    <t>2、ICE（油车）来店：管控目标：12日来店目标0，来店量2,382，达成率-；月累来店目标0，来店量19,154，达成率-；月度目标0，达成率-；同比-57.0%，环比-31.7%；必达目标，达成率-</t>
+  </si>
+  <si>
+    <t>3、NEV来店：12日来店量4,201，1-12日来店总量30,098，环比83.3%</t>
+  </si>
+  <si>
+    <t>—自然来店10,817，达成率-，同比-50.1%，环比-29.4%；</t>
+  </si>
+  <si>
+    <t>—开拓渠道来店7,110，达成率-，同比-65.0%，环比-36.0%；</t>
+  </si>
+  <si>
+    <t>—保有客户来店1,227，达成率-，同比-50.9%，环比-23.4%</t>
   </si>
 </sst>
 </file>
@@ -718,7 +718,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -1117,19 +1117,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1139,7 +1126,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1588,21 +1575,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="57" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="57" fontId="24" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1621,19 +1593,43 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="57" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="57" fontId="24" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1641,7 +1637,7 @@
     <cellStyle name="百分比" xfId="1" builtinId="5"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="93">
+  <dxfs count="49">
     <dxf>
       <font>
         <color theme="0"/>
@@ -1908,16 +1904,6 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
           <bgColor theme="1"/>
         </patternFill>
       </fill>
@@ -1969,436 +1955,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -21863,6 +21419,678 @@
     </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>55559</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>31749</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>269877</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>426860</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="12" name="组合 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42299510-F87B-4D0F-AD9A-BC7A81105E14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="55559" y="31749"/>
+          <a:ext cx="1776418" cy="395111"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="1531943" cy="395111"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="13" name="组合 12">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAA9FBE3-E551-B6D0-5B1E-75B53B586733}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="1531943" cy="395111"/>
+            <a:chOff x="0" y="0"/>
+            <a:chExt cx="1243417" cy="395111"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="15" name="矩形 14">
+              <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBFB41C9-E2DF-05F4-C67A-3E2C8E709520}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="297581" y="39511"/>
+              <a:ext cx="945836" cy="333552"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr"/>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:ea typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:cs typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                </a:rPr>
+                <a:t>返回目录</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="16" name="椭圆 15">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5ACC7541-39AD-C5FC-9160-19D3B9C637CC}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="380773" cy="395111"/>
+            </a:xfrm>
+            <a:prstGeom prst="ellipse">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="14" name="图片 13">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBB87CB5-96E3-916D-C255-3B9FDB318FF3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr preferRelativeResize="0"/>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="87507" y="32927"/>
+            <a:ext cx="325247" cy="329259"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:miter lim="800000"/>
+                <a:headEnd/>
+                <a:tailEnd/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>55559</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>31749</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>269877</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>426860</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="22" name="组合 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B66637FC-C6D1-4113-AC65-AFA63C820B3B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="55559" y="31749"/>
+          <a:ext cx="1776418" cy="395111"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="1531943" cy="395111"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="23" name="组合 22">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98EAFCBB-52A8-61FB-6497-8E1634F9029C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="1531943" cy="395111"/>
+            <a:chOff x="0" y="0"/>
+            <a:chExt cx="1243417" cy="395111"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="25" name="矩形 24">
+              <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E3D8AA6-E74F-219A-904A-C3ACFFD3903F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="297581" y="39511"/>
+              <a:ext cx="945836" cy="333552"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr"/>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:ea typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:cs typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                </a:rPr>
+                <a:t>返回目录</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="26" name="椭圆 25">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BB31080-209E-0CCB-6CAE-4A4857D00F90}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="380773" cy="395111"/>
+            </a:xfrm>
+            <a:prstGeom prst="ellipse">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="24" name="图片 23">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6121886C-E07E-84E4-DDEC-6D02FCD765BF}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr preferRelativeResize="0"/>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="87507" y="32927"/>
+            <a:ext cx="325247" cy="329259"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:miter lim="800000"/>
+                <a:headEnd/>
+                <a:tailEnd/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>55559</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>31749</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>269877</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>426860</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="27" name="组合 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35C2B02B-95A0-4F9B-85D9-6897CB34E83D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="55559" y="31749"/>
+          <a:ext cx="1776418" cy="395111"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="1531943" cy="395111"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="28" name="组合 27">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92721AC2-6227-FD3B-0933-BA21388FB454}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="1531943" cy="395111"/>
+            <a:chOff x="0" y="0"/>
+            <a:chExt cx="1243417" cy="395111"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="30" name="矩形 29">
+              <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2092ABCA-A3A1-AFF4-BA2C-916163E5674D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="297581" y="39511"/>
+              <a:ext cx="945836" cy="333552"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr"/>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:ea typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:cs typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                </a:rPr>
+                <a:t>返回目录</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="31" name="椭圆 30">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F22A6962-9B68-A471-62D0-3EE8876528CB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="380773" cy="395111"/>
+            </a:xfrm>
+            <a:prstGeom prst="ellipse">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="29" name="图片 28">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00C66637-6608-7E50-E487-1405C1CA31AE}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr preferRelativeResize="0"/>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="87507" y="32927"/>
+            <a:ext cx="325247" cy="329259"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:miter lim="800000"/>
+                <a:headEnd/>
+                <a:tailEnd/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -26523,19 +26751,19 @@
     <row r="1" ht="33.950000000000003" customHeight="1"/>
     <row r="2" ht="29.1" customHeight="1"/>
     <row r="29" spans="2:33">
-      <c r="C29" s="155"/>
-      <c r="D29" s="155"/>
-      <c r="E29" s="155"/>
-      <c r="F29" s="155"/>
-      <c r="Q29" s="156"/>
-      <c r="R29" s="156"/>
-      <c r="S29" s="156"/>
-      <c r="T29" s="156"/>
-      <c r="U29" s="156"/>
-      <c r="V29" s="156"/>
-      <c r="W29" s="156"/>
-      <c r="X29" s="156"/>
-      <c r="Y29" s="156"/>
+      <c r="C29" s="163"/>
+      <c r="D29" s="163"/>
+      <c r="E29" s="163"/>
+      <c r="F29" s="163"/>
+      <c r="Q29" s="164"/>
+      <c r="R29" s="164"/>
+      <c r="S29" s="164"/>
+      <c r="T29" s="164"/>
+      <c r="U29" s="164"/>
+      <c r="V29" s="164"/>
+      <c r="W29" s="164"/>
+      <c r="X29" s="164"/>
+      <c r="Y29" s="164"/>
     </row>
     <row r="30" spans="2:33">
       <c r="B30" s="132" t="s">
@@ -27286,19 +27514,19 @@
     </row>
     <row r="44" spans="2:33" s="144" customFormat="1"/>
     <row r="72" spans="2:33">
-      <c r="C72" s="157"/>
-      <c r="D72" s="157"/>
-      <c r="E72" s="157"/>
-      <c r="F72" s="157"/>
-      <c r="Q72" s="158"/>
-      <c r="R72" s="158"/>
-      <c r="S72" s="158"/>
-      <c r="T72" s="158"/>
-      <c r="U72" s="158"/>
-      <c r="V72" s="158"/>
-      <c r="W72" s="158"/>
-      <c r="X72" s="158"/>
-      <c r="Y72" s="158"/>
+      <c r="C72" s="165"/>
+      <c r="D72" s="165"/>
+      <c r="E72" s="165"/>
+      <c r="F72" s="165"/>
+      <c r="Q72" s="166"/>
+      <c r="R72" s="166"/>
+      <c r="S72" s="166"/>
+      <c r="T72" s="166"/>
+      <c r="U72" s="166"/>
+      <c r="V72" s="166"/>
+      <c r="W72" s="166"/>
+      <c r="X72" s="166"/>
+      <c r="Y72" s="166"/>
     </row>
     <row r="73" spans="2:33">
       <c r="B73" s="145" t="s">
@@ -27878,19 +28106,19 @@
     </row>
     <row r="85" s="149" customFormat="1"/>
     <row r="115" spans="2:33">
-      <c r="C115" s="157"/>
-      <c r="D115" s="157"/>
-      <c r="E115" s="157"/>
-      <c r="F115" s="157"/>
-      <c r="Q115" s="158"/>
-      <c r="R115" s="158"/>
-      <c r="S115" s="158"/>
-      <c r="T115" s="158"/>
-      <c r="U115" s="158"/>
-      <c r="V115" s="158"/>
-      <c r="W115" s="158"/>
-      <c r="X115" s="158"/>
-      <c r="Y115" s="158"/>
+      <c r="C115" s="165"/>
+      <c r="D115" s="165"/>
+      <c r="E115" s="165"/>
+      <c r="F115" s="165"/>
+      <c r="Q115" s="166"/>
+      <c r="R115" s="166"/>
+      <c r="S115" s="166"/>
+      <c r="T115" s="166"/>
+      <c r="U115" s="166"/>
+      <c r="V115" s="166"/>
+      <c r="W115" s="166"/>
+      <c r="X115" s="166"/>
+      <c r="Y115" s="166"/>
     </row>
     <row r="116" spans="2:33">
       <c r="B116" s="150" t="s">
@@ -28488,27 +28716,27 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="C33 I33 O33 U33 AA33">
-    <cfRule type="expression" dxfId="92" priority="4">
+    <cfRule type="expression" dxfId="48" priority="4">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C31:AF31">
-    <cfRule type="expression" dxfId="91" priority="2">
+    <cfRule type="expression" dxfId="47" priority="2">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C74:AF77">
-    <cfRule type="expression" dxfId="90" priority="5">
+    <cfRule type="expression" dxfId="46" priority="5">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C117:AF120">
-    <cfRule type="expression" dxfId="89" priority="3">
+    <cfRule type="expression" dxfId="45" priority="3">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D33:H36 J33:N36 P33:T37 V33:Z37 AB33:AF37 M37:N37">
-    <cfRule type="expression" dxfId="88" priority="1">
+    <cfRule type="expression" dxfId="44" priority="1">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -28578,13 +28806,13 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
-      <c r="AG2" s="154" t="s">
-        <v>104</v>
+      <c r="AG2" s="167" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:33" ht="15" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -28639,7 +28867,7 @@
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -28675,7 +28903,7 @@
     </row>
     <row r="8" spans="1:33" s="6" customFormat="1" ht="16.5" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -28711,7 +28939,7 @@
     </row>
     <row r="10" spans="1:33" ht="15" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -28766,7 +28994,7 @@
     </row>
     <row r="13" spans="1:33" ht="16.5" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -28785,7 +29013,7 @@
     </row>
     <row r="14" spans="1:33" ht="15" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -28804,7 +29032,7 @@
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -28876,7 +29104,7 @@
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
     </row>
-    <row r="19" spans="1:32" hidden="1">
+    <row r="19" spans="1:32" ht="14.25" hidden="1" customHeight="1">
       <c r="A19" s="5" t="e">
         <v>#REF!</v>
       </c>
@@ -28929,18 +29157,18 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22" spans="1:32" ht="30.95" customHeight="1" thickBot="1">
-      <c r="A22" s="159" t="s">
+      <c r="A22" s="160" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="160"/>
-      <c r="C22" s="160"/>
-      <c r="D22" s="160"/>
-      <c r="E22" s="160"/>
-      <c r="F22" s="160"/>
-      <c r="G22" s="160"/>
-      <c r="H22" s="160"/>
-      <c r="I22" s="160"/>
-      <c r="J22" s="161"/>
+      <c r="B22" s="161"/>
+      <c r="C22" s="161"/>
+      <c r="D22" s="161"/>
+      <c r="E22" s="161"/>
+      <c r="F22" s="161"/>
+      <c r="G22" s="161"/>
+      <c r="H22" s="161"/>
+      <c r="I22" s="161"/>
+      <c r="J22" s="162"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -28993,31 +29221,31 @@
         <v>16</v>
       </c>
       <c r="B24" s="20">
-        <v>6584</v>
+        <v>6583</v>
       </c>
       <c r="C24" s="20">
-        <v>42640</v>
+        <v>49252</v>
       </c>
       <c r="D24" s="21">
         <v>228521</v>
       </c>
       <c r="E24" s="22">
-        <v>0.18659116667614792</v>
+        <v>0.21552505021420351</v>
       </c>
       <c r="F24" s="22">
         <v>0.4</v>
       </c>
       <c r="G24" s="20">
-        <v>39991</v>
+        <v>44511</v>
       </c>
       <c r="H24" s="23">
-        <v>41529</v>
+        <v>44458</v>
       </c>
       <c r="I24" s="24">
-        <v>6.6239903978395187E-2</v>
+        <v>0.10651299678731108</v>
       </c>
       <c r="J24" s="22">
-        <v>2.6752389896217199E-2</v>
+        <v>0.10783211120608205</v>
       </c>
       <c r="K24" s="16"/>
       <c r="L24" s="16" t="s">
@@ -29036,31 +29264,31 @@
         <v>18</v>
       </c>
       <c r="B25" s="20">
-        <v>4193</v>
+        <v>4201</v>
       </c>
       <c r="C25" s="20">
-        <v>25898</v>
+        <v>30098</v>
       </c>
       <c r="D25" s="20">
         <v>100601</v>
       </c>
       <c r="E25" s="22">
-        <v>0.25743282869951589</v>
+        <v>0.29918191668074873</v>
       </c>
       <c r="F25" s="22">
         <v>0.4</v>
       </c>
       <c r="G25" s="20">
-        <v>695</v>
+        <v>793</v>
       </c>
       <c r="H25" s="20">
-        <v>15274</v>
+        <v>16422</v>
       </c>
       <c r="I25" s="20">
-        <v>36.263309352517986</v>
+        <v>36.954602774274903</v>
       </c>
       <c r="J25" s="22">
-        <v>0.69556108419536478</v>
+        <v>0.83278528802825469</v>
       </c>
       <c r="K25" s="17"/>
       <c r="L25" s="17"/>
@@ -29077,31 +29305,31 @@
         <v>20</v>
       </c>
       <c r="B26" s="20">
-        <v>2391</v>
+        <v>2382</v>
       </c>
       <c r="C26" s="20">
-        <v>16742</v>
+        <v>19154</v>
       </c>
       <c r="D26" s="20">
         <v>127920</v>
       </c>
       <c r="E26" s="22">
-        <v>0.1308786741713571</v>
+        <v>0.14973420888055033</v>
       </c>
       <c r="F26" s="22">
         <v>0.4</v>
       </c>
       <c r="G26" s="20">
-        <v>39991</v>
+        <v>44511</v>
       </c>
       <c r="H26" s="20">
-        <v>26255</v>
+        <v>28036</v>
       </c>
       <c r="I26" s="22">
-        <v>-0.5813558050561376</v>
+        <v>-0.56967940509087645</v>
       </c>
       <c r="J26" s="22">
-        <v>-0.36233098457436674</v>
+        <v>-0.3168069624768155</v>
       </c>
       <c r="K26" s="17"/>
       <c r="L26" s="17"/>
@@ -30290,7 +30518,7 @@
         <v>49254</v>
       </c>
       <c r="C49" s="46" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="D49" s="37"/>
       <c r="E49" s="37"/>
@@ -30486,7 +30714,7 @@
         <v>6583</v>
       </c>
       <c r="C54" s="46" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="D54" s="48"/>
       <c r="E54" s="48"/>
@@ -30558,7 +30786,7 @@
     </row>
     <row r="56" spans="1:32" s="38" customFormat="1" ht="14.1" customHeight="1">
       <c r="A56" s="49" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B56" s="48"/>
       <c r="C56" s="48"/>
@@ -30610,18 +30838,18 @@
       <c r="O57" s="4"/>
     </row>
     <row r="58" spans="1:32" ht="30.95" customHeight="1" thickBot="1">
-      <c r="A58" s="159" t="s">
+      <c r="A58" s="154" t="s">
         <v>33</v>
       </c>
-      <c r="B58" s="160"/>
-      <c r="C58" s="160"/>
-      <c r="D58" s="160"/>
-      <c r="E58" s="160"/>
-      <c r="F58" s="160"/>
-      <c r="G58" s="160"/>
-      <c r="H58" s="160"/>
-      <c r="I58" s="160"/>
-      <c r="J58" s="161"/>
+      <c r="B58" s="155"/>
+      <c r="C58" s="155"/>
+      <c r="D58" s="155"/>
+      <c r="E58" s="155"/>
+      <c r="F58" s="155"/>
+      <c r="G58" s="155"/>
+      <c r="H58" s="155"/>
+      <c r="I58" s="155"/>
+      <c r="J58" s="156"/>
       <c r="K58" s="4"/>
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
@@ -30674,10 +30902,10 @@
         <v>16</v>
       </c>
       <c r="B60" s="50">
-        <v>2391</v>
+        <v>2382</v>
       </c>
       <c r="C60" s="21">
-        <v>16742</v>
+        <v>19154</v>
       </c>
       <c r="D60" s="21">
         <v>0</v>
@@ -30689,16 +30917,16 @@
         <v>0.4</v>
       </c>
       <c r="G60" s="23">
-        <v>593</v>
+        <v>650</v>
       </c>
       <c r="H60" s="23">
-        <v>604</v>
+        <v>653</v>
       </c>
       <c r="I60" s="22">
-        <v>-0.23440134907251264</v>
+        <v>-0.21846153846153848</v>
       </c>
       <c r="J60" s="51">
-        <v>-0.2483443708609272</v>
+        <v>-0.222052067381317</v>
       </c>
       <c r="K60" s="16"/>
       <c r="L60" s="16" t="s">
@@ -30713,10 +30941,10 @@
         <v>35</v>
       </c>
       <c r="B61" s="52">
-        <v>1287</v>
+        <v>1278</v>
       </c>
       <c r="C61" s="53">
-        <v>9518</v>
+        <v>10817</v>
       </c>
       <c r="D61" s="54"/>
       <c r="E61" s="55" t="s">
@@ -30726,16 +30954,16 @@
         <v>0.4</v>
       </c>
       <c r="G61" s="31">
-        <v>19803</v>
+        <v>21687</v>
       </c>
       <c r="H61" s="31">
-        <v>14393</v>
+        <v>15322</v>
       </c>
       <c r="I61" s="56">
-        <v>-0.51936575266373786</v>
+        <v>-0.50122193018859229</v>
       </c>
       <c r="J61" s="57">
-        <v>-0.33870631557006881</v>
+        <v>-0.29402166818953135</v>
       </c>
       <c r="K61" s="17"/>
       <c r="L61" s="17"/>
@@ -30751,7 +30979,7 @@
         <v>975</v>
       </c>
       <c r="C62" s="53">
-        <v>6130</v>
+        <v>7110</v>
       </c>
       <c r="D62" s="54"/>
       <c r="E62" s="55" t="s">
@@ -30761,16 +30989,16 @@
         <v>0.4</v>
       </c>
       <c r="G62" s="31">
-        <v>17947</v>
+        <v>20327</v>
       </c>
       <c r="H62" s="31">
-        <v>10378</v>
+        <v>11113</v>
       </c>
       <c r="I62" s="56">
-        <v>-0.65843873627904381</v>
+        <v>-0.65021892064741471</v>
       </c>
       <c r="J62" s="57">
-        <v>-0.40932742339564465</v>
+        <v>-0.36020876451003325</v>
       </c>
       <c r="K62" s="17"/>
       <c r="L62" s="17"/>
@@ -30786,7 +31014,7 @@
         <v>129</v>
       </c>
       <c r="C63" s="60">
-        <v>1094</v>
+        <v>1227</v>
       </c>
       <c r="D63" s="61"/>
       <c r="E63" s="62" t="s">
@@ -30796,16 +31024,16 @@
         <v>0.4</v>
       </c>
       <c r="G63" s="63">
-        <v>2241</v>
+        <v>2497</v>
       </c>
       <c r="H63" s="63">
-        <v>1484</v>
+        <v>1601</v>
       </c>
       <c r="I63" s="64">
-        <v>-0.51182507809013833</v>
+        <v>-0.50861033239887865</v>
       </c>
       <c r="J63" s="65">
-        <v>-0.26280323450134768</v>
+        <v>-0.23360399750156158</v>
       </c>
       <c r="K63" s="17"/>
       <c r="L63" s="17"/>
@@ -32075,7 +32303,7 @@
         <v>19154</v>
       </c>
       <c r="C85" s="46" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="D85" s="37"/>
       <c r="E85" s="37"/>
@@ -32115,7 +32343,7 @@
         <v>44511</v>
       </c>
       <c r="C86" s="46" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="D86" s="37"/>
       <c r="E86" s="37"/>
@@ -32193,7 +32421,7 @@
         <v>2.3238488044272736</v>
       </c>
       <c r="C88" s="46" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="D88" s="37"/>
       <c r="E88" s="37"/>
@@ -32271,7 +32499,7 @@
         <v>2382</v>
       </c>
       <c r="C90" s="46" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D90" s="48"/>
       <c r="E90" s="48"/>
@@ -32311,7 +32539,7 @@
         <v>4520</v>
       </c>
       <c r="C91" s="46" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D91" s="48"/>
       <c r="E91" s="48"/>
@@ -32383,7 +32611,7 @@
     </row>
     <row r="93" spans="1:32" s="38" customFormat="1" ht="14.1" customHeight="1">
       <c r="A93" s="49" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B93" s="48"/>
       <c r="C93" s="48"/>
@@ -32435,18 +32663,18 @@
       <c r="O94" s="4"/>
     </row>
     <row r="95" spans="1:32" ht="30.95" customHeight="1" thickBot="1">
-      <c r="A95" s="159" t="s">
+      <c r="A95" s="154" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="160"/>
-      <c r="C95" s="160"/>
-      <c r="D95" s="160"/>
-      <c r="E95" s="160"/>
-      <c r="F95" s="160"/>
-      <c r="G95" s="160"/>
-      <c r="H95" s="160"/>
-      <c r="I95" s="160"/>
-      <c r="J95" s="161"/>
+      <c r="B95" s="155"/>
+      <c r="C95" s="155"/>
+      <c r="D95" s="155"/>
+      <c r="E95" s="155"/>
+      <c r="F95" s="155"/>
+      <c r="G95" s="155"/>
+      <c r="H95" s="155"/>
+      <c r="I95" s="155"/>
+      <c r="J95" s="156"/>
       <c r="K95" s="4"/>
       <c r="L95" s="4"/>
       <c r="M95" s="4"/>
@@ -32499,10 +32727,10 @@
         <v>16</v>
       </c>
       <c r="B97" s="68">
-        <v>4193</v>
+        <v>4201</v>
       </c>
       <c r="C97" s="21">
-        <v>25898</v>
+        <v>30098</v>
       </c>
       <c r="D97" s="21">
         <v>0</v>
@@ -32514,16 +32742,16 @@
         <v>0.4</v>
       </c>
       <c r="G97" s="23">
-        <v>695</v>
+        <v>793</v>
       </c>
       <c r="H97" s="23">
-        <v>15274</v>
+        <v>16422</v>
       </c>
       <c r="I97" s="22">
-        <v>36.263309352517986</v>
+        <v>36.954602774274903</v>
       </c>
       <c r="J97" s="22">
-        <v>0.69556108419536478</v>
+        <v>0.83278528802825469</v>
       </c>
       <c r="K97" s="16"/>
       <c r="L97" s="16" t="s">
@@ -33841,7 +34069,7 @@
         <v>167765</v>
       </c>
       <c r="C121" s="46" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D121" s="37"/>
       <c r="E121" s="37"/>
@@ -34037,7 +34265,7 @@
         <v>30100</v>
       </c>
       <c r="C126" s="46" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D126" s="48"/>
       <c r="E126" s="48"/>
@@ -34109,7 +34337,7 @@
     </row>
     <row r="128" spans="1:32" s="38" customFormat="1" ht="14.1" customHeight="1">
       <c r="A128" s="49" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B128" s="48"/>
       <c r="C128" s="48"/>
@@ -34211,21 +34439,21 @@
       <c r="N131" s="4"/>
       <c r="O131" s="4"/>
     </row>
-    <row r="132" spans="1:32" ht="23.25" hidden="1" thickBot="1">
-      <c r="A132" s="159" t="s">
+    <row r="132" spans="1:32" ht="29.1" hidden="1" customHeight="1" thickBot="1">
+      <c r="A132" s="154" t="s">
         <v>42</v>
       </c>
-      <c r="B132" s="160"/>
-      <c r="C132" s="160"/>
-      <c r="D132" s="160"/>
-      <c r="E132" s="160"/>
-      <c r="F132" s="160"/>
-      <c r="G132" s="160"/>
-      <c r="H132" s="160"/>
-      <c r="I132" s="160"/>
-      <c r="J132" s="160"/>
-      <c r="K132" s="160"/>
-      <c r="L132" s="161"/>
+      <c r="B132" s="155"/>
+      <c r="C132" s="155"/>
+      <c r="D132" s="155"/>
+      <c r="E132" s="155"/>
+      <c r="F132" s="155"/>
+      <c r="G132" s="155"/>
+      <c r="H132" s="155"/>
+      <c r="I132" s="155"/>
+      <c r="J132" s="155"/>
+      <c r="K132" s="155"/>
+      <c r="L132" s="156"/>
       <c r="M132" s="4"/>
       <c r="N132" s="4"/>
       <c r="O132" s="4"/>
@@ -34346,33 +34574,33 @@
       <c r="M137" s="86"/>
       <c r="N137" s="86"/>
       <c r="O137" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="138" spans="1:32">
-      <c r="A138" s="162" t="s">
+      <c r="A138" s="157" t="s">
         <v>54</v>
       </c>
-      <c r="B138" s="163"/>
-      <c r="C138" s="163"/>
-      <c r="D138" s="163"/>
-      <c r="E138" s="163"/>
-      <c r="F138" s="164"/>
+      <c r="B138" s="158"/>
+      <c r="C138" s="158"/>
+      <c r="D138" s="158"/>
+      <c r="E138" s="158"/>
+      <c r="F138" s="159"/>
       <c r="G138" s="168" t="s">
         <v>55</v>
       </c>
-      <c r="H138" s="166"/>
-      <c r="I138" s="167"/>
-      <c r="J138" s="165" t="s">
+      <c r="H138" s="169"/>
+      <c r="I138" s="169"/>
+      <c r="J138" s="170" t="s">
         <v>56</v>
       </c>
-      <c r="K138" s="166"/>
-      <c r="L138" s="167"/>
-      <c r="M138" s="165" t="s">
+      <c r="K138" s="171"/>
+      <c r="L138" s="171"/>
+      <c r="M138" s="170" t="s">
         <v>57</v>
       </c>
-      <c r="N138" s="166"/>
-      <c r="O138" s="169"/>
+      <c r="N138" s="171"/>
+      <c r="O138" s="172"/>
     </row>
     <row r="139" spans="1:32" ht="42.75">
       <c r="A139" s="88" t="s">
@@ -34429,43 +34657,43 @@
         <v>0</v>
       </c>
       <c r="C140" s="92">
-        <v>16742</v>
+        <v>19154</v>
       </c>
       <c r="D140" s="93">
         <v>0</v>
       </c>
       <c r="E140" s="93">
-        <v>-0.5813558050561376</v>
+        <v>-0.56967940509087645</v>
       </c>
       <c r="F140" s="94">
-        <v>-0.36233098457436674</v>
+        <v>-0.3168069624768155</v>
       </c>
       <c r="G140" s="95">
-        <v>9518</v>
+        <v>10817</v>
       </c>
       <c r="H140" s="93">
-        <v>-0.51936575266373786</v>
+        <v>-0.50122193018859229</v>
       </c>
       <c r="I140" s="93">
-        <v>-0.33870631557006881</v>
+        <v>-0.29402166818953135</v>
       </c>
       <c r="J140" s="96">
-        <v>6130</v>
+        <v>7110</v>
       </c>
       <c r="K140" s="93">
-        <v>-0.65843873627904381</v>
+        <v>-0.65021892064741471</v>
       </c>
       <c r="L140" s="93">
-        <v>-0.40932742339564465</v>
+        <v>-0.36020876451003325</v>
       </c>
       <c r="M140" s="96">
-        <v>1094</v>
+        <v>1227</v>
       </c>
       <c r="N140" s="93">
-        <v>-0.51182507809013833</v>
+        <v>-0.50861033239887865</v>
       </c>
       <c r="O140" s="94">
-        <v>-0.26280323450134768</v>
+        <v>-0.23360399750156158</v>
       </c>
     </row>
     <row r="141" spans="1:32" ht="15.75">
@@ -34947,7 +35175,7 @@
       <c r="D153" s="110"/>
       <c r="E153" s="110"/>
       <c r="F153" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J153" s="109"/>
       <c r="K153" s="111"/>
@@ -34957,7 +35185,7 @@
       <c r="M153" s="110"/>
       <c r="N153" s="110"/>
       <c r="O153" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="154" spans="1:15" ht="24.6" customHeight="1">
@@ -35006,16 +35234,16 @@
         <v>0</v>
       </c>
       <c r="C155" s="92">
-        <v>3010</v>
+        <v>3431</v>
       </c>
       <c r="D155" s="93">
         <v>0</v>
       </c>
       <c r="E155" s="93">
-        <v>-0.65</v>
+        <v>-0.63792739552553823</v>
       </c>
       <c r="F155" s="94">
-        <v>-0.45726649837720879</v>
+        <v>-0.41738835116318562</v>
       </c>
       <c r="J155" s="114" t="s">
         <v>16</v>
@@ -35024,16 +35252,16 @@
         <v>0</v>
       </c>
       <c r="L155" s="92">
-        <v>5015</v>
+        <v>5747</v>
       </c>
       <c r="M155" s="93">
         <v>0</v>
       </c>
       <c r="N155" s="93">
-        <v>-0.6023628290516968</v>
+        <v>-0.59148421950526009</v>
       </c>
       <c r="O155" s="94">
-        <v>-0.45801361720523071</v>
+        <v>-0.41796637634190803</v>
       </c>
     </row>
     <row r="156" spans="1:15" ht="15.75">
@@ -35425,7 +35653,7 @@
       <c r="D168" s="110"/>
       <c r="E168" s="110"/>
       <c r="F168" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J168" s="109"/>
       <c r="K168" s="110"/>
@@ -35435,7 +35663,7 @@
       <c r="M168" s="110"/>
       <c r="N168" s="110"/>
       <c r="O168" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="169" spans="1:15" ht="26.45" customHeight="1">
@@ -35484,16 +35712,16 @@
         <v>0</v>
       </c>
       <c r="C170" s="92">
-        <v>1120</v>
+        <v>1247</v>
       </c>
       <c r="D170" s="93">
         <v>0</v>
       </c>
       <c r="E170" s="93">
-        <v>-0.77635782747603832</v>
+        <v>-0.77767873061151715</v>
       </c>
       <c r="F170" s="94">
-        <v>-0.28525845564773455</v>
+        <v>-0.24424242424242426</v>
       </c>
       <c r="J170" s="114" t="s">
         <v>16</v>
@@ -35502,16 +35730,16 @@
         <v>0</v>
       </c>
       <c r="L170" s="92">
-        <v>2505</v>
+        <v>2853</v>
       </c>
       <c r="M170" s="93">
         <v>0</v>
       </c>
       <c r="N170" s="93">
-        <v>-0.65839356334378829</v>
+        <v>-0.65338354999392534</v>
       </c>
       <c r="O170" s="94">
-        <v>-0.38010393466963621</v>
+        <v>-0.33728222996515678</v>
       </c>
     </row>
     <row r="171" spans="1:15" ht="15.75">
@@ -35522,16 +35750,16 @@
         <v>0</v>
       </c>
       <c r="C171" s="116">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="D171" s="98">
         <v>0</v>
       </c>
       <c r="E171" s="98">
-        <v>-0.80962800875273522</v>
+        <v>-0.7880658436213992</v>
       </c>
       <c r="F171" s="117">
-        <v>-0.35074626865671643</v>
+        <v>-0.28965517241379313</v>
       </c>
       <c r="J171" s="115" t="e">
         <v>#N/A</v>
@@ -35560,16 +35788,16 @@
         <v>0</v>
       </c>
       <c r="C172" s="116">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="D172" s="98">
         <v>0</v>
       </c>
       <c r="E172" s="98">
-        <v>-0.81297709923664119</v>
+        <v>-0.81305114638447973</v>
       </c>
       <c r="F172" s="117">
-        <v>-0.3098591549295775</v>
+        <v>-0.29333333333333333</v>
       </c>
       <c r="J172" s="115" t="e">
         <v>#N/A</v>
@@ -35598,16 +35826,16 @@
         <v>0</v>
       </c>
       <c r="C173" s="116">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="D173" s="98">
         <v>0</v>
       </c>
       <c r="E173" s="98">
-        <v>-0.68892508143322473</v>
+        <v>-0.68562874251497008</v>
       </c>
       <c r="F173" s="117">
-        <v>-0.18376068376068377</v>
+        <v>-0.13580246913580252</v>
       </c>
       <c r="J173" s="115" t="e">
         <v>#N/A</v>
@@ -35636,16 +35864,16 @@
         <v>0</v>
       </c>
       <c r="C174" s="116">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="D174" s="98">
         <v>0</v>
       </c>
       <c r="E174" s="98">
-        <v>-0.8303167420814479</v>
+        <v>-0.83586337760910823</v>
       </c>
       <c r="F174" s="117">
-        <v>-0.2990654205607477</v>
+        <v>-0.23451327433628322</v>
       </c>
       <c r="J174" s="115" t="e">
         <v>#N/A</v>
@@ -35674,16 +35902,16 @@
         <v>0</v>
       </c>
       <c r="C175" s="116">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="D175" s="98">
         <v>0</v>
       </c>
       <c r="E175" s="98">
-        <v>-0.68921775898520088</v>
+        <v>-0.69673704414587334</v>
       </c>
       <c r="F175" s="117">
-        <v>-0.35242290748898675</v>
+        <v>-0.34979423868312753</v>
       </c>
       <c r="J175" s="115" t="e">
         <v>#N/A</v>
@@ -35712,16 +35940,16 @@
         <v>0</v>
       </c>
       <c r="C176" s="116">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D176" s="98">
         <v>0</v>
       </c>
       <c r="E176" s="98">
-        <v>-0.80952380952380953</v>
+        <v>-0.82282282282282282</v>
       </c>
       <c r="F176" s="117">
-        <v>-0.4285714285714286</v>
+        <v>-0.42439024390243907</v>
       </c>
       <c r="J176" s="115" t="e">
         <v>#N/A</v>
@@ -35750,16 +35978,16 @@
         <v>0</v>
       </c>
       <c r="C177" s="116">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D177" s="98">
         <v>0</v>
       </c>
       <c r="E177" s="98">
-        <v>-0.6947368421052631</v>
+        <v>-0.69230769230769229</v>
       </c>
       <c r="F177" s="117">
-        <v>-0.10309278350515461</v>
+        <v>9.7087378640776656E-3</v>
       </c>
       <c r="J177" s="115" t="e">
         <v>#N/A</v>
@@ -35788,16 +36016,16 @@
         <v>0</v>
       </c>
       <c r="C178" s="116">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D178" s="98">
         <v>0</v>
       </c>
       <c r="E178" s="98">
-        <v>-0.52755905511811019</v>
+        <v>-0.57615894039735105</v>
       </c>
       <c r="F178" s="117">
-        <v>-0.10447761194029848</v>
+        <v>-7.2463768115942018E-2</v>
       </c>
       <c r="J178" s="115" t="e">
         <v>#N/A</v>
@@ -35826,16 +36054,16 @@
         <v>0</v>
       </c>
       <c r="C179" s="116">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="D179" s="98">
         <v>0</v>
       </c>
       <c r="E179" s="98">
-        <v>-0.83976608187134505</v>
+        <v>-0.8349307774227902</v>
       </c>
       <c r="F179" s="117">
-        <v>-0.18934911242603547</v>
+        <v>-0.10919540229885061</v>
       </c>
       <c r="J179" s="115" t="e">
         <v>#N/A</v>
@@ -35864,16 +36092,16 @@
         <v>0</v>
       </c>
       <c r="C180" s="119">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D180" s="104">
         <v>0</v>
       </c>
       <c r="E180" s="104">
-        <v>-0.74626865671641784</v>
+        <v>-0.74429223744292239</v>
       </c>
       <c r="F180" s="120">
-        <v>-0.41379310344827591</v>
+        <v>-0.39130434782608692</v>
       </c>
       <c r="J180" s="118" t="e">
         <v>#N/A</v>
@@ -35903,7 +36131,7 @@
       <c r="D183" s="110"/>
       <c r="E183" s="110"/>
       <c r="F183" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J183" s="109"/>
       <c r="K183" s="110"/>
@@ -35913,7 +36141,7 @@
       <c r="M183" s="110"/>
       <c r="N183" s="110"/>
       <c r="O183" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="184" spans="1:20" ht="26.45" customHeight="1">
@@ -35962,16 +36190,16 @@
         <v>0</v>
       </c>
       <c r="C185" s="92">
-        <v>490</v>
+        <v>565</v>
       </c>
       <c r="D185" s="93">
         <v>0</v>
       </c>
       <c r="E185" s="93">
-        <v>-0.80524642289348169</v>
+        <v>-0.79558610709117228</v>
       </c>
       <c r="F185" s="94">
-        <v>-9.5940959409594129E-2</v>
+        <v>-4.2372881355932202E-2</v>
       </c>
       <c r="J185" s="114" t="s">
         <v>16</v>
@@ -35980,16 +36208,16 @@
         <v>0</v>
       </c>
       <c r="L185" s="92">
-        <v>2550</v>
+        <v>2927</v>
       </c>
       <c r="M185" s="93">
         <v>0</v>
       </c>
       <c r="N185" s="93">
-        <v>-5.0632911392405111E-2</v>
+        <v>-2.8865295288653003E-2</v>
       </c>
       <c r="O185" s="94">
-        <v>-0.2812852311161218</v>
+        <v>-0.23437091289563172</v>
       </c>
     </row>
     <row r="186" spans="1:20" ht="15.75">
@@ -36373,7 +36601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:15" hidden="1"/>
+    <row r="197" spans="1:15" ht="14.25" hidden="1" customHeight="1"/>
     <row r="198" spans="1:15" ht="23.45" hidden="1" customHeight="1">
       <c r="A198" s="109"/>
       <c r="B198" s="110"/>
@@ -36383,7 +36611,7 @@
       <c r="D198" s="110"/>
       <c r="E198" s="110"/>
       <c r="F198" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J198" s="109"/>
       <c r="K198" s="110"/>
@@ -36393,7 +36621,7 @@
       <c r="M198" s="110"/>
       <c r="N198" s="110"/>
       <c r="O198" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="199" spans="1:15" ht="23.45" hidden="1" customHeight="1">
@@ -36434,7 +36662,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="200" spans="1:15" ht="15.75" hidden="1">
+    <row r="200" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A200" s="114" t="s">
         <v>16</v>
       </c>
@@ -36442,16 +36670,16 @@
         <v>0</v>
       </c>
       <c r="C200" s="92">
-        <v>490</v>
+        <v>565</v>
       </c>
       <c r="D200" s="93">
         <v>0</v>
       </c>
       <c r="E200" s="93">
-        <v>-0.80524642289348169</v>
+        <v>-0.79558610709117228</v>
       </c>
       <c r="F200" s="94">
-        <v>-9.5940959409594129E-2</v>
+        <v>-4.2372881355932202E-2</v>
       </c>
       <c r="J200" s="114" t="s">
         <v>16</v>
@@ -36472,7 +36700,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="201" spans="1:15" ht="15.75" hidden="1">
+    <row r="201" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A201" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36510,7 +36738,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="202" spans="1:15" ht="15.75" hidden="1">
+    <row r="202" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A202" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36548,7 +36776,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="203" spans="1:15" ht="15.75" hidden="1">
+    <row r="203" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A203" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36586,7 +36814,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="204" spans="1:15" ht="15.75" hidden="1">
+    <row r="204" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A204" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36624,7 +36852,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="205" spans="1:15" ht="15.75" hidden="1">
+    <row r="205" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A205" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36662,7 +36890,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="206" spans="1:15" ht="15.75" hidden="1">
+    <row r="206" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A206" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36700,7 +36928,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="207" spans="1:15" ht="15.75" hidden="1">
+    <row r="207" spans="1:15" ht="15.75" hidden="1" customHeight="1">
       <c r="A207" s="115" t="e">
         <v>#N/A</v>
       </c>
@@ -36738,7 +36966,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="208" spans="1:15" ht="16.5" hidden="1" thickBot="1">
+    <row r="208" spans="1:15" ht="15.75" hidden="1" customHeight="1" thickBot="1">
       <c r="A208" s="118" t="e">
         <v>#N/A</v>
       </c>
@@ -36776,7 +37004,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="209" spans="1:18" hidden="1"/>
+    <row r="209" spans="1:18" ht="14.25" hidden="1" customHeight="1"/>
     <row r="210" spans="1:18" ht="15" thickBot="1"/>
     <row r="211" spans="1:18" ht="29.1" customHeight="1" thickBot="1">
       <c r="A211" s="109"/>
@@ -36787,7 +37015,7 @@
       <c r="D211" s="110"/>
       <c r="E211" s="110"/>
       <c r="F211" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J211" s="109"/>
       <c r="K211" s="110"/>
@@ -36797,7 +37025,7 @@
       <c r="M211" s="110"/>
       <c r="N211" s="110"/>
       <c r="O211" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="212" spans="1:18" ht="26.1" customHeight="1">
@@ -36851,16 +37079,16 @@
         <v>0</v>
       </c>
       <c r="C213" s="92">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="D213" s="93">
         <v>0</v>
       </c>
       <c r="E213" s="93">
-        <v>-0.86574654956085317</v>
+        <v>-0.85172413793103452</v>
       </c>
       <c r="F213" s="94">
-        <v>-0.27702702702702697</v>
+        <v>-0.16774193548387095</v>
       </c>
       <c r="J213" s="114" t="s">
         <v>16</v>
@@ -36869,19 +37097,19 @@
         <v>0</v>
       </c>
       <c r="L213" s="92">
-        <v>3412</v>
+        <v>3808</v>
       </c>
       <c r="M213" s="93">
         <v>0</v>
       </c>
       <c r="N213" s="93">
-        <v>3.9093525179856119</v>
+        <v>3.8020176544766713</v>
       </c>
       <c r="O213" s="125">
-        <v>-3.1232254400908599E-2</v>
+        <v>-5.2246603970741434E-3</v>
       </c>
       <c r="P213" s="126">
-        <v>4193</v>
+        <v>4201</v>
       </c>
       <c r="Q213" s="124"/>
       <c r="R213" s="124"/>
@@ -37284,7 +37512,7 @@
       <c r="D226" s="110"/>
       <c r="E226" s="110"/>
       <c r="F226" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J226" s="109"/>
       <c r="K226" s="110"/>
@@ -37294,7 +37522,7 @@
       <c r="M226" s="110"/>
       <c r="N226" s="110"/>
       <c r="O226" s="87" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="227" spans="1:15" ht="42.75">
@@ -37343,7 +37571,7 @@
         <v>0</v>
       </c>
       <c r="C228" s="92">
-        <v>3032</v>
+        <v>3351</v>
       </c>
       <c r="D228" s="93">
         <v>0</v>
@@ -37352,7 +37580,7 @@
         <v>0</v>
       </c>
       <c r="F228" s="94">
-        <v>-0.23026148768723032</v>
+        <v>-0.20460479468312365</v>
       </c>
       <c r="J228" s="114" t="s">
         <v>16</v>
@@ -37361,7 +37589,7 @@
         <v>0</v>
       </c>
       <c r="L228" s="92">
-        <v>5701</v>
+        <v>6344</v>
       </c>
       <c r="M228" s="93">
         <v>0</v>
@@ -37370,7 +37598,7 @@
         <v>0</v>
       </c>
       <c r="O228" s="94">
-        <v>-0.26076244813278004</v>
+        <v>-0.23279719434030721</v>
       </c>
     </row>
     <row r="229" spans="1:15" ht="15.75">
@@ -37754,60 +37982,53 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="M138:O138"/>
+  <mergeCells count="1">
     <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A58:J58"/>
-    <mergeCell ref="A95:J95"/>
-    <mergeCell ref="A132:L132"/>
-    <mergeCell ref="A138:F138"/>
-    <mergeCell ref="G138:I138"/>
-    <mergeCell ref="J138:L138"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="D141:D150">
-    <cfRule type="top10" dxfId="43" priority="21" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="42" priority="22" rank="3"/>
+    <cfRule type="top10" dxfId="21" priority="21" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="20" priority="22" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D156:D165">
-    <cfRule type="top10" dxfId="39" priority="19" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="38" priority="20" rank="3"/>
+    <cfRule type="top10" dxfId="19" priority="19" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="18" priority="20" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D186:D195">
-    <cfRule type="top10" dxfId="35" priority="17" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="34" priority="17" rank="3"/>
+    <cfRule type="top10" dxfId="17" priority="5" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="16" priority="6" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D201:D208">
-    <cfRule type="top10" dxfId="31" priority="15" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="30" priority="15" rank="3"/>
+    <cfRule type="top10" dxfId="15" priority="11" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="14" priority="12" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D214:D223">
-    <cfRule type="top10" dxfId="27" priority="13" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="26" priority="13" rank="3"/>
+    <cfRule type="top10" dxfId="13" priority="9" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="12" priority="10" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D229:D238">
-    <cfRule type="top10" dxfId="23" priority="11" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="22" priority="11" rank="3"/>
+    <cfRule type="top10" dxfId="11" priority="1" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="10" priority="2" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M156:M165">
-    <cfRule type="top10" dxfId="19" priority="17" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="18" priority="18" rank="3"/>
+    <cfRule type="top10" dxfId="9" priority="17" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="8" priority="18" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M171:M180">
-    <cfRule type="top10" dxfId="15" priority="15" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="14" priority="16" rank="3"/>
+    <cfRule type="top10" dxfId="7" priority="15" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="6" priority="16" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M186:M195">
-    <cfRule type="top10" dxfId="11" priority="13" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="10" priority="14" rank="3"/>
+    <cfRule type="top10" dxfId="5" priority="13" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="4" priority="14" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M214:M223">
-    <cfRule type="top10" dxfId="7" priority="7" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="6" priority="8" rank="3"/>
+    <cfRule type="top10" dxfId="3" priority="7" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="2" priority="8" rank="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M229:M238">
-    <cfRule type="top10" dxfId="3" priority="3" bottom="1" rank="3"/>
-    <cfRule type="top10" dxfId="2" priority="4" rank="3"/>
+    <cfRule type="top10" dxfId="1" priority="3" bottom="1" rank="3"/>
+    <cfRule type="top10" dxfId="0" priority="4" rank="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Add valid leads control dashboard and rebuild data parsing
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkCode\AI_Digest\data\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0CABA7-8CDB-4305-9E52-F4B6D7A71D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19178379-C8FE-4531-9519-AC998A606777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4F6CCF54-37E5-4816-9B51-3E2CFD892ED8}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4F6CCF54-37E5-4816-9B51-3E2CFD892ED8}"/>
   </bookViews>
   <sheets>
     <sheet name="来店日趋势汇总" sheetId="2" r:id="rId1"/>
@@ -371,70 +371,70 @@
     <t/>
   </si>
   <si>
-    <t>请查收4月1-12日的来店业绩：</t>
+    <t>【整体来店】
+ICE+NEV累计来店 53,071；当日来店 3,783
+① ICE累计来店 20,814；当日来店 1,626
+② NEV累计来店 32,257；当日来店 2,157</t>
   </si>
   <si>
-    <t>累计实绩：49254（累计同比9%）</t>
+    <t>请查收4月1-13日的来店业绩：</t>
   </si>
   <si>
-    <t>当日实绩：6583</t>
+    <t>1、ICE+NEV合计来店：13日来店量3,783，1-13日来店总量53,069，同比4.3%，环比11.3%</t>
   </si>
   <si>
-    <t>累计实绩49254，累计达成率-；当日实绩6583，当日达成率-</t>
+    <t>2、ICE（油车）来店：管控目标：13日来店目标0，来店量1,626，达成率-；月累来店目标0，来店量20,814，达成率-；月度目标0，达成率-；同比-58.3%，环比-30.8%；必达目标，达成率-</t>
   </si>
   <si>
-    <t>累计目标：19154</t>
+    <t>3、NEV来店：13日来店量2,157，1-13日来店总量32,255，环比83.0%</t>
   </si>
   <si>
-    <t>累计实绩：44511（累计同比-61%）</t>
+    <t>—自然来店11,585，达成率-，同比-51.9%，环比-29.0%；</t>
   </si>
   <si>
-    <t>累计达成率：232%</t>
+    <t>—开拓渠道来店7,900，达成率-，同比-65.8%，环比-34.4%；</t>
   </si>
   <si>
-    <t>当日目标：2382</t>
+    <t>—保有客户来店1,329，达成率-，同比-52.1%，环比-22.1%</t>
   </si>
   <si>
-    <t>当日实绩：4520</t>
+    <t>累计实绩：53071（累计同比4%）</t>
   </si>
   <si>
-    <t>累计实绩44511，累计达成率232%；当日实绩4520，当日达成率190%</t>
+    <t>当日实绩：3783</t>
   </si>
   <si>
-    <t>累计实绩：167765（累计同比922%）</t>
+    <t>累计实绩53071，累计达成率-；当日实绩3783，当日达成率-</t>
   </si>
   <si>
-    <t>当日实绩：30100</t>
+    <t>累计目标：20814</t>
   </si>
   <si>
-    <t>累计实绩167765，累计达成率-；当日实绩30100，当日达成率-</t>
+    <t>累计实绩：49958（累计同比-63%）</t>
   </si>
   <si>
-    <t>统计周期4.1-4.12</t>
+    <t>累计达成率：240%</t>
   </si>
   <si>
-    <t>【整体来店】
-ICE+NEV累计来店 49,254；当日来店 6,583
-① ICE累计来店 19,154；当日来店 2,382
-② NEV累计来店 30,100；当日来店 4,201</t>
+    <t>当日目标：1626</t>
   </si>
   <si>
-    <t>1、ICE+NEV合计来店：12日来店量6,583，1-12日来店总量49,252，同比8.7%，环比10.8%</t>
+    <t>当日实绩：5447</t>
   </si>
   <si>
-    <t>2、ICE（油车）来店：管控目标：12日来店目标0，来店量2,382，达成率-；月累来店目标0，来店量19,154，达成率-；月度目标0，达成率-；同比-57.0%，环比-31.7%；必达目标，达成率-</t>
+    <t>累计实绩49958，累计达成率240%；当日实绩5447，当日达成率335%</t>
   </si>
   <si>
-    <t>3、NEV来店：12日来店量4,201，1-12日来店总量30,098，环比83.3%</t>
+    <t>累计实绩：200022（累计同比1035%）</t>
   </si>
   <si>
-    <t>—自然来店10,817，达成率-，同比-50.1%，环比-29.4%；</t>
+    <t>当日实绩：32257</t>
   </si>
   <si>
-    <t>—开拓渠道来店7,110，达成率-，同比-65.0%，环比-36.0%；</t>
+    <t>累计实绩200022，累计达成率-；当日实绩32257，当日达成率-</t>
   </si>
   <si>
-    <t>—保有客户来店1,227，达成率-，同比-50.9%，环比-23.4%</t>
+    <t>统计周期4.1-4.13</t>
   </si>
 </sst>
 </file>
@@ -1593,6 +1593,24 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1613,24 +1631,6 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1904,6 +1904,16 @@
       </font>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="1"/>
         </patternFill>
       </fill>
@@ -1945,16 +1955,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -22091,6 +22091,454 @@
     </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>55559</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>31749</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>269877</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>426860</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="32" name="组合 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED222645-C8B1-4BB9-A827-B31D38CF35FA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="55559" y="31749"/>
+          <a:ext cx="1776418" cy="395111"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="1531943" cy="395111"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="33" name="组合 32">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D32C061-B653-18DC-440A-1705DD957D7E}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="1531943" cy="395111"/>
+            <a:chOff x="0" y="0"/>
+            <a:chExt cx="1243417" cy="395111"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="35" name="矩形 34">
+              <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DFA12D9-7DDB-486C-8B70-775C24F4D062}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="297581" y="39511"/>
+              <a:ext cx="945836" cy="333552"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr"/>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:ea typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:cs typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                </a:rPr>
+                <a:t>返回目录</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="36" name="椭圆 35">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C23190FB-E4F4-4005-6319-A2CBB0F455CE}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="380773" cy="395111"/>
+            </a:xfrm>
+            <a:prstGeom prst="ellipse">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="34" name="图片 33">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA82EB42-89A6-DF81-20CF-D551E6BF5F71}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr preferRelativeResize="0"/>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="87507" y="32927"/>
+            <a:ext cx="325247" cy="329259"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:miter lim="800000"/>
+                <a:headEnd/>
+                <a:tailEnd/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>55559</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>31749</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>269877</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>426860</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="37" name="组合 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F798767-D59A-4A10-8B8F-C2CEB94F7D0A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="55559" y="31749"/>
+          <a:ext cx="1776418" cy="395111"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="1531943" cy="395111"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="38" name="组合 37">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87CC98C8-7C00-C89B-60A9-934E80B85944}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="1531943" cy="395111"/>
+            <a:chOff x="0" y="0"/>
+            <a:chExt cx="1243417" cy="395111"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="40" name="矩形 39">
+              <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{231B862E-B63C-B834-B9FF-8CFC75288FB8}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="297581" y="39511"/>
+              <a:ext cx="945836" cy="333552"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr"/>
+              <a:r>
+                <a:rPr lang="zh-CN" altLang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="bg1"/>
+                  </a:solidFill>
+                  <a:latin typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:ea typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                  <a:cs typeface="微软雅黑" panose="020B0503020204020204" charset="-122"/>
+                </a:rPr>
+                <a:t>返回目录</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="41" name="椭圆 40">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9DCAF0CB-C676-BF1B-5AC8-0E01DFD4A6BB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="380773" cy="395111"/>
+            </a:xfrm>
+            <a:prstGeom prst="ellipse">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="2">
+              <a:schemeClr val="accent1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:lnRef>
+            <a:fillRef idx="1">
+              <a:schemeClr val="accent1"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:schemeClr val="accent1"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="lt1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="39" name="图片 38">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DEFB1FAE-F2AC-278B-BEAD-8E3399EE389F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr preferRelativeResize="0"/>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="87507" y="32927"/>
+            <a:ext cx="325247" cy="329259"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:miter lim="800000"/>
+                <a:headEnd/>
+                <a:tailEnd/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -26751,19 +27199,19 @@
     <row r="1" ht="33.950000000000003" customHeight="1"/>
     <row r="2" ht="29.1" customHeight="1"/>
     <row r="29" spans="2:33">
-      <c r="C29" s="163"/>
-      <c r="D29" s="163"/>
-      <c r="E29" s="163"/>
-      <c r="F29" s="163"/>
-      <c r="Q29" s="164"/>
-      <c r="R29" s="164"/>
-      <c r="S29" s="164"/>
-      <c r="T29" s="164"/>
-      <c r="U29" s="164"/>
-      <c r="V29" s="164"/>
-      <c r="W29" s="164"/>
-      <c r="X29" s="164"/>
-      <c r="Y29" s="164"/>
+      <c r="C29" s="169"/>
+      <c r="D29" s="169"/>
+      <c r="E29" s="169"/>
+      <c r="F29" s="169"/>
+      <c r="Q29" s="170"/>
+      <c r="R29" s="170"/>
+      <c r="S29" s="170"/>
+      <c r="T29" s="170"/>
+      <c r="U29" s="170"/>
+      <c r="V29" s="170"/>
+      <c r="W29" s="170"/>
+      <c r="X29" s="170"/>
+      <c r="Y29" s="170"/>
     </row>
     <row r="30" spans="2:33">
       <c r="B30" s="132" t="s">
@@ -27514,19 +27962,19 @@
     </row>
     <row r="44" spans="2:33" s="144" customFormat="1"/>
     <row r="72" spans="2:33">
-      <c r="C72" s="165"/>
-      <c r="D72" s="165"/>
-      <c r="E72" s="165"/>
-      <c r="F72" s="165"/>
-      <c r="Q72" s="166"/>
-      <c r="R72" s="166"/>
-      <c r="S72" s="166"/>
-      <c r="T72" s="166"/>
-      <c r="U72" s="166"/>
-      <c r="V72" s="166"/>
-      <c r="W72" s="166"/>
-      <c r="X72" s="166"/>
-      <c r="Y72" s="166"/>
+      <c r="C72" s="171"/>
+      <c r="D72" s="171"/>
+      <c r="E72" s="171"/>
+      <c r="F72" s="171"/>
+      <c r="Q72" s="172"/>
+      <c r="R72" s="172"/>
+      <c r="S72" s="172"/>
+      <c r="T72" s="172"/>
+      <c r="U72" s="172"/>
+      <c r="V72" s="172"/>
+      <c r="W72" s="172"/>
+      <c r="X72" s="172"/>
+      <c r="Y72" s="172"/>
     </row>
     <row r="73" spans="2:33">
       <c r="B73" s="145" t="s">
@@ -28106,19 +28554,19 @@
     </row>
     <row r="85" s="149" customFormat="1"/>
     <row r="115" spans="2:33">
-      <c r="C115" s="165"/>
-      <c r="D115" s="165"/>
-      <c r="E115" s="165"/>
-      <c r="F115" s="165"/>
-      <c r="Q115" s="166"/>
-      <c r="R115" s="166"/>
-      <c r="S115" s="166"/>
-      <c r="T115" s="166"/>
-      <c r="U115" s="166"/>
-      <c r="V115" s="166"/>
-      <c r="W115" s="166"/>
-      <c r="X115" s="166"/>
-      <c r="Y115" s="166"/>
+      <c r="C115" s="171"/>
+      <c r="D115" s="171"/>
+      <c r="E115" s="171"/>
+      <c r="F115" s="171"/>
+      <c r="Q115" s="172"/>
+      <c r="R115" s="172"/>
+      <c r="S115" s="172"/>
+      <c r="T115" s="172"/>
+      <c r="U115" s="172"/>
+      <c r="V115" s="172"/>
+      <c r="W115" s="172"/>
+      <c r="X115" s="172"/>
+      <c r="Y115" s="172"/>
     </row>
     <row r="116" spans="2:33">
       <c r="B116" s="150" t="s">
@@ -28806,13 +29254,13 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
-      <c r="AG2" s="167" t="s">
-        <v>118</v>
+      <c r="AG2" s="160" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:33" ht="15" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -28867,7 +29315,7 @@
     </row>
     <row r="6" spans="1:33" ht="15" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -28903,7 +29351,7 @@
     </row>
     <row r="8" spans="1:33" s="6" customFormat="1" ht="16.5" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -28939,7 +29387,7 @@
     </row>
     <row r="10" spans="1:33" ht="15" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -28994,7 +29442,7 @@
     </row>
     <row r="13" spans="1:33" ht="16.5" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -29013,7 +29461,7 @@
     </row>
     <row r="14" spans="1:33" ht="15" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -29032,7 +29480,7 @@
     </row>
     <row r="15" spans="1:33" ht="15" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -29157,18 +29605,18 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22" spans="1:32" ht="30.95" customHeight="1" thickBot="1">
-      <c r="A22" s="160" t="s">
+      <c r="A22" s="166" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="161"/>
-      <c r="C22" s="161"/>
-      <c r="D22" s="161"/>
-      <c r="E22" s="161"/>
-      <c r="F22" s="161"/>
-      <c r="G22" s="161"/>
-      <c r="H22" s="161"/>
-      <c r="I22" s="161"/>
-      <c r="J22" s="162"/>
+      <c r="B22" s="167"/>
+      <c r="C22" s="167"/>
+      <c r="D22" s="167"/>
+      <c r="E22" s="167"/>
+      <c r="F22" s="167"/>
+      <c r="G22" s="167"/>
+      <c r="H22" s="167"/>
+      <c r="I22" s="167"/>
+      <c r="J22" s="168"/>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -29221,31 +29669,31 @@
         <v>16</v>
       </c>
       <c r="B24" s="20">
-        <v>6583</v>
+        <v>3783</v>
       </c>
       <c r="C24" s="20">
-        <v>49252</v>
+        <v>53069</v>
       </c>
       <c r="D24" s="21">
         <v>228521</v>
       </c>
       <c r="E24" s="22">
-        <v>0.21552505021420351</v>
+        <v>0.23222811032684085</v>
       </c>
       <c r="F24" s="22">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G24" s="20">
-        <v>44511</v>
+        <v>49958</v>
       </c>
       <c r="H24" s="23">
-        <v>44458</v>
+        <v>47682</v>
       </c>
       <c r="I24" s="24">
-        <v>0.10651299678731108</v>
+        <v>6.2272308739341087E-2</v>
       </c>
       <c r="J24" s="22">
-        <v>0.10783211120608205</v>
+        <v>0.11297764355522011</v>
       </c>
       <c r="K24" s="16"/>
       <c r="L24" s="16" t="s">
@@ -29256,7 +29704,7 @@
         <v>17</v>
       </c>
       <c r="O24" s="27">
-        <v>49254</v>
+        <v>53071</v>
       </c>
     </row>
     <row r="25" spans="1:32" s="18" customFormat="1" ht="25.5" customHeight="1">
@@ -29264,31 +29712,31 @@
         <v>18</v>
       </c>
       <c r="B25" s="20">
-        <v>4201</v>
+        <v>2157</v>
       </c>
       <c r="C25" s="20">
-        <v>30098</v>
+        <v>32255</v>
       </c>
       <c r="D25" s="20">
         <v>100601</v>
       </c>
       <c r="E25" s="22">
-        <v>0.29918191668074873</v>
+        <v>0.32062305543682468</v>
       </c>
       <c r="F25" s="22">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G25" s="20">
-        <v>793</v>
+        <v>915</v>
       </c>
       <c r="H25" s="20">
-        <v>16422</v>
+        <v>17624</v>
       </c>
       <c r="I25" s="20">
-        <v>36.954602774274903</v>
+        <v>34.251366120218577</v>
       </c>
       <c r="J25" s="22">
-        <v>0.83278528802825469</v>
+        <v>0.83017476168860638</v>
       </c>
       <c r="K25" s="17"/>
       <c r="L25" s="17"/>
@@ -29297,7 +29745,7 @@
         <v>19</v>
       </c>
       <c r="O25" s="30">
-        <v>30100</v>
+        <v>32257</v>
       </c>
     </row>
     <row r="26" spans="1:32" s="18" customFormat="1" ht="25.5" customHeight="1">
@@ -29305,31 +29753,31 @@
         <v>20</v>
       </c>
       <c r="B26" s="20">
-        <v>2382</v>
+        <v>1626</v>
       </c>
       <c r="C26" s="20">
-        <v>19154</v>
+        <v>20814</v>
       </c>
       <c r="D26" s="20">
         <v>127920</v>
       </c>
       <c r="E26" s="22">
-        <v>0.14973420888055033</v>
+        <v>0.16271106941838648</v>
       </c>
       <c r="F26" s="22">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G26" s="20">
-        <v>44511</v>
+        <v>49958</v>
       </c>
       <c r="H26" s="20">
-        <v>28036</v>
+        <v>30058</v>
       </c>
       <c r="I26" s="22">
-        <v>-0.56967940509087645</v>
+        <v>-0.58337003082589378</v>
       </c>
       <c r="J26" s="22">
-        <v>-0.3168069624768155</v>
+        <v>-0.30753875840042588</v>
       </c>
       <c r="K26" s="17"/>
       <c r="L26" s="17"/>
@@ -29338,7 +29786,7 @@
         <v>21</v>
       </c>
       <c r="O26" s="31">
-        <v>19154</v>
+        <v>20814</v>
       </c>
     </row>
     <row r="27" spans="1:32" s="18" customFormat="1" ht="9.9499999999999993" customHeight="1">
@@ -29709,8 +30157,8 @@
       <c r="M33" s="41">
         <v>0</v>
       </c>
-      <c r="N33" s="41" t="e">
-        <v>#N/A</v>
+      <c r="N33" s="41">
+        <v>0</v>
       </c>
       <c r="O33" s="41" t="e">
         <v>#N/A</v>
@@ -29802,13 +30250,13 @@
         <v>36384</v>
       </c>
       <c r="L34" s="41">
-        <v>42671</v>
+        <v>42676</v>
       </c>
       <c r="M34" s="41">
-        <v>49254</v>
-      </c>
-      <c r="N34" s="41" t="e">
-        <v>#N/A</v>
+        <v>49288</v>
+      </c>
+      <c r="N34" s="41">
+        <v>53071</v>
       </c>
       <c r="O34" s="41" t="e">
         <v>#N/A</v>
@@ -30035,13 +30483,13 @@
         <v>3868</v>
       </c>
       <c r="L37" s="42">
-        <v>6287</v>
+        <v>6292</v>
       </c>
       <c r="M37" s="42">
-        <v>6583</v>
+        <v>6612</v>
       </c>
       <c r="N37" s="42">
-        <v>0</v>
+        <v>3783</v>
       </c>
       <c r="O37" s="42">
         <v>0</v>
@@ -30515,10 +30963,10 @@
         <v>26</v>
       </c>
       <c r="B49" s="37">
-        <v>49254</v>
+        <v>53071</v>
       </c>
       <c r="C49" s="46" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="D49" s="37"/>
       <c r="E49" s="37"/>
@@ -30555,7 +31003,7 @@
         <v>27</v>
       </c>
       <c r="B50" s="37">
-        <v>45304</v>
+        <v>50873</v>
       </c>
       <c r="C50" s="37"/>
       <c r="D50" s="37"/>
@@ -30633,7 +31081,7 @@
         <v>29</v>
       </c>
       <c r="B52" s="47">
-        <v>8.7188769203602412E-2</v>
+        <v>4.3205629705344695E-2</v>
       </c>
       <c r="C52" s="46"/>
       <c r="D52" s="37"/>
@@ -30711,10 +31159,10 @@
         <v>31</v>
       </c>
       <c r="B54" s="37">
-        <v>6583</v>
+        <v>3783</v>
       </c>
       <c r="C54" s="46" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D54" s="48"/>
       <c r="E54" s="48"/>
@@ -30786,7 +31234,7 @@
     </row>
     <row r="56" spans="1:32" s="38" customFormat="1" ht="14.1" customHeight="1">
       <c r="A56" s="49" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B56" s="48"/>
       <c r="C56" s="48"/>
@@ -30838,18 +31286,18 @@
       <c r="O57" s="4"/>
     </row>
     <row r="58" spans="1:32" ht="30.95" customHeight="1" thickBot="1">
-      <c r="A58" s="154" t="s">
+      <c r="A58" s="166" t="s">
         <v>33</v>
       </c>
-      <c r="B58" s="155"/>
-      <c r="C58" s="155"/>
-      <c r="D58" s="155"/>
-      <c r="E58" s="155"/>
-      <c r="F58" s="155"/>
-      <c r="G58" s="155"/>
-      <c r="H58" s="155"/>
-      <c r="I58" s="155"/>
-      <c r="J58" s="156"/>
+      <c r="B58" s="167"/>
+      <c r="C58" s="167"/>
+      <c r="D58" s="167"/>
+      <c r="E58" s="167"/>
+      <c r="F58" s="167"/>
+      <c r="G58" s="167"/>
+      <c r="H58" s="167"/>
+      <c r="I58" s="167"/>
+      <c r="J58" s="168"/>
       <c r="K58" s="4"/>
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
@@ -30902,10 +31350,10 @@
         <v>16</v>
       </c>
       <c r="B60" s="50">
-        <v>2382</v>
+        <v>1626</v>
       </c>
       <c r="C60" s="21">
-        <v>19154</v>
+        <v>20814</v>
       </c>
       <c r="D60" s="21">
         <v>0</v>
@@ -30914,19 +31362,19 @@
         <v>95</v>
       </c>
       <c r="F60" s="22">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G60" s="23">
-        <v>650</v>
+        <v>715</v>
       </c>
       <c r="H60" s="23">
-        <v>653</v>
+        <v>680</v>
       </c>
       <c r="I60" s="22">
-        <v>-0.21846153846153848</v>
+        <v>-0.24755244755244754</v>
       </c>
       <c r="J60" s="51">
-        <v>-0.222052067381317</v>
+        <v>-0.20882352941176474</v>
       </c>
       <c r="K60" s="16"/>
       <c r="L60" s="16" t="s">
@@ -30941,29 +31389,29 @@
         <v>35</v>
       </c>
       <c r="B61" s="52">
-        <v>1278</v>
+        <v>738</v>
       </c>
       <c r="C61" s="53">
-        <v>10817</v>
+        <v>11585</v>
       </c>
       <c r="D61" s="54"/>
       <c r="E61" s="55" t="s">
         <v>95</v>
       </c>
       <c r="F61" s="55">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G61" s="31">
-        <v>21687</v>
+        <v>24098</v>
       </c>
       <c r="H61" s="31">
-        <v>15322</v>
+        <v>16314</v>
       </c>
       <c r="I61" s="56">
-        <v>-0.50122193018859229</v>
+        <v>-0.51925470993443446</v>
       </c>
       <c r="J61" s="57">
-        <v>-0.29402166818953135</v>
+        <v>-0.28987372808630629</v>
       </c>
       <c r="K61" s="17"/>
       <c r="L61" s="17"/>
@@ -30976,29 +31424,29 @@
         <v>36</v>
       </c>
       <c r="B62" s="52">
-        <v>975</v>
+        <v>786</v>
       </c>
       <c r="C62" s="53">
-        <v>7110</v>
+        <v>7900</v>
       </c>
       <c r="D62" s="54"/>
       <c r="E62" s="55" t="s">
         <v>95</v>
       </c>
       <c r="F62" s="55">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G62" s="31">
-        <v>20327</v>
+        <v>23084</v>
       </c>
       <c r="H62" s="31">
-        <v>11113</v>
+        <v>12037</v>
       </c>
       <c r="I62" s="56">
-        <v>-0.65021892064741471</v>
+        <v>-0.65777161670421069</v>
       </c>
       <c r="J62" s="57">
-        <v>-0.36020876451003325</v>
+        <v>-0.34369028827781012</v>
       </c>
       <c r="K62" s="17"/>
       <c r="L62" s="17"/>
@@ -31011,29 +31459,29 @@
         <v>37</v>
       </c>
       <c r="B63" s="59">
-        <v>129</v>
+        <v>102</v>
       </c>
       <c r="C63" s="60">
-        <v>1227</v>
+        <v>1329</v>
       </c>
       <c r="D63" s="61"/>
       <c r="E63" s="62" t="s">
         <v>95</v>
       </c>
       <c r="F63" s="62">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G63" s="63">
-        <v>2497</v>
+        <v>2776</v>
       </c>
       <c r="H63" s="63">
-        <v>1601</v>
+        <v>1707</v>
       </c>
       <c r="I63" s="64">
-        <v>-0.50861033239887865</v>
+        <v>-0.52125360230547546</v>
       </c>
       <c r="J63" s="65">
-        <v>-0.23360399750156158</v>
+        <v>-0.2214411247803163</v>
       </c>
       <c r="K63" s="17"/>
       <c r="L63" s="17"/>
@@ -31502,13 +31950,13 @@
         <v>14677</v>
       </c>
       <c r="L71" s="41">
-        <v>16772</v>
+        <v>16777</v>
       </c>
       <c r="M71" s="41">
-        <v>19154</v>
-      </c>
-      <c r="N71" s="41" t="e">
-        <v>#N/A</v>
+        <v>19188</v>
+      </c>
+      <c r="N71" s="41">
+        <v>20814</v>
       </c>
       <c r="O71" s="41" t="e">
         <v>#N/A</v>
@@ -31796,12 +32244,14 @@
         <v>1381</v>
       </c>
       <c r="L74" s="42">
-        <v>2095</v>
+        <v>2100</v>
       </c>
       <c r="M74" s="42">
-        <v>2382</v>
-      </c>
-      <c r="N74" s="42"/>
+        <v>2411</v>
+      </c>
+      <c r="N74" s="42">
+        <v>1626</v>
+      </c>
       <c r="O74" s="42"/>
       <c r="P74" s="42"/>
       <c r="Q74" s="42"/>
@@ -32003,13 +32453,13 @@
         <v>-0.59560761346998536</v>
       </c>
       <c r="L78" s="66">
-        <v>-0.42696936542669583</v>
+        <v>-0.42560175054704596</v>
       </c>
       <c r="M78" s="66">
-        <v>-0.47300884955752215</v>
+        <v>-0.46659292035398231</v>
       </c>
       <c r="N78" s="66">
-        <v>-1</v>
+        <v>-0.70148705709564896</v>
       </c>
       <c r="O78" s="66">
         <v>-1</v>
@@ -32300,10 +32750,10 @@
         <v>25</v>
       </c>
       <c r="B85" s="37">
-        <v>19154</v>
+        <v>20814</v>
       </c>
       <c r="C85" s="46" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="D85" s="37"/>
       <c r="E85" s="37"/>
@@ -32340,10 +32790,10 @@
         <v>26</v>
       </c>
       <c r="B86" s="37">
-        <v>44511</v>
+        <v>49958</v>
       </c>
       <c r="C86" s="46" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D86" s="37"/>
       <c r="E86" s="37"/>
@@ -32380,7 +32830,7 @@
         <v>27</v>
       </c>
       <c r="B87" s="37">
-        <v>115413</v>
+        <v>136266</v>
       </c>
       <c r="C87" s="37"/>
       <c r="D87" s="37"/>
@@ -32418,10 +32868,10 @@
         <v>28</v>
       </c>
       <c r="B88" s="37">
-        <v>2.3238488044272736</v>
+        <v>2.400211396175651</v>
       </c>
       <c r="C88" s="46" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D88" s="37"/>
       <c r="E88" s="37"/>
@@ -32458,7 +32908,7 @@
         <v>29</v>
       </c>
       <c r="B89" s="47">
-        <v>-0.61433287411296822</v>
+        <v>-0.63337883257745875</v>
       </c>
       <c r="C89" s="46"/>
       <c r="D89" s="37"/>
@@ -32496,10 +32946,10 @@
         <v>30</v>
       </c>
       <c r="B90" s="37">
-        <v>2382</v>
+        <v>1626</v>
       </c>
       <c r="C90" s="46" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D90" s="48"/>
       <c r="E90" s="48"/>
@@ -32536,10 +32986,10 @@
         <v>31</v>
       </c>
       <c r="B91" s="37">
-        <v>4520</v>
+        <v>5447</v>
       </c>
       <c r="C91" s="46" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D91" s="48"/>
       <c r="E91" s="48"/>
@@ -32576,7 +33026,7 @@
         <v>32</v>
       </c>
       <c r="B92" s="47">
-        <v>1.8975650713685979</v>
+        <v>3.3499384993849937</v>
       </c>
       <c r="C92" s="48"/>
       <c r="D92" s="48"/>
@@ -32611,7 +33061,7 @@
     </row>
     <row r="93" spans="1:32" s="38" customFormat="1" ht="14.1" customHeight="1">
       <c r="A93" s="49" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B93" s="48"/>
       <c r="C93" s="48"/>
@@ -32727,10 +33177,10 @@
         <v>16</v>
       </c>
       <c r="B97" s="68">
-        <v>4201</v>
+        <v>2157</v>
       </c>
       <c r="C97" s="21">
-        <v>30098</v>
+        <v>32255</v>
       </c>
       <c r="D97" s="21">
         <v>0</v>
@@ -32739,19 +33189,19 @@
         <v>95</v>
       </c>
       <c r="F97" s="22">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="G97" s="23">
-        <v>793</v>
+        <v>915</v>
       </c>
       <c r="H97" s="23">
-        <v>16422</v>
+        <v>17624</v>
       </c>
       <c r="I97" s="22">
-        <v>36.954602774274903</v>
+        <v>34.251366120218577</v>
       </c>
       <c r="J97" s="22">
-        <v>0.83278528802825469</v>
+        <v>0.83017476168860638</v>
       </c>
       <c r="K97" s="16"/>
       <c r="L97" s="16" t="s">
@@ -33227,8 +33677,8 @@
       <c r="M105" s="41">
         <v>30100</v>
       </c>
-      <c r="N105" s="41" t="e">
-        <v>#N/A</v>
+      <c r="N105" s="41">
+        <v>32257</v>
       </c>
       <c r="O105" s="41" t="e">
         <v>#N/A</v>
@@ -33521,7 +33971,9 @@
       <c r="M108" s="69">
         <v>4201</v>
       </c>
-      <c r="N108" s="69"/>
+      <c r="N108" s="69">
+        <v>2157</v>
+      </c>
       <c r="O108" s="69"/>
       <c r="P108" s="69"/>
       <c r="Q108" s="69"/>
@@ -34066,10 +34518,10 @@
         <v>26</v>
       </c>
       <c r="B121" s="37">
-        <v>167765</v>
+        <v>200022</v>
       </c>
       <c r="C121" s="46" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D121" s="37"/>
       <c r="E121" s="37"/>
@@ -34106,7 +34558,7 @@
         <v>27</v>
       </c>
       <c r="B122" s="37">
-        <v>16422</v>
+        <v>17624</v>
       </c>
       <c r="C122" s="37"/>
       <c r="D122" s="37"/>
@@ -34184,7 +34636,7 @@
         <v>29</v>
       </c>
       <c r="B124" s="47">
-        <v>9.2158689562781628</v>
+        <v>10.349409895596914</v>
       </c>
       <c r="C124" s="46"/>
       <c r="D124" s="37"/>
@@ -34262,10 +34714,10 @@
         <v>31</v>
       </c>
       <c r="B126" s="37">
-        <v>30100</v>
+        <v>32257</v>
       </c>
       <c r="C126" s="46" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D126" s="48"/>
       <c r="E126" s="48"/>
@@ -34337,7 +34789,7 @@
     </row>
     <row r="128" spans="1:32" s="38" customFormat="1" ht="14.1" customHeight="1">
       <c r="A128" s="49" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B128" s="48"/>
       <c r="C128" s="48"/>
@@ -34511,7 +34963,7 @@
         <v>95</v>
       </c>
       <c r="E134" s="78">
-        <v>0.4</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="F134" s="78" t="e">
         <v>#REF!</v>
@@ -34574,7 +35026,7 @@
       <c r="M137" s="86"/>
       <c r="N137" s="86"/>
       <c r="O137" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="138" spans="1:32">
@@ -34586,21 +35038,21 @@
       <c r="D138" s="158"/>
       <c r="E138" s="158"/>
       <c r="F138" s="159"/>
-      <c r="G138" s="168" t="s">
+      <c r="G138" s="161" t="s">
         <v>55</v>
       </c>
-      <c r="H138" s="169"/>
-      <c r="I138" s="169"/>
-      <c r="J138" s="170" t="s">
+      <c r="H138" s="162"/>
+      <c r="I138" s="162"/>
+      <c r="J138" s="163" t="s">
         <v>56</v>
       </c>
-      <c r="K138" s="171"/>
-      <c r="L138" s="171"/>
-      <c r="M138" s="170" t="s">
+      <c r="K138" s="164"/>
+      <c r="L138" s="164"/>
+      <c r="M138" s="163" t="s">
         <v>57</v>
       </c>
-      <c r="N138" s="171"/>
-      <c r="O138" s="172"/>
+      <c r="N138" s="164"/>
+      <c r="O138" s="165"/>
     </row>
     <row r="139" spans="1:32" ht="42.75">
       <c r="A139" s="88" t="s">
@@ -34657,43 +35109,43 @@
         <v>0</v>
       </c>
       <c r="C140" s="92">
-        <v>19154</v>
+        <v>20814</v>
       </c>
       <c r="D140" s="93">
         <v>0</v>
       </c>
       <c r="E140" s="93">
-        <v>-0.56967940509087645</v>
+        <v>-0.58337003082589378</v>
       </c>
       <c r="F140" s="94">
-        <v>-0.3168069624768155</v>
+        <v>-0.30753875840042588</v>
       </c>
       <c r="G140" s="95">
-        <v>10817</v>
+        <v>11585</v>
       </c>
       <c r="H140" s="93">
-        <v>-0.50122193018859229</v>
+        <v>-0.51925470993443446</v>
       </c>
       <c r="I140" s="93">
-        <v>-0.29402166818953135</v>
+        <v>-0.28987372808630629</v>
       </c>
       <c r="J140" s="96">
-        <v>7110</v>
+        <v>7900</v>
       </c>
       <c r="K140" s="93">
-        <v>-0.65021892064741471</v>
+        <v>-0.65777161670421069</v>
       </c>
       <c r="L140" s="93">
-        <v>-0.36020876451003325</v>
+        <v>-0.34369028827781012</v>
       </c>
       <c r="M140" s="96">
-        <v>1227</v>
+        <v>1329</v>
       </c>
       <c r="N140" s="93">
-        <v>-0.50861033239887865</v>
+        <v>-0.52125360230547546</v>
       </c>
       <c r="O140" s="94">
-        <v>-0.23360399750156158</v>
+        <v>-0.2214411247803163</v>
       </c>
     </row>
     <row r="141" spans="1:32" ht="15.75">
@@ -35175,7 +35627,7 @@
       <c r="D153" s="110"/>
       <c r="E153" s="110"/>
       <c r="F153" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J153" s="109"/>
       <c r="K153" s="111"/>
@@ -35185,7 +35637,7 @@
       <c r="M153" s="110"/>
       <c r="N153" s="110"/>
       <c r="O153" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="154" spans="1:15" ht="24.6" customHeight="1">
@@ -35234,16 +35686,16 @@
         <v>0</v>
       </c>
       <c r="C155" s="92">
-        <v>3431</v>
+        <v>3717</v>
       </c>
       <c r="D155" s="93">
         <v>0</v>
       </c>
       <c r="E155" s="93">
-        <v>-0.63792739552553823</v>
+        <v>-0.65147679324894514</v>
       </c>
       <c r="F155" s="94">
-        <v>-0.41738835116318562</v>
+        <v>-0.41418439716312061</v>
       </c>
       <c r="J155" s="114" t="s">
         <v>16</v>
@@ -35252,16 +35704,16 @@
         <v>0</v>
       </c>
       <c r="L155" s="92">
-        <v>5747</v>
+        <v>6288</v>
       </c>
       <c r="M155" s="93">
         <v>0</v>
       </c>
       <c r="N155" s="93">
-        <v>-0.59148421950526009</v>
+        <v>-0.6018489204077756</v>
       </c>
       <c r="O155" s="94">
-        <v>-0.41796637634190803</v>
+        <v>-0.40392454261067401</v>
       </c>
     </row>
     <row r="156" spans="1:15" ht="15.75">
@@ -35653,7 +36105,7 @@
       <c r="D168" s="110"/>
       <c r="E168" s="110"/>
       <c r="F168" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J168" s="109"/>
       <c r="K168" s="110"/>
@@ -35663,7 +36115,7 @@
       <c r="M168" s="110"/>
       <c r="N168" s="110"/>
       <c r="O168" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="169" spans="1:15" ht="26.45" customHeight="1">
@@ -35712,16 +36164,16 @@
         <v>0</v>
       </c>
       <c r="C170" s="92">
-        <v>1247</v>
+        <v>1329</v>
       </c>
       <c r="D170" s="93">
         <v>0</v>
       </c>
       <c r="E170" s="93">
-        <v>-0.77767873061151715</v>
+        <v>-0.78974845752254397</v>
       </c>
       <c r="F170" s="94">
-        <v>-0.24424242424242426</v>
+        <v>-0.24531516183986368</v>
       </c>
       <c r="J170" s="114" t="s">
         <v>16</v>
@@ -35730,16 +36182,16 @@
         <v>0</v>
       </c>
       <c r="L170" s="92">
-        <v>2853</v>
+        <v>3112</v>
       </c>
       <c r="M170" s="93">
         <v>0</v>
       </c>
       <c r="N170" s="93">
-        <v>-0.65338354999392534</v>
+        <v>-0.66432963002912304</v>
       </c>
       <c r="O170" s="94">
-        <v>-0.33728222996515678</v>
+        <v>-0.32611520138588135</v>
       </c>
     </row>
     <row r="171" spans="1:15" ht="15.75">
@@ -35750,16 +36202,16 @@
         <v>0</v>
       </c>
       <c r="C171" s="116">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="D171" s="98">
         <v>0</v>
       </c>
       <c r="E171" s="98">
-        <v>-0.7880658436213992</v>
+        <v>-0.78691588785046729</v>
       </c>
       <c r="F171" s="117">
-        <v>-0.28965517241379313</v>
+        <v>-0.24503311258278149</v>
       </c>
       <c r="J171" s="115" t="e">
         <v>#N/A</v>
@@ -35788,16 +36240,16 @@
         <v>0</v>
       </c>
       <c r="C172" s="116">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D172" s="98">
         <v>0</v>
       </c>
       <c r="E172" s="98">
-        <v>-0.81305114638447973</v>
+        <v>-0.83234421364985167</v>
       </c>
       <c r="F172" s="117">
-        <v>-0.29333333333333333</v>
+        <v>-0.33136094674556216</v>
       </c>
       <c r="J172" s="115" t="e">
         <v>#N/A</v>
@@ -35826,16 +36278,16 @@
         <v>0</v>
       </c>
       <c r="C173" s="116">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="D173" s="98">
         <v>0</v>
       </c>
       <c r="E173" s="98">
-        <v>-0.68562874251497008</v>
+        <v>-0.69931972789115648</v>
       </c>
       <c r="F173" s="117">
-        <v>-0.13580246913580252</v>
+        <v>-0.15969581749049433</v>
       </c>
       <c r="J173" s="115" t="e">
         <v>#N/A</v>
@@ -35864,16 +36316,16 @@
         <v>0</v>
       </c>
       <c r="C174" s="116">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="D174" s="98">
         <v>0</v>
       </c>
       <c r="E174" s="98">
-        <v>-0.83586337760910823</v>
+        <v>-0.8435146443514645</v>
       </c>
       <c r="F174" s="117">
-        <v>-0.23451327433628322</v>
+        <v>-0.20425531914893613</v>
       </c>
       <c r="J174" s="115" t="e">
         <v>#N/A</v>
@@ -35902,16 +36354,16 @@
         <v>0</v>
       </c>
       <c r="C175" s="116">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="D175" s="98">
         <v>0</v>
       </c>
       <c r="E175" s="98">
-        <v>-0.69673704414587334</v>
+        <v>-0.70862068965517233</v>
       </c>
       <c r="F175" s="117">
-        <v>-0.34979423868312753</v>
+        <v>-0.34496124031007747</v>
       </c>
       <c r="J175" s="115" t="e">
         <v>#N/A</v>
@@ -35940,16 +36392,16 @@
         <v>0</v>
       </c>
       <c r="C176" s="116">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D176" s="98">
         <v>0</v>
       </c>
       <c r="E176" s="98">
-        <v>-0.82282282282282282</v>
+        <v>-0.83641160949868076</v>
       </c>
       <c r="F176" s="117">
-        <v>-0.42439024390243907</v>
+        <v>-0.43891402714932126</v>
       </c>
       <c r="J176" s="115" t="e">
         <v>#N/A</v>
@@ -35978,16 +36430,16 @@
         <v>0</v>
       </c>
       <c r="C177" s="116">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D177" s="98">
         <v>0</v>
       </c>
       <c r="E177" s="98">
-        <v>-0.69230769230769229</v>
+        <v>-0.69786096256684493</v>
       </c>
       <c r="F177" s="117">
-        <v>9.7087378640776656E-3</v>
+        <v>1.8018018018018056E-2</v>
       </c>
       <c r="J177" s="115" t="e">
         <v>#N/A</v>
@@ -36016,16 +36468,16 @@
         <v>0</v>
       </c>
       <c r="C178" s="116">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D178" s="98">
         <v>0</v>
       </c>
       <c r="E178" s="98">
-        <v>-0.57615894039735105</v>
+        <v>-0.61309523809523814</v>
       </c>
       <c r="F178" s="117">
-        <v>-7.2463768115942018E-2</v>
+        <v>-0.1333333333333333</v>
       </c>
       <c r="J178" s="115" t="e">
         <v>#N/A</v>
@@ -36054,16 +36506,16 @@
         <v>0</v>
       </c>
       <c r="C179" s="116">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="D179" s="98">
         <v>0</v>
       </c>
       <c r="E179" s="98">
-        <v>-0.8349307774227902</v>
+        <v>-0.84528301886792456</v>
       </c>
       <c r="F179" s="117">
-        <v>-0.10919540229885061</v>
+        <v>-9.392265193370164E-2</v>
       </c>
       <c r="J179" s="115" t="e">
         <v>#N/A</v>
@@ -36092,16 +36544,16 @@
         <v>0</v>
       </c>
       <c r="C180" s="119">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D180" s="104">
         <v>0</v>
       </c>
       <c r="E180" s="104">
-        <v>-0.74429223744292239</v>
+        <v>-0.75619834710743805</v>
       </c>
       <c r="F180" s="120">
-        <v>-0.39130434782608692</v>
+        <v>-0.39175257731958768</v>
       </c>
       <c r="J180" s="118" t="e">
         <v>#N/A</v>
@@ -36131,7 +36583,7 @@
       <c r="D183" s="110"/>
       <c r="E183" s="110"/>
       <c r="F183" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J183" s="109"/>
       <c r="K183" s="110"/>
@@ -36141,7 +36593,7 @@
       <c r="M183" s="110"/>
       <c r="N183" s="110"/>
       <c r="O183" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="184" spans="1:20" ht="26.45" customHeight="1">
@@ -36190,16 +36642,16 @@
         <v>0</v>
       </c>
       <c r="C185" s="92">
-        <v>565</v>
+        <v>605</v>
       </c>
       <c r="D185" s="93">
         <v>0</v>
       </c>
       <c r="E185" s="93">
-        <v>-0.79558610709117228</v>
+        <v>-0.80305989583333337</v>
       </c>
       <c r="F185" s="94">
-        <v>-4.2372881355932202E-2</v>
+        <v>-5.0235478806907374E-2</v>
       </c>
       <c r="J185" s="114" t="s">
         <v>16</v>
@@ -36208,16 +36660,16 @@
         <v>0</v>
       </c>
       <c r="L185" s="92">
-        <v>2927</v>
+        <v>3191</v>
       </c>
       <c r="M185" s="93">
         <v>0</v>
       </c>
       <c r="N185" s="93">
-        <v>-2.8865295288653003E-2</v>
+        <v>-5.1990493166963803E-2</v>
       </c>
       <c r="O185" s="94">
-        <v>-0.23437091289563172</v>
+        <v>-0.22378983215762593</v>
       </c>
     </row>
     <row r="186" spans="1:20" ht="15.75">
@@ -36611,7 +37063,7 @@
       <c r="D198" s="110"/>
       <c r="E198" s="110"/>
       <c r="F198" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J198" s="109"/>
       <c r="K198" s="110"/>
@@ -36621,7 +37073,7 @@
       <c r="M198" s="110"/>
       <c r="N198" s="110"/>
       <c r="O198" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="199" spans="1:15" ht="23.45" hidden="1" customHeight="1">
@@ -36670,16 +37122,16 @@
         <v>0</v>
       </c>
       <c r="C200" s="92">
-        <v>565</v>
+        <v>605</v>
       </c>
       <c r="D200" s="93">
         <v>0</v>
       </c>
       <c r="E200" s="93">
-        <v>-0.79558610709117228</v>
+        <v>-0.80305989583333337</v>
       </c>
       <c r="F200" s="94">
-        <v>-4.2372881355932202E-2</v>
+        <v>-5.0235478806907374E-2</v>
       </c>
       <c r="J200" s="114" t="s">
         <v>16</v>
@@ -37015,7 +37467,7 @@
       <c r="D211" s="110"/>
       <c r="E211" s="110"/>
       <c r="F211" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J211" s="109"/>
       <c r="K211" s="110"/>
@@ -37025,7 +37477,7 @@
       <c r="M211" s="110"/>
       <c r="N211" s="110"/>
       <c r="O211" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="212" spans="1:18" ht="26.1" customHeight="1">
@@ -37079,16 +37531,16 @@
         <v>0</v>
       </c>
       <c r="C213" s="92">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="D213" s="93">
         <v>0</v>
       </c>
       <c r="E213" s="93">
-        <v>-0.85172413793103452</v>
+        <v>-0.85244161358811044</v>
       </c>
       <c r="F213" s="94">
-        <v>-0.16774193548387095</v>
+        <v>-0.15757575757575759</v>
       </c>
       <c r="J213" s="114" t="s">
         <v>16</v>
@@ -37097,19 +37549,19 @@
         <v>0</v>
       </c>
       <c r="L213" s="92">
-        <v>3808</v>
+        <v>4029</v>
       </c>
       <c r="M213" s="93">
         <v>0</v>
       </c>
       <c r="N213" s="93">
-        <v>3.8020176544766713</v>
+        <v>3.4032786885245905</v>
       </c>
       <c r="O213" s="125">
-        <v>-5.2246603970741434E-3</v>
+        <v>-2.5163319622550251E-2</v>
       </c>
       <c r="P213" s="126">
-        <v>4201</v>
+        <v>2157</v>
       </c>
       <c r="Q213" s="124"/>
       <c r="R213" s="124"/>
@@ -37512,7 +37964,7 @@
       <c r="D226" s="110"/>
       <c r="E226" s="110"/>
       <c r="F226" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="J226" s="109"/>
       <c r="K226" s="110"/>
@@ -37522,7 +37974,7 @@
       <c r="M226" s="110"/>
       <c r="N226" s="110"/>
       <c r="O226" s="87" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="227" spans="1:15" ht="42.75">
@@ -37571,7 +38023,7 @@
         <v>0</v>
       </c>
       <c r="C228" s="92">
-        <v>3351</v>
+        <v>3546</v>
       </c>
       <c r="D228" s="93">
         <v>0</v>
@@ -37580,7 +38032,7 @@
         <v>0</v>
       </c>
       <c r="F228" s="94">
-        <v>-0.20460479468312365</v>
+        <v>-0.21513944223107573</v>
       </c>
       <c r="J228" s="114" t="s">
         <v>16</v>
@@ -37589,7 +38041,7 @@
         <v>0</v>
       </c>
       <c r="L228" s="92">
-        <v>6344</v>
+        <v>6753</v>
       </c>
       <c r="M228" s="93">
         <v>0</v>
@@ -37598,7 +38050,7 @@
         <v>0</v>
       </c>
       <c r="O228" s="94">
-        <v>-0.23279719434030721</v>
+        <v>-0.23669040352661919</v>
       </c>
     </row>
     <row r="229" spans="1:15" ht="15.75">
@@ -37982,8 +38434,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A58:J58"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="D141:D150">

</xml_diff>

<commit_message>
Rebuild arrival dashboard from source arrival tables
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -8,17 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkCode\AI_Digest\data\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19178379-C8FE-4531-9519-AC998A606777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9915AA-9686-472C-9BF2-6C58EC1E9F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4F6CCF54-37E5-4816-9B51-3E2CFD892ED8}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4F6CCF54-37E5-4816-9B51-3E2CFD892ED8}"/>
   </bookViews>
   <sheets>
     <sheet name="来店日趋势汇总" sheetId="2" r:id="rId1"/>
     <sheet name="来店简报" sheetId="1" r:id="rId2"/>
+    <sheet name="NEV本期来店" sheetId="3" r:id="rId3"/>
+    <sheet name="NEV同期来店" sheetId="4" r:id="rId4"/>
+    <sheet name="ICE本期来店" sheetId="5" r:id="rId5"/>
+    <sheet name="ICE同期来店" sheetId="6" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
-    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="214">
   <si>
     <t>简报模板</t>
     <phoneticPr fontId="4" type="noConversion"/>
@@ -436,6 +440,273 @@
   <si>
     <t>统计周期4.1-4.13</t>
   </si>
+  <si>
+    <t>日期</t>
+  </si>
+  <si>
+    <t>来店量</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-04</t>
+  </si>
+  <si>
+    <t>2026-04-05</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>2026-04-12</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>日(日期)</t>
+  </si>
+  <si>
+    <t>2026年4月1日</t>
+  </si>
+  <si>
+    <t>2026年4月2日</t>
+  </si>
+  <si>
+    <t>2026年4月3日</t>
+  </si>
+  <si>
+    <t>2026年4月4日</t>
+  </si>
+  <si>
+    <t>2026年4月5日</t>
+  </si>
+  <si>
+    <t>2026年4月6日</t>
+  </si>
+  <si>
+    <t>2026年4月7日</t>
+  </si>
+  <si>
+    <t>2026年4月8日</t>
+  </si>
+  <si>
+    <t>2026年4月9日</t>
+  </si>
+  <si>
+    <t>2026年4月10日</t>
+  </si>
+  <si>
+    <t>2026年4月11日</t>
+  </si>
+  <si>
+    <t>2026年4月12日</t>
+  </si>
+  <si>
+    <t>2026年4月13日</t>
+  </si>
+  <si>
+    <t>2025年4月1日</t>
+  </si>
+  <si>
+    <t>2025年4月2日</t>
+  </si>
+  <si>
+    <t>2025年4月3日</t>
+  </si>
+  <si>
+    <t>2025年4月4日</t>
+  </si>
+  <si>
+    <t>2025年4月5日</t>
+  </si>
+  <si>
+    <t>2025年4月6日</t>
+  </si>
+  <si>
+    <t>2025年4月7日</t>
+  </si>
+  <si>
+    <t>2025年4月8日</t>
+  </si>
+  <si>
+    <t>2025年4月9日</t>
+  </si>
+  <si>
+    <t>2025年4月10日</t>
+  </si>
+  <si>
+    <t>2025年4月11日</t>
+  </si>
+  <si>
+    <t>2025年4月12日</t>
+  </si>
+  <si>
+    <t>2025年4月13日</t>
+  </si>
+  <si>
+    <t>2025年4月14日</t>
+  </si>
+  <si>
+    <t>2025年4月15日</t>
+  </si>
+  <si>
+    <t>2025年4月16日</t>
+  </si>
+  <si>
+    <t>2025年4月17日</t>
+  </si>
+  <si>
+    <t>2025年4月18日</t>
+  </si>
+  <si>
+    <t>2025年4月19日</t>
+  </si>
+  <si>
+    <t>2025年4月20日</t>
+  </si>
+  <si>
+    <t>2025年4月21日</t>
+  </si>
+  <si>
+    <t>2025年4月22日</t>
+  </si>
+  <si>
+    <t>2025年4月23日</t>
+  </si>
+  <si>
+    <t>2025年4月24日</t>
+  </si>
+  <si>
+    <t>2025年4月25日</t>
+  </si>
+  <si>
+    <t>2025年4月26日</t>
+  </si>
+  <si>
+    <t>2025年4月27日</t>
+  </si>
+  <si>
+    <t>2025年4月28日</t>
+  </si>
+  <si>
+    <t>2025年4月29日</t>
+  </si>
+  <si>
+    <t>2025年4月30日</t>
+  </si>
+  <si>
+    <t>2025-04-01</t>
+  </si>
+  <si>
+    <t>2025-04-02</t>
+  </si>
+  <si>
+    <t>2025-04-03</t>
+  </si>
+  <si>
+    <t>2025-04-04</t>
+  </si>
+  <si>
+    <t>2025-04-05</t>
+  </si>
+  <si>
+    <t>2025-04-06</t>
+  </si>
+  <si>
+    <t>2025-04-07</t>
+  </si>
+  <si>
+    <t>2025-04-08</t>
+  </si>
+  <si>
+    <t>2025-04-09</t>
+  </si>
+  <si>
+    <t>2025-04-10</t>
+  </si>
+  <si>
+    <t>2025-04-11</t>
+  </si>
+  <si>
+    <t>2025-04-12</t>
+  </si>
+  <si>
+    <t>2025-04-13</t>
+  </si>
+  <si>
+    <t>2025-04-14</t>
+  </si>
+  <si>
+    <t>2025-04-15</t>
+  </si>
+  <si>
+    <t>2025-04-16</t>
+  </si>
+  <si>
+    <t>2025-04-17</t>
+  </si>
+  <si>
+    <t>2025-04-18</t>
+  </si>
+  <si>
+    <t>2025-04-19</t>
+  </si>
+  <si>
+    <t>2025-04-20</t>
+  </si>
+  <si>
+    <t>2025-04-21</t>
+  </si>
+  <si>
+    <t>2025-04-22</t>
+  </si>
+  <si>
+    <t>2025-04-23</t>
+  </si>
+  <si>
+    <t>2025-04-24</t>
+  </si>
+  <si>
+    <t>2025-04-25</t>
+  </si>
+  <si>
+    <t>2025-04-26</t>
+  </si>
+  <si>
+    <t>2025-04-27</t>
+  </si>
+  <si>
+    <t>2025-04-28</t>
+  </si>
+  <si>
+    <t>2025-04-29</t>
+  </si>
+  <si>
+    <t>2025-04-30</t>
+  </si>
 </sst>
 </file>
 
@@ -446,7 +717,7 @@
     <numFmt numFmtId="177" formatCode="0.0%"/>
     <numFmt numFmtId="178" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -652,6 +923,20 @@
     <font>
       <sz val="9"/>
       <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="黑体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1126,7 +1411,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1632,232 +1917,21 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="百分比" xfId="1" builtinId="5"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="49">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="27">
     <dxf>
       <font>
         <color theme="0"/>
@@ -29164,27 +29238,27 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="C33 I33 O33 U33 AA33">
-    <cfRule type="expression" dxfId="48" priority="4">
+    <cfRule type="expression" dxfId="26" priority="4">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C31:AF31">
-    <cfRule type="expression" dxfId="47" priority="2">
+    <cfRule type="expression" dxfId="25" priority="2">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C74:AF77">
-    <cfRule type="expression" dxfId="46" priority="5">
+    <cfRule type="expression" dxfId="24" priority="5">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C117:AF120">
-    <cfRule type="expression" dxfId="45" priority="3">
+    <cfRule type="expression" dxfId="23" priority="3">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D33:H36 J33:N36 P33:T37 V33:Z37 AB33:AF37 M37:N37">
-    <cfRule type="expression" dxfId="44" priority="1">
+    <cfRule type="expression" dxfId="22" priority="1">
       <formula>#REF!&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38486,4 +38560,776 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ADF50C6-13A6-4168-A17A-E17785AA487D}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="2" width="9.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15" customHeight="1">
+      <c r="A1" s="173" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="173" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15" customHeight="1">
+      <c r="A2" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="69">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" customHeight="1">
+      <c r="A3" s="69" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="69">
+        <v>1524</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" customHeight="1">
+      <c r="A4" s="69" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" s="69">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" customHeight="1">
+      <c r="A5" s="69" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" s="69">
+        <v>3001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15" customHeight="1">
+      <c r="A6" s="69" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="69">
+        <v>2826</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15" customHeight="1">
+      <c r="A7" s="69" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" s="69">
+        <v>2731</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15" customHeight="1">
+      <c r="A8" s="69" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="69">
+        <v>1827</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" customHeight="1">
+      <c r="A9" s="69" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="69">
+        <v>1933</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15" customHeight="1">
+      <c r="A10" s="69" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="69">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15" customHeight="1">
+      <c r="A11" s="69" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" s="69">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15" customHeight="1">
+      <c r="A12" s="69" t="s">
+        <v>137</v>
+      </c>
+      <c r="B12" s="69">
+        <v>4192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1">
+      <c r="A13" s="69" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" s="69">
+        <v>4201</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" customHeight="1">
+      <c r="A14" s="69" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="69">
+        <v>2157</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A97DAB-DB21-4C58-9A62-D25173AB7A23}">
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="2" width="9.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15" customHeight="1">
+      <c r="A1" s="173" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="173" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15" customHeight="1">
+      <c r="A2" s="69" t="s">
+        <v>184</v>
+      </c>
+      <c r="B2" s="69">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" customHeight="1">
+      <c r="A3" s="69" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="69">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" customHeight="1">
+      <c r="A4" s="69" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" s="69">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" customHeight="1">
+      <c r="A5" s="69" t="s">
+        <v>187</v>
+      </c>
+      <c r="B5" s="69">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15" customHeight="1">
+      <c r="A6" s="69" t="s">
+        <v>188</v>
+      </c>
+      <c r="B6" s="69">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15" customHeight="1">
+      <c r="A7" s="69" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" s="69">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15" customHeight="1">
+      <c r="A8" s="69" t="s">
+        <v>190</v>
+      </c>
+      <c r="B8" s="69">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" customHeight="1">
+      <c r="A9" s="69" t="s">
+        <v>191</v>
+      </c>
+      <c r="B9" s="69">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15" customHeight="1">
+      <c r="A10" s="69" t="s">
+        <v>192</v>
+      </c>
+      <c r="B10" s="69">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15" customHeight="1">
+      <c r="A11" s="69" t="s">
+        <v>193</v>
+      </c>
+      <c r="B11" s="69">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15" customHeight="1">
+      <c r="A12" s="69" t="s">
+        <v>194</v>
+      </c>
+      <c r="B12" s="69">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1">
+      <c r="A13" s="69" t="s">
+        <v>195</v>
+      </c>
+      <c r="B13" s="69">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" customHeight="1">
+      <c r="A14" s="69" t="s">
+        <v>196</v>
+      </c>
+      <c r="B14" s="69">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15" customHeight="1">
+      <c r="A15" s="69" t="s">
+        <v>197</v>
+      </c>
+      <c r="B15" s="69">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15" customHeight="1">
+      <c r="A16" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="B16" s="69">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15" customHeight="1">
+      <c r="A17" s="69" t="s">
+        <v>199</v>
+      </c>
+      <c r="B17" s="69">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15" customHeight="1">
+      <c r="A18" s="69" t="s">
+        <v>200</v>
+      </c>
+      <c r="B18" s="69">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15" customHeight="1">
+      <c r="A19" s="69" t="s">
+        <v>201</v>
+      </c>
+      <c r="B19" s="69">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15" customHeight="1">
+      <c r="A20" s="69" t="s">
+        <v>202</v>
+      </c>
+      <c r="B20" s="69">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15" customHeight="1">
+      <c r="A21" s="69" t="s">
+        <v>203</v>
+      </c>
+      <c r="B21" s="69">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15" customHeight="1">
+      <c r="A22" s="69" t="s">
+        <v>204</v>
+      </c>
+      <c r="B22" s="69">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15" customHeight="1">
+      <c r="A23" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="B23" s="69">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15" customHeight="1">
+      <c r="A24" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="B24" s="69">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15" customHeight="1">
+      <c r="A25" s="69" t="s">
+        <v>207</v>
+      </c>
+      <c r="B25" s="69">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15" customHeight="1">
+      <c r="A26" s="69" t="s">
+        <v>208</v>
+      </c>
+      <c r="B26" s="69">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15" customHeight="1">
+      <c r="A27" s="69" t="s">
+        <v>209</v>
+      </c>
+      <c r="B27" s="69">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15" customHeight="1">
+      <c r="A28" s="69" t="s">
+        <v>210</v>
+      </c>
+      <c r="B28" s="69">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15" customHeight="1">
+      <c r="A29" s="69" t="s">
+        <v>211</v>
+      </c>
+      <c r="B29" s="69">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15" customHeight="1">
+      <c r="A30" s="69" t="s">
+        <v>212</v>
+      </c>
+      <c r="B30" s="69">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15" customHeight="1">
+      <c r="A31" s="69" t="s">
+        <v>213</v>
+      </c>
+      <c r="B31" s="69">
+        <v>1089</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B218CA06-0190-4514-A3A9-83514D58FA31}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultColWidth="15.5" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="16384" width="15.5" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="174" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="175" t="s">
+        <v>141</v>
+      </c>
+      <c r="B2" s="42">
+        <v>1187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="175" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="42">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="175" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="42">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="175" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" s="42">
+        <v>1942</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="175" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="42">
+        <v>2282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="175" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7" s="42">
+        <v>1951</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="175" t="s">
+        <v>147</v>
+      </c>
+      <c r="B8" s="42">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="175" t="s">
+        <v>148</v>
+      </c>
+      <c r="B9" s="42">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="175" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" s="42">
+        <v>1283</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="175" t="s">
+        <v>150</v>
+      </c>
+      <c r="B11" s="42">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="175" t="s">
+        <v>151</v>
+      </c>
+      <c r="B12" s="42">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="175" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="42">
+        <v>2411</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="175" t="s">
+        <v>153</v>
+      </c>
+      <c r="B14" s="42">
+        <v>1626</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21AD5EE-7805-4208-8AB4-F7EFD579406E}">
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="12.375" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.375" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="174" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="175" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="42">
+        <v>2390</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="175" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="42">
+        <v>2533</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="175" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" s="42">
+        <v>2713</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="175" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5" s="42">
+        <v>4926</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="175" t="s">
+        <v>158</v>
+      </c>
+      <c r="B6" s="42">
+        <v>5284</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="175" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="42">
+        <v>4669</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="175" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8" s="42">
+        <v>3066</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="175" t="s">
+        <v>161</v>
+      </c>
+      <c r="B9" s="42">
+        <v>3895</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="175" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" s="42">
+        <v>3444</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="175" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="42">
+        <v>3415</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="175" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12" s="42">
+        <v>3656</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="175" t="s">
+        <v>165</v>
+      </c>
+      <c r="B13" s="42">
+        <v>4520</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="175" t="s">
+        <v>166</v>
+      </c>
+      <c r="B14" s="42">
+        <v>5447</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="175" t="s">
+        <v>167</v>
+      </c>
+      <c r="B15" s="42">
+        <v>4293</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="175" t="s">
+        <v>168</v>
+      </c>
+      <c r="B16" s="42">
+        <v>2885</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="175" t="s">
+        <v>169</v>
+      </c>
+      <c r="B17" s="42">
+        <v>2950</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="175" t="s">
+        <v>170</v>
+      </c>
+      <c r="B18" s="42">
+        <v>2832</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="175" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19" s="42">
+        <v>2924</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="175" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="42">
+        <v>5129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="175" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="42">
+        <v>5532</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="175" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="42">
+        <v>4002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="175" t="s">
+        <v>175</v>
+      </c>
+      <c r="B23" s="42">
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="175" t="s">
+        <v>176</v>
+      </c>
+      <c r="B24" s="42">
+        <v>3944</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="175" t="s">
+        <v>177</v>
+      </c>
+      <c r="B25" s="42">
+        <v>3894</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="175" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="42">
+        <v>4445</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="175" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="42">
+        <v>5119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="175" t="s">
+        <v>180</v>
+      </c>
+      <c r="B28" s="42">
+        <v>4734</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="175" t="s">
+        <v>181</v>
+      </c>
+      <c r="B29" s="42">
+        <v>4750</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="175" t="s">
+        <v>182</v>
+      </c>
+      <c r="B30" s="42">
+        <v>6646</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="175" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" s="42">
+        <v>6299</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-23 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5387,8 +5387,12 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n"/>
-      <c r="B24" s="13" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>2038</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14099,8 +14103,12 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n"/>
-      <c r="B24" s="13" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>45770</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>230</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -18649,7 +18657,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>1968</v>
+        <v>1970</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18682,7 +18690,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>2113</v>
+        <v>2125</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18709,8 +18717,14 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="n"/>
-      <c r="B23" s="15" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>1852</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -33968,8 +33982,14 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="n"/>
-      <c r="B23" s="15" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>3944</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>

</xml_diff>

<commit_message>
Manually roll dashboard data back to 2026-04-22 for silent update verification
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5387,12 +5387,8 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>46135</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>2038</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14103,12 +14099,8 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>45770</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>230</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -18717,14 +18709,8 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>1852</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -33982,14 +33968,8 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>3944</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-24 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -22,9 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -5391,7 +5392,7 @@
         <v>46135</v>
       </c>
       <c r="B24" s="21" t="n">
-        <v>2038</v>
+        <v>2037</v>
       </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
@@ -5404,8 +5405,12 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="13" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>2116</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14116,8 +14121,12 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="13" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>45771</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>251</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -18690,7 +18699,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>2125</v>
+        <v>2128</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18723,7 +18732,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>1852</v>
+        <v>1862</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18750,8 +18759,14 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="n"/>
-      <c r="B24" s="15" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>2035</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34011,8 +34026,14 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="n"/>
-      <c r="B24" s="15" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>3894</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-25 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5324,7 +5324,7 @@
         <v>46131</v>
       </c>
       <c r="B20" s="21" t="n">
-        <v>3587</v>
+        <v>3586</v>
       </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
@@ -5422,8 +5422,12 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n"/>
-      <c r="B26" s="13" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>3286</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14134,8 +14138,12 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n"/>
-      <c r="B26" s="13" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>45772</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>207</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -18732,7 +18740,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>1862</v>
+        <v>1865</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18765,7 +18773,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>2035</v>
+        <v>2042</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18792,8 +18800,14 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="n"/>
-      <c r="B25" s="15" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>2476</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34055,8 +34069,14 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="n"/>
-      <c r="B25" s="15" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>4445</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-26 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5188,7 +5188,7 @@
         <v>46123</v>
       </c>
       <c r="B12" s="21" t="n">
-        <v>4192</v>
+        <v>4193</v>
       </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
@@ -5307,7 +5307,7 @@
         <v>46130</v>
       </c>
       <c r="B19" s="21" t="n">
-        <v>3747</v>
+        <v>3746</v>
       </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
@@ -5439,8 +5439,12 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="13" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>3328</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14151,8 +14155,12 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="13" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>45773</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>446</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -18773,7 +18781,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>2042</v>
+        <v>2047</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18806,7 +18814,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>2476</v>
+        <v>2491</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18833,8 +18841,14 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="n"/>
-      <c r="B26" s="15" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>2677</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34098,8 +34112,14 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="n"/>
-      <c r="B26" s="15" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>5119</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-27 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5456,8 +5456,12 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="13" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>1915</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14168,8 +14172,12 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="13" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>45774</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>425</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -18814,7 +18822,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18847,7 +18855,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>2677</v>
+        <v>2702</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18874,8 +18882,14 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="n"/>
-      <c r="B27" s="15" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>2286</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34141,8 +34155,14 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="n"/>
-      <c r="B27" s="15" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>4734</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-28 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5473,8 +5473,12 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="13" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>1832</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14185,8 +14189,12 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
-      <c r="B29" s="13" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>45775</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>961</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -18855,7 +18863,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>2702</v>
+        <v>2715</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18888,7 +18896,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>2286</v>
+        <v>2296</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18915,8 +18923,14 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="n"/>
-      <c r="B28" s="15" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>3052</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34184,8 +34198,14 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="n"/>
-      <c r="B28" s="15" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>4750</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>

</xml_diff>

<commit_message>
Update dashboard data 2026-04-29
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5239,7 +5239,7 @@
         <v>46126</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>2201</v>
+        <v>2200</v>
       </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
@@ -5341,7 +5341,7 @@
         <v>46132</v>
       </c>
       <c r="B21" s="21" t="n">
-        <v>1991</v>
+        <v>1992</v>
       </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
@@ -5490,8 +5490,12 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n"/>
-      <c r="B30" s="13" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>1930</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14202,8 +14206,12 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n"/>
-      <c r="B30" s="13" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>45776</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>983</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -18896,7 +18904,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>2296</v>
+        <v>2302</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18929,7 +18937,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>3052</v>
+        <v>3067</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18956,8 +18964,14 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="n"/>
-      <c r="B29" s="15" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>3376</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34227,8 +34241,14 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="n"/>
-      <c r="B29" s="15" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>6646</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-04-30 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5507,8 +5507,12 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
-      <c r="B31" s="13" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1945</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -14219,8 +14223,12 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
-      <c r="B31" s="13" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>45777</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1089</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -18937,7 +18945,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>3067</v>
+        <v>3077</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18970,7 +18978,7 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>3376</v>
+        <v>3410</v>
       </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
@@ -18997,8 +19005,14 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="n"/>
-      <c r="B30" s="15" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2026年4月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>6343</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -34270,8 +34284,14 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="n"/>
-      <c r="B30" s="15" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2025年4月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>6299</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-01 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -22,10 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -5018,10 +5017,10 @@
     </row>
     <row r="2">
       <c r="A2" s="23" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>1286</v>
+        <v>2431</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
@@ -5031,12 +5030,8 @@
       <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46114</v>
-      </c>
-      <c r="B3" s="21" t="n">
-        <v>1524</v>
-      </c>
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="21" t="n"/>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -5048,12 +5043,8 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>46115</v>
-      </c>
-      <c r="B4" s="21" t="n">
-        <v>1630</v>
-      </c>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -5065,12 +5056,8 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>46116</v>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>3001</v>
-      </c>
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -5082,12 +5069,8 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>46117</v>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>2826</v>
-      </c>
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="21" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -5099,12 +5082,8 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>46118</v>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>2731</v>
-      </c>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -5116,12 +5095,8 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>46119</v>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>1827</v>
-      </c>
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="21" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -5133,12 +5108,8 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>46120</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>1933</v>
-      </c>
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -5150,12 +5121,8 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>46121</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>2460</v>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -5167,12 +5134,8 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>46122</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>2487</v>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -5184,12 +5147,8 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>46123</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>4193</v>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -5201,12 +5160,8 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>46124</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>4201</v>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -5218,12 +5173,8 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>46125</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>2157</v>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -5235,12 +5186,8 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>46126</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>2200</v>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -5252,12 +5199,8 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>46127</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <v>2383</v>
-      </c>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="21" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -5269,12 +5212,8 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>46128</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <v>2327</v>
-      </c>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -5286,12 +5225,8 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>46129</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>2451</v>
-      </c>
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="21" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -5303,12 +5238,8 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <v>3746</v>
-      </c>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -5320,12 +5251,8 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>46131</v>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>3586</v>
-      </c>
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="21" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -5337,12 +5264,8 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>46132</v>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>1992</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -5354,12 +5277,8 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>2017</v>
-      </c>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="21" t="n"/>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -5371,12 +5290,8 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>46134</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <v>1986</v>
-      </c>
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -5388,12 +5303,8 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>46135</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>2037</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -5405,12 +5316,8 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
-        <v>46136</v>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>2116</v>
-      </c>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -5422,12 +5329,8 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>3286</v>
-      </c>
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="21" t="n"/>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -5439,12 +5342,8 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n">
-        <v>46138</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>3328</v>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -5456,12 +5355,8 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
-        <v>46139</v>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>1915</v>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="21" t="n"/>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -5473,12 +5368,8 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
-        <v>46140</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>1832</v>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -5490,12 +5381,8 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
-        <v>46141</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>1930</v>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="21" t="n"/>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -5507,12 +5394,8 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
-        <v>46142</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>1945</v>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -13850,21 +13733,17 @@
     </row>
     <row r="2">
       <c r="A2" s="23" t="n">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>82</v>
+        <v>2798</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>45749</v>
-      </c>
-      <c r="B3" s="21" t="n">
-        <v>108</v>
-      </c>
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="21" t="n"/>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -13872,12 +13751,8 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>45750</v>
-      </c>
-      <c r="B4" s="21" t="n">
-        <v>54</v>
-      </c>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -13885,12 +13760,8 @@
       <c r="G4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>45751</v>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>69</v>
-      </c>
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -13898,12 +13769,8 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>45752</v>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>60</v>
-      </c>
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="21" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -13911,12 +13778,8 @@
       <c r="G6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>45753</v>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>62</v>
-      </c>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -13924,12 +13787,8 @@
       <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>45754</v>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>58</v>
-      </c>
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="21" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -13937,12 +13796,8 @@
       <c r="G8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>45755</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>36</v>
-      </c>
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -13950,12 +13805,8 @@
       <c r="G9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>45756</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>40</v>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -13963,12 +13814,8 @@
       <c r="G10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>45757</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>49</v>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -13976,12 +13823,8 @@
       <c r="G11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>45758</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>77</v>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -13989,12 +13832,8 @@
       <c r="G12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>45759</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>98</v>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -14002,12 +13841,8 @@
       <c r="G13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>45760</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>122</v>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -14015,12 +13850,8 @@
       <c r="G14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>45761</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>41</v>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -14028,12 +13859,8 @@
       <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>45762</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <v>132</v>
-      </c>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="21" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -14041,12 +13868,8 @@
       <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>45763</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <v>127</v>
-      </c>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -14054,12 +13877,8 @@
       <c r="G17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>45764</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>250</v>
-      </c>
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="21" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -14067,12 +13886,8 @@
       <c r="G18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>45765</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <v>275</v>
-      </c>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -14080,12 +13895,8 @@
       <c r="G19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>45766</v>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>448</v>
-      </c>
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="21" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -14093,12 +13904,8 @@
       <c r="G20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>45767</v>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>406</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -14106,12 +13913,8 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>45768</v>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>263</v>
-      </c>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="21" t="n"/>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -14119,12 +13922,8 @@
       <c r="G22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>45769</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <v>223</v>
-      </c>
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -14132,12 +13931,8 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>45770</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>230</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14145,12 +13940,8 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
-        <v>45771</v>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>251</v>
-      </c>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14158,12 +13949,8 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
-        <v>45772</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>207</v>
-      </c>
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="21" t="n"/>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14171,12 +13958,8 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n">
-        <v>45773</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>446</v>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14184,12 +13967,8 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
-        <v>45774</v>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>425</v>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="21" t="n"/>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14197,12 +13976,8 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
-        <v>45775</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>961</v>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14210,12 +13985,8 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
-        <v>45776</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>983</v>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="21" t="n"/>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14223,12 +13994,8 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
-        <v>45777</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>1089</v>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -18050,11 +17817,11 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>2026年4月1日</t>
+          <t>2026年5月1日</t>
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>1187</v>
+        <v>3323</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -18081,14 +17848,8 @@
       <c r="Y1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月2日</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>1006</v>
-      </c>
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="20" t="n"/>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -18114,14 +17875,8 @@
       <c r="Y2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月3日</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>1059</v>
-      </c>
+      <c r="A3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -18147,14 +17902,8 @@
       <c r="Y3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月4日</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>1942</v>
-      </c>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -18180,14 +17929,8 @@
       <c r="Y4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月5日</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>2282</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="20" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -18213,14 +17956,8 @@
       <c r="Y5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月6日</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>1951</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -18246,14 +17983,8 @@
       <c r="Y6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月7日</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>1345</v>
-      </c>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -18279,14 +18010,8 @@
       <c r="Y7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月8日</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>1241</v>
-      </c>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -18312,14 +18037,8 @@
       <c r="Y8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月9日</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>1283</v>
-      </c>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -18345,14 +18064,8 @@
       <c r="Y9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月10日</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n">
-        <v>1381</v>
-      </c>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -18378,14 +18091,8 @@
       <c r="Y10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月11日</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>2100</v>
-      </c>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -18411,14 +18118,8 @@
       <c r="Y11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月12日</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>2418</v>
-      </c>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -18444,14 +18145,8 @@
       <c r="Y12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月13日</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>1644</v>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -18477,14 +18172,8 @@
       <c r="Y13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月14日</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>1398</v>
-      </c>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -18510,14 +18199,8 @@
       <c r="Y14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月15日</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>1400</v>
-      </c>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -18543,14 +18226,8 @@
       <c r="Y15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月16日</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>1397</v>
-      </c>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -18576,14 +18253,8 @@
       <c r="Y16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月17日</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>1549</v>
-      </c>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -18609,14 +18280,8 @@
       <c r="Y17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月18日</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="n">
-        <v>2796</v>
-      </c>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="20" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -18642,14 +18307,8 @@
       <c r="Y18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月19日</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>2851</v>
-      </c>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -18675,14 +18334,8 @@
       <c r="Y19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月20日</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="n">
-        <v>2133</v>
-      </c>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="20" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -18708,14 +18361,8 @@
       <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月21日</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>1970</v>
-      </c>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -18741,14 +18388,8 @@
       <c r="Y21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月22日</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>2128</v>
-      </c>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="20" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -18774,14 +18415,8 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>1865</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -18807,14 +18442,8 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月24日</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>2047</v>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="20" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -18840,14 +18469,8 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月25日</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>2494</v>
-      </c>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="20" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -18873,14 +18496,8 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月26日</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
-        <v>2715</v>
-      </c>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="20" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -18906,14 +18523,8 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月27日</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>2302</v>
-      </c>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="20" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -18939,14 +18550,8 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月28日</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>3077</v>
-      </c>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="20" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -18972,14 +18577,8 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月29日</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>3410</v>
-      </c>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="20" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -19005,14 +18604,8 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>2026年4月30日</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>6343</v>
-      </c>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -33445,11 +33038,11 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>2025年4月1日</t>
+          <t>2025年5月1日</t>
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>2390</v>
+        <v>6619</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -33472,14 +33065,8 @@
       <c r="U1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月2日</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>2533</v>
-      </c>
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="20" t="n"/>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -33501,14 +33088,8 @@
       <c r="U2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月3日</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>2713</v>
-      </c>
+      <c r="A3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -33530,14 +33111,8 @@
       <c r="U3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月4日</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>4926</v>
-      </c>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -33559,14 +33134,8 @@
       <c r="U4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月5日</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>5284</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="20" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -33588,14 +33157,8 @@
       <c r="U5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月6日</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>4669</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -33617,14 +33180,8 @@
       <c r="U6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月7日</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>3066</v>
-      </c>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -33646,14 +33203,8 @@
       <c r="U7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月8日</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>3895</v>
-      </c>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -33675,14 +33226,8 @@
       <c r="U8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月9日</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>3444</v>
-      </c>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -33704,14 +33249,8 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月10日</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n">
-        <v>3415</v>
-      </c>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -33733,14 +33272,8 @@
       <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月11日</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>3656</v>
-      </c>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -33762,14 +33295,8 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月12日</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>4520</v>
-      </c>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -33791,14 +33318,8 @@
       <c r="U12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月13日</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>5447</v>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -33820,14 +33341,8 @@
       <c r="U13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月14日</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>4293</v>
-      </c>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -33849,14 +33364,8 @@
       <c r="U14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月15日</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>2885</v>
-      </c>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -33878,14 +33387,8 @@
       <c r="U15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月16日</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>2950</v>
-      </c>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -33907,14 +33410,8 @@
       <c r="U16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月17日</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>2832</v>
-      </c>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -33936,14 +33433,8 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月18日</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="n">
-        <v>2924</v>
-      </c>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="20" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -33965,14 +33456,8 @@
       <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月19日</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>5129</v>
-      </c>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -33994,14 +33479,8 @@
       <c r="U19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月20日</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="n">
-        <v>5532</v>
-      </c>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="20" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -34023,14 +33502,8 @@
       <c r="U20" s="18" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月21日</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>4002</v>
-      </c>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -34052,14 +33525,8 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月22日</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>3480</v>
-      </c>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="20" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -34081,14 +33548,8 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>3944</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -34110,14 +33571,8 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月24日</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>3894</v>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="20" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34139,14 +33594,8 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月25日</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>4445</v>
-      </c>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="20" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34168,14 +33617,8 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月26日</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
-        <v>5119</v>
-      </c>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="20" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34197,14 +33640,8 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月27日</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>4734</v>
-      </c>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="20" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34226,14 +33663,8 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月28日</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>4750</v>
-      </c>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="20" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34255,14 +33686,8 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月29日</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>6646</v>
-      </c>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="20" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34284,14 +33709,8 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>2025年4月30日</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>6299</v>
-      </c>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-02 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -22,9 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -219,7 +220,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -278,6 +279,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -5020,7 +5024,7 @@
         <v>46143</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>2431</v>
+        <v>2429</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
@@ -5030,8 +5034,12 @@
       <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n"/>
-      <c r="B3" s="21" t="n"/>
+      <c r="A3" s="23" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B3" s="21" t="n">
+        <v>2386</v>
+      </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -13742,8 +13750,12 @@
       <c r="G2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n"/>
-      <c r="B3" s="21" t="n"/>
+      <c r="A3" s="23" t="n">
+        <v>45779</v>
+      </c>
+      <c r="B3" s="21" t="n">
+        <v>2695</v>
+      </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -17820,8 +17832,8 @@
           <t>2026年5月1日</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n">
-        <v>3323</v>
+      <c r="B1" s="24" t="n">
+        <v>3352</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17848,8 +17860,14 @@
       <c r="Y1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月2日</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="n">
+        <v>3655</v>
+      </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -33041,7 +33059,7 @@
           <t>2025年5月1日</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n">
+      <c r="B1" s="24" t="n">
         <v>6619</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33065,8 +33083,14 @@
       <c r="U1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月2日</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="n">
+        <v>6313</v>
+      </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-03 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5051,8 +5051,12 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
-      <c r="B4" s="21" t="n"/>
+      <c r="A4" s="23" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>2436</v>
+      </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -13763,8 +13767,12 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
-      <c r="B4" s="21" t="n"/>
+      <c r="A4" s="23" t="n">
+        <v>45780</v>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>2701</v>
+      </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -17833,7 +17841,7 @@
         </is>
       </c>
       <c r="B1" s="24" t="n">
-        <v>3352</v>
+        <v>3371</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17866,7 +17874,7 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>3655</v>
+        <v>3694</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17893,8 +17901,14 @@
       <c r="Y2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月3日</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n">
+        <v>3323</v>
+      </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -33059,7 +33073,7 @@
           <t>2025年5月1日</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n">
+      <c r="B1" s="20" t="n">
         <v>6619</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33088,7 +33102,7 @@
           <t>2025年5月2日</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="20" t="n">
         <v>6313</v>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -33112,8 +33126,14 @@
       <c r="U2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月3日</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="n">
+        <v>5619</v>
+      </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-04 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5055,7 +5055,7 @@
         <v>46145</v>
       </c>
       <c r="B4" s="21" t="n">
-        <v>2436</v>
+        <v>2435</v>
       </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
@@ -5068,8 +5068,12 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="21" t="n"/>
+      <c r="A5" s="23" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>2281</v>
+      </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -13780,8 +13784,12 @@
       <c r="G4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="21" t="n"/>
+      <c r="A5" s="23" t="n">
+        <v>45781</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>2597</v>
+      </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -17874,7 +17882,7 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>3694</v>
+        <v>3699</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17907,7 +17915,7 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>3323</v>
+        <v>3343</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17934,8 +17942,14 @@
       <c r="Y3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月4日</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>3406</v>
+      </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -33155,8 +33169,14 @@
       <c r="U3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月4日</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="n">
+        <v>5576</v>
+      </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-05 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5085,8 +5085,12 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="21" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>2104</v>
+      </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -13797,8 +13801,12 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="21" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>45782</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>2520</v>
+      </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -17915,7 +17923,7 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>3343</v>
+        <v>3351</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17948,7 +17956,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>3406</v>
+        <v>3422</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -17975,8 +17983,14 @@
       <c r="Y4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月5日</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>4312</v>
+      </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -33198,8 +33212,14 @@
       <c r="U4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月5日</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>5963</v>
+      </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-06 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5072,7 +5072,7 @@
         <v>46146</v>
       </c>
       <c r="B5" s="21" t="n">
-        <v>2281</v>
+        <v>2280</v>
       </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
@@ -5102,8 +5102,12 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="21" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>1298</v>
+      </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -13814,8 +13818,12 @@
       <c r="G6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="21" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>45783</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>1435</v>
+      </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -17856,8 +17864,8 @@
           <t>2026年5月1日</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n">
-        <v>3371</v>
+      <c r="B1" s="20" t="n">
+        <v>3369</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17889,8 +17897,8 @@
           <t>2026年5月2日</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
-        <v>3699</v>
+      <c r="B2" s="20" t="n">
+        <v>3695</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17922,8 +17930,8 @@
           <t>2026年5月3日</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
-        <v>3351</v>
+      <c r="B3" s="20" t="n">
+        <v>3350</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17955,8 +17963,8 @@
           <t>2026年5月4日</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
-        <v>3422</v>
+      <c r="B4" s="20" t="n">
+        <v>3428</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -17988,8 +17996,8 @@
           <t>2026年5月5日</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
-        <v>4312</v>
+      <c r="B5" s="20" t="n">
+        <v>4328</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18016,8 +18024,14 @@
       <c r="Y5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月6日</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>2941</v>
+      </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -33241,8 +33255,14 @@
       <c r="U5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月6日</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>5196</v>
+      </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-07 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5106,7 +5106,7 @@
         <v>46148</v>
       </c>
       <c r="B7" s="21" t="n">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
@@ -5119,8 +5119,12 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="21" t="n"/>
+      <c r="A8" s="23" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>1466</v>
+      </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -13831,8 +13835,12 @@
       <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="21" t="n"/>
+      <c r="A8" s="23" t="n">
+        <v>45784</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>1540</v>
+      </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -17997,7 +18005,7 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>4328</v>
+        <v>4335</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18030,7 +18038,7 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>2941</v>
+        <v>2953</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18057,8 +18065,14 @@
       <c r="Y6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月7日</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>2893</v>
+      </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -33284,8 +33298,14 @@
       <c r="U6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月7日</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>6078</v>
+      </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-08 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5106,7 +5106,7 @@
         <v>46148</v>
       </c>
       <c r="B7" s="21" t="n">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
@@ -5136,8 +5136,12 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="21" t="n"/>
+      <c r="A9" s="23" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>1492</v>
+      </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -13848,8 +13852,12 @@
       <c r="G8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="21" t="n"/>
+      <c r="A9" s="23" t="n">
+        <v>45785</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>1538</v>
+      </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -18038,7 +18046,7 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>2953</v>
+        <v>2954</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18071,7 +18079,7 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>2893</v>
+        <v>2904</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -18098,8 +18106,14 @@
       <c r="Y7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月8日</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>1214</v>
+      </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -33327,8 +33341,14 @@
       <c r="U7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月8日</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>2247</v>
+      </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-09 (manual-web)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5153,8 +5153,12 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>1826</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -13865,8 +13869,12 @@
       <c r="G9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>45786</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>1766</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -18079,7 +18087,7 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>2904</v>
+        <v>2909</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -18112,7 +18120,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>1214</v>
+        <v>1229</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18139,8 +18147,14 @@
       <c r="Y8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月9日</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>1222</v>
+      </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -33370,8 +33384,14 @@
       <c r="U8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月9日</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>2354</v>
+      </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-10 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5170,8 +5170,12 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>2701</v>
+      </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -13882,8 +13886,12 @@
       <c r="G10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>45787</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>3124</v>
+      </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -18120,7 +18128,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>1229</v>
+        <v>1236</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18153,7 +18161,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>1222</v>
+        <v>1236</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18180,8 +18188,14 @@
       <c r="Y9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月10日</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>1809</v>
+      </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -33413,8 +33427,14 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月10日</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>3606</v>
+      </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-11 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5187,8 +5187,12 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="21" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>1558</v>
+      </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -13899,8 +13903,12 @@
       <c r="G11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="21" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>45788</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>3042</v>
+      </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -18161,7 +18169,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>1236</v>
+        <v>1239</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18194,7 +18202,7 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>1809</v>
+        <v>1828</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -18221,8 +18229,14 @@
       <c r="Y10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月11日</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>1499</v>
+      </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -33456,8 +33470,14 @@
       <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月11日</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>4047</v>
+      </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-12 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5204,8 +5204,12 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>1607</v>
+      </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -13916,8 +13920,12 @@
       <c r="G12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>45789</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>1571</v>
+      </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -18202,7 +18210,7 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>1828</v>
+        <v>1829</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -18235,7 +18243,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1499</v>
+        <v>1505</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18262,8 +18270,14 @@
       <c r="Y11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月12日</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>1212</v>
+      </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -33499,8 +33513,14 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月12日</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>2740</v>
+      </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-13 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5055,7 +5055,7 @@
         <v>46145</v>
       </c>
       <c r="B4" s="21" t="n">
-        <v>2435</v>
+        <v>2434</v>
       </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
@@ -5208,7 +5208,7 @@
         <v>46154</v>
       </c>
       <c r="B13" s="21" t="n">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
@@ -5221,8 +5221,12 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>1705</v>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -13933,8 +13937,12 @@
       <c r="G13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>45790</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>1518</v>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -18243,7 +18251,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1505</v>
+        <v>1513</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18276,7 +18284,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1212</v>
+        <v>1215</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18303,8 +18311,14 @@
       <c r="Y12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月13日</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>1052</v>
+      </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -33542,8 +33556,14 @@
       <c r="U12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月13日</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>2405</v>
+      </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-14 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5238,8 +5238,12 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
+      <c r="A15" s="23" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1707</v>
+      </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -13950,8 +13954,12 @@
       <c r="G14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
+      <c r="A15" s="23" t="n">
+        <v>45791</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1544</v>
+      </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -18284,7 +18292,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18317,7 +18325,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -18344,8 +18352,14 @@
       <c r="Y13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月14日</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>990</v>
+      </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -33585,8 +33599,14 @@
       <c r="U13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月14日</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>2575</v>
+      </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-15 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5255,8 +5255,12 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="21" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1793</v>
+      </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -13967,8 +13971,12 @@
       <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="21" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>45792</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1507</v>
+      </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -18325,7 +18333,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1058</v>
+        <v>1060</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -18358,7 +18366,7 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>990</v>
+        <v>997</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18385,8 +18393,14 @@
       <c r="Y14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月15日</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>1052</v>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -33628,8 +33642,14 @@
       <c r="U14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月15日</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>2513</v>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-16 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5272,8 +5272,12 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="21" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>2854</v>
+      </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -13984,8 +13988,12 @@
       <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="21" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>45793</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>1531</v>
+      </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -18366,7 +18374,7 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>997</v>
+        <v>1000</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18399,7 +18407,7 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>1052</v>
+        <v>1060</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18426,8 +18434,14 @@
       <c r="Y15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月16日</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>1687</v>
+      </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -33671,8 +33685,14 @@
       <c r="U15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月16日</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>2771</v>
+      </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-17 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5055,7 +5055,7 @@
         <v>46145</v>
       </c>
       <c r="B4" s="21" t="n">
-        <v>2434</v>
+        <v>2433</v>
       </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
@@ -5259,7 +5259,7 @@
         <v>46157</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1793</v>
+        <v>1792</v>
       </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
@@ -5289,8 +5289,12 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="21" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>46159</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>2773</v>
+      </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -14001,8 +14005,12 @@
       <c r="G17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="21" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>45794</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>2884</v>
+      </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -18407,7 +18415,7 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18440,7 +18448,7 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1687</v>
+        <v>1699</v>
       </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -18467,8 +18475,14 @@
       <c r="Y16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月17日</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>2041</v>
+      </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -33714,8 +33728,14 @@
       <c r="U16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月17日</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>4030</v>
+      </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-18 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5174,7 +5174,7 @@
         <v>46152</v>
       </c>
       <c r="B11" s="21" t="n">
-        <v>2701</v>
+        <v>2700</v>
       </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
@@ -5293,7 +5293,7 @@
         <v>46159</v>
       </c>
       <c r="B18" s="21" t="n">
-        <v>2773</v>
+        <v>2771</v>
       </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
@@ -5306,8 +5306,12 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="21" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>1567</v>
+      </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -14018,8 +14022,12 @@
       <c r="G18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="21" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>45795</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>2879</v>
+      </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -18448,7 +18456,7 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1699</v>
+        <v>1705</v>
       </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -18481,7 +18489,7 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>2041</v>
+        <v>2062</v>
       </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -18508,8 +18516,14 @@
       <c r="Y17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月18日</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>1320</v>
+      </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -33757,8 +33771,14 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月18日</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>4424</v>
+      </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-19 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5310,7 +5310,7 @@
         <v>46160</v>
       </c>
       <c r="B19" s="21" t="n">
-        <v>1567</v>
+        <v>1566</v>
       </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
@@ -5323,8 +5323,12 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="21" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>1721</v>
+      </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -14035,8 +14039,12 @@
       <c r="G19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="21" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>45796</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>1506</v>
+      </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -18489,7 +18497,7 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>2062</v>
+        <v>2083</v>
       </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -18522,7 +18530,7 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1320</v>
+        <v>1339</v>
       </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
@@ -18549,8 +18557,14 @@
       <c r="Y18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月19日</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>1247</v>
+      </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -33800,8 +33814,14 @@
       <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月19日</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>3066</v>
+      </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-20 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5340,8 +5340,12 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="21" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>1762</v>
+      </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -14052,8 +14056,12 @@
       <c r="G20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="21" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>45797</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>1427</v>
+      </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -18563,7 +18571,7 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>1247</v>
+        <v>1249</v>
       </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
@@ -18590,8 +18598,14 @@
       <c r="Y19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月20日</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>1097</v>
+      </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -33843,8 +33857,14 @@
       <c r="U19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月20日</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>2845</v>
+      </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-21 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5344,7 +5344,7 @@
         <v>46162</v>
       </c>
       <c r="B21" s="21" t="n">
-        <v>1762</v>
+        <v>1760</v>
       </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
@@ -5357,8 +5357,12 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="21" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>1816</v>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -14069,8 +14073,12 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="21" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>45798</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>1426</v>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -18571,7 +18579,7 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>1249</v>
+        <v>1261</v>
       </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
@@ -18604,7 +18612,7 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>1097</v>
+        <v>1105</v>
       </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
@@ -18631,8 +18639,14 @@
       <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月21日</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>1171</v>
+      </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -33886,8 +33900,14 @@
       <c r="U20" s="18" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月21日</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>3188</v>
+      </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-22 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5374,8 +5374,12 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="21" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>1482</v>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -14086,8 +14090,12 @@
       <c r="G22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="21" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>45799</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>1405</v>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -18645,7 +18653,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18672,8 +18680,14 @@
       <c r="Y21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月22日</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>999</v>
+      </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -33929,8 +33943,14 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月22日</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>3080</v>
+      </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-23 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5391,8 +5391,12 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="21" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>2903</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14103,8 +14107,12 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="21" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>45800</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>1557</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -18653,7 +18661,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>1174</v>
+        <v>1183</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18686,7 +18694,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>999</v>
+        <v>1010</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18713,8 +18721,14 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>1765</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -33972,8 +33986,14 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>3506</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-24 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5276,7 +5276,7 @@
         <v>46158</v>
       </c>
       <c r="B17" s="21" t="n">
-        <v>2854</v>
+        <v>2853</v>
       </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
@@ -5408,8 +5408,12 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="21" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>2808</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14120,8 +14124,12 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="21" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>45801</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>2841</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -18694,7 +18702,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18727,7 +18735,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>1765</v>
+        <v>1773</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18754,8 +18762,14 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>1922</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34015,8 +34029,14 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>4639</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-25 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5425,8 +5425,12 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="21" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>1650</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14137,8 +14141,12 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="21" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>45802</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>2888</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -18735,7 +18743,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>1773</v>
+        <v>1778</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18768,7 +18776,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1922</v>
+        <v>1941</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18795,8 +18803,14 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>1470</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34058,8 +34072,14 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>4546</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-26 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5276,7 +5276,7 @@
         <v>46158</v>
       </c>
       <c r="B17" s="21" t="n">
-        <v>2853</v>
+        <v>2852</v>
       </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
@@ -5310,7 +5310,7 @@
         <v>46160</v>
       </c>
       <c r="B19" s="21" t="n">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
@@ -5344,7 +5344,7 @@
         <v>46162</v>
       </c>
       <c r="B21" s="21" t="n">
-        <v>1760</v>
+        <v>1759</v>
       </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
@@ -5442,8 +5442,12 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="21" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>46168</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>1769</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14154,8 +14158,12 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="21" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>45803</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>1501</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -18776,7 +18784,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1941</v>
+        <v>1944</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18809,7 +18817,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1470</v>
+        <v>1488</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18836,8 +18844,14 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>1351</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34101,8 +34115,14 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>4370</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-27 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5412,7 +5412,7 @@
         <v>46166</v>
       </c>
       <c r="B25" s="21" t="n">
-        <v>2808</v>
+        <v>2807</v>
       </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
@@ -5446,7 +5446,7 @@
         <v>46168</v>
       </c>
       <c r="B27" s="21" t="n">
-        <v>1769</v>
+        <v>1768</v>
       </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
@@ -5459,8 +5459,12 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="21" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>1825</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14171,8 +14175,12 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="21" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>45804</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>1476</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -18850,7 +18858,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1351</v>
+        <v>1362</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18877,8 +18885,14 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>1442</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34144,8 +34158,14 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>3834</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-28 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5476,8 +5476,12 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="21" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>1804</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14188,8 +14192,12 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="21" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>45805</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>1518</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -18858,7 +18866,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1362</v>
+        <v>1367</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18891,7 +18899,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>1442</v>
+        <v>1456</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18918,8 +18926,14 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>1650</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34187,8 +34201,14 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>3669</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-29 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5493,8 +5493,12 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="21" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>1744</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14205,8 +14209,12 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="21" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>45806</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>1529</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -18899,7 +18907,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>1456</v>
+        <v>1458</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18932,7 +18940,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>1650</v>
+        <v>1654</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18959,8 +18967,14 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>1711</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34230,8 +34244,14 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>3709</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-30 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5497,7 +5497,7 @@
         <v>46171</v>
       </c>
       <c r="B30" s="21" t="n">
-        <v>1744</v>
+        <v>1743</v>
       </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
@@ -5510,8 +5510,12 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="21" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>2642</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -14222,8 +14226,12 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="21" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>45807</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1527</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -18940,7 +18948,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>1654</v>
+        <v>1657</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18973,7 +18981,7 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>1711</v>
+        <v>1719</v>
       </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
@@ -19000,8 +19008,14 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>3528</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -34273,8 +34287,14 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>12066</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-05-31 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -5514,7 +5515,7 @@
         <v>46172</v>
       </c>
       <c r="B31" s="21" t="n">
-        <v>2642</v>
+        <v>2641</v>
       </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
@@ -5527,8 +5528,12 @@
       <c r="K31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n"/>
-      <c r="B32" s="13" t="n"/>
+      <c r="A32" s="23" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B32" s="21" t="n">
+        <v>2501</v>
+      </c>
       <c r="C32" s="13" t="n"/>
       <c r="D32" s="13" t="n"/>
       <c r="E32" s="13" t="n"/>
@@ -14239,8 +14244,12 @@
       <c r="G31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n"/>
-      <c r="B32" s="13" t="n"/>
+      <c r="A32" s="23" t="n">
+        <v>45808</v>
+      </c>
+      <c r="B32" s="21" t="n">
+        <v>2374</v>
+      </c>
       <c r="C32" s="13" t="n"/>
       <c r="D32" s="13" t="n"/>
       <c r="E32" s="13" t="n"/>
@@ -18981,7 +18990,7 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>1719</v>
+        <v>1725</v>
       </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
@@ -19014,7 +19023,7 @@
         </is>
       </c>
       <c r="B30" s="20" t="n">
-        <v>3528</v>
+        <v>3541</v>
       </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
@@ -19041,8 +19050,14 @@
       <c r="Y30" s="18" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="n"/>
-      <c r="B31" s="15" t="n"/>
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>2026年5月31日</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>3318</v>
+      </c>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="15" t="n"/>
       <c r="E31" s="17" t="n"/>
@@ -34316,8 +34331,14 @@
       <c r="U30" s="18" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="n"/>
-      <c r="B31" s="15" t="n"/>
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>2025年5月31日</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>9878</v>
+      </c>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="15" t="n"/>
       <c r="E31" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-01 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -22,11 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -5022,10 +5021,10 @@
     </row>
     <row r="2">
       <c r="A2" s="23" t="n">
-        <v>46143</v>
+        <v>46174</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>2429</v>
+        <v>1262</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
@@ -5035,12 +5034,8 @@
       <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46144</v>
-      </c>
-      <c r="B3" s="21" t="n">
-        <v>2386</v>
-      </c>
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="21" t="n"/>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -5052,12 +5047,8 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>46145</v>
-      </c>
-      <c r="B4" s="21" t="n">
-        <v>2433</v>
-      </c>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -5069,12 +5060,8 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>46146</v>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>2280</v>
-      </c>
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -5086,12 +5073,8 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>46147</v>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>2104</v>
-      </c>
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="21" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -5103,12 +5086,8 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>46148</v>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>1298</v>
-      </c>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -5120,12 +5099,8 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>46149</v>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>1466</v>
-      </c>
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="21" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -5137,12 +5112,8 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>46150</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>1492</v>
-      </c>
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -5154,12 +5125,8 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>46151</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>1826</v>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -5171,12 +5138,8 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>2700</v>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -5188,12 +5151,8 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>46153</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>1558</v>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -5205,12 +5164,8 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>46154</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>1606</v>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -5222,12 +5177,8 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>46155</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>1705</v>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -5239,12 +5190,8 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>46156</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>1707</v>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -5256,12 +5203,8 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>46157</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <v>1792</v>
-      </c>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="21" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -5273,12 +5216,8 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>46158</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <v>2852</v>
-      </c>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -5290,12 +5229,8 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>46159</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>2771</v>
-      </c>
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="21" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -5307,12 +5242,8 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>46160</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <v>1565</v>
-      </c>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -5324,12 +5255,8 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>46161</v>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>1721</v>
-      </c>
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="21" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -5341,12 +5268,8 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>46162</v>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>1759</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -5358,12 +5281,8 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>46163</v>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>1816</v>
-      </c>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="21" t="n"/>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -5375,12 +5294,8 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>46164</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <v>1482</v>
-      </c>
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -5392,12 +5307,8 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>46165</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>2903</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -5409,12 +5320,8 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
-        <v>46166</v>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>2807</v>
-      </c>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -5426,12 +5333,8 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
-        <v>46167</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>1650</v>
-      </c>
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="21" t="n"/>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -5443,12 +5346,8 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n">
-        <v>46168</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>1768</v>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -5460,12 +5359,8 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
-        <v>46169</v>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>1825</v>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="21" t="n"/>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -5477,12 +5372,8 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
-        <v>46170</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>1804</v>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -5494,12 +5385,8 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
-        <v>46171</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>1743</v>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="21" t="n"/>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -5511,12 +5398,8 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
-        <v>46172</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>2641</v>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -5528,12 +5411,8 @@
       <c r="K31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B32" s="21" t="n">
-        <v>2501</v>
-      </c>
+      <c r="A32" s="23" t="n"/>
+      <c r="B32" s="21" t="n"/>
       <c r="C32" s="13" t="n"/>
       <c r="D32" s="13" t="n"/>
       <c r="E32" s="13" t="n"/>
@@ -13858,21 +13737,17 @@
     </row>
     <row r="2">
       <c r="A2" s="23" t="n">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>2798</v>
+        <v>2129</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>45779</v>
-      </c>
-      <c r="B3" s="21" t="n">
-        <v>2695</v>
-      </c>
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="21" t="n"/>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -13880,12 +13755,8 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>45780</v>
-      </c>
-      <c r="B4" s="21" t="n">
-        <v>2701</v>
-      </c>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -13893,12 +13764,8 @@
       <c r="G4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>45781</v>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>2597</v>
-      </c>
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -13906,12 +13773,8 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>45782</v>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>2520</v>
-      </c>
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="21" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -13919,12 +13782,8 @@
       <c r="G6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>45783</v>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>1435</v>
-      </c>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -13932,12 +13791,8 @@
       <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>45784</v>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>1540</v>
-      </c>
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="21" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -13945,12 +13800,8 @@
       <c r="G8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>45785</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>1538</v>
-      </c>
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -13958,12 +13809,8 @@
       <c r="G9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>45786</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>1766</v>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -13971,12 +13818,8 @@
       <c r="G10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>45787</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>3124</v>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -13984,12 +13827,8 @@
       <c r="G11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>45788</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>3042</v>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -13997,12 +13836,8 @@
       <c r="G12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>45789</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>1571</v>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -14010,12 +13845,8 @@
       <c r="G13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>45790</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>1518</v>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -14023,12 +13854,8 @@
       <c r="G14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>45791</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>1544</v>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -14036,12 +13863,8 @@
       <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>45792</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <v>1507</v>
-      </c>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="21" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -14049,12 +13872,8 @@
       <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>45793</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <v>1531</v>
-      </c>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -14062,12 +13881,8 @@
       <c r="G17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>45794</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>2884</v>
-      </c>
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="21" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -14075,12 +13890,8 @@
       <c r="G18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>45795</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <v>2879</v>
-      </c>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -14088,12 +13899,8 @@
       <c r="G19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>45796</v>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>1506</v>
-      </c>
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="21" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -14101,12 +13908,8 @@
       <c r="G20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>45797</v>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>1427</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -14114,12 +13917,8 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>45798</v>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>1426</v>
-      </c>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="21" t="n"/>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -14127,12 +13926,8 @@
       <c r="G22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>45799</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <v>1405</v>
-      </c>
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -14140,12 +13935,8 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>45800</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>1557</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14153,12 +13944,8 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
-        <v>45801</v>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>2841</v>
-      </c>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14166,12 +13953,8 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
-        <v>45802</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>2888</v>
-      </c>
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="21" t="n"/>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14179,12 +13962,8 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n">
-        <v>45803</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>1501</v>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14192,12 +13971,8 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
-        <v>45804</v>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>1476</v>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="21" t="n"/>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14205,12 +13980,8 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
-        <v>45805</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>1518</v>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14218,12 +13989,8 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
-        <v>45806</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>1529</v>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="21" t="n"/>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14231,12 +13998,8 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
-        <v>45807</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>1527</v>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -14244,12 +14007,8 @@
       <c r="G31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="n">
-        <v>45808</v>
-      </c>
-      <c r="B32" s="21" t="n">
-        <v>2374</v>
-      </c>
+      <c r="A32" s="23" t="n"/>
+      <c r="B32" s="21" t="n"/>
       <c r="C32" s="13" t="n"/>
       <c r="D32" s="13" t="n"/>
       <c r="E32" s="13" t="n"/>
@@ -18062,11 +17821,11 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>2026年5月1日</t>
+          <t>2026年6月1日</t>
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>3369</v>
+        <v>1023</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -18093,14 +17852,8 @@
       <c r="Y1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月2日</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>3695</v>
-      </c>
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="20" t="n"/>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -18126,14 +17879,8 @@
       <c r="Y2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月3日</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>3350</v>
-      </c>
+      <c r="A3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -18159,14 +17906,8 @@
       <c r="Y3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月4日</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>3428</v>
-      </c>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -18192,14 +17933,8 @@
       <c r="Y4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月5日</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>4335</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="20" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -18225,14 +17960,8 @@
       <c r="Y5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月6日</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>2954</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -18258,14 +17987,8 @@
       <c r="Y6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月7日</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>2909</v>
-      </c>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -18291,14 +18014,8 @@
       <c r="Y7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月8日</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>1236</v>
-      </c>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -18324,14 +18041,8 @@
       <c r="Y8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月9日</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>1239</v>
-      </c>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -18357,14 +18068,8 @@
       <c r="Y9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月10日</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n">
-        <v>1829</v>
-      </c>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -18390,14 +18095,8 @@
       <c r="Y10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月11日</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>1513</v>
-      </c>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -18423,14 +18122,8 @@
       <c r="Y11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月12日</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>1218</v>
-      </c>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -18456,14 +18149,8 @@
       <c r="Y12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月13日</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>1060</v>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -18489,14 +18176,8 @@
       <c r="Y13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月14日</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>1000</v>
-      </c>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -18522,14 +18203,8 @@
       <c r="Y14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月15日</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>1066</v>
-      </c>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -18555,14 +18230,8 @@
       <c r="Y15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月16日</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>1705</v>
-      </c>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -18588,14 +18257,8 @@
       <c r="Y16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月17日</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>2083</v>
-      </c>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -18621,14 +18284,8 @@
       <c r="Y17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月18日</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="n">
-        <v>1339</v>
-      </c>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="20" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -18654,14 +18311,8 @@
       <c r="Y18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月19日</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>1261</v>
-      </c>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -18687,14 +18338,8 @@
       <c r="Y19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月20日</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="n">
-        <v>1105</v>
-      </c>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="20" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -18720,14 +18365,8 @@
       <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月21日</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>1183</v>
-      </c>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -18753,14 +18392,8 @@
       <c r="Y21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月22日</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>1011</v>
-      </c>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="20" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -18786,14 +18419,8 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>1778</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -18819,14 +18446,8 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月24日</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>1944</v>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="20" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -18852,14 +18473,8 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月25日</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>1488</v>
-      </c>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="20" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -18885,14 +18500,8 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月26日</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
-        <v>1367</v>
-      </c>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="20" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -18918,14 +18527,8 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月27日</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>1458</v>
-      </c>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="20" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -18951,14 +18554,8 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月28日</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>1657</v>
-      </c>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="20" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -18984,14 +18581,8 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月29日</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>1725</v>
-      </c>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="20" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -19017,14 +18608,8 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月30日</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>3541</v>
-      </c>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -19050,14 +18635,8 @@
       <c r="Y30" s="18" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>2026年5月31日</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="n">
-        <v>3318</v>
-      </c>
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="20" t="n"/>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="15" t="n"/>
       <c r="E31" s="17" t="n"/>
@@ -33463,11 +33042,11 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>2025年5月1日</t>
+          <t>2025年6月1日</t>
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>6619</v>
+        <v>5322</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -33490,14 +33069,8 @@
       <c r="U1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月2日</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>6313</v>
-      </c>
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="20" t="n"/>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -33519,14 +33092,8 @@
       <c r="U2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月3日</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>5619</v>
-      </c>
+      <c r="A3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -33548,14 +33115,8 @@
       <c r="U3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月4日</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>5576</v>
-      </c>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -33577,14 +33138,8 @@
       <c r="U4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月5日</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>5963</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="20" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -33606,14 +33161,8 @@
       <c r="U5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月6日</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>5196</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -33635,14 +33184,8 @@
       <c r="U6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月7日</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>6078</v>
-      </c>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -33664,14 +33207,8 @@
       <c r="U7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月8日</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>2247</v>
-      </c>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -33693,14 +33230,8 @@
       <c r="U8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月9日</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>2354</v>
-      </c>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -33722,14 +33253,8 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月10日</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n">
-        <v>3606</v>
-      </c>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -33751,14 +33276,8 @@
       <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月11日</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>4047</v>
-      </c>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -33780,14 +33299,8 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月12日</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>2740</v>
-      </c>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -33809,14 +33322,8 @@
       <c r="U12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月13日</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>2405</v>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -33838,14 +33345,8 @@
       <c r="U13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月14日</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>2575</v>
-      </c>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -33867,14 +33368,8 @@
       <c r="U14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月15日</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>2513</v>
-      </c>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -33896,14 +33391,8 @@
       <c r="U15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月16日</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>2771</v>
-      </c>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -33925,14 +33414,8 @@
       <c r="U16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月17日</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>4030</v>
-      </c>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -33954,14 +33437,8 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月18日</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="n">
-        <v>4424</v>
-      </c>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="20" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -33983,14 +33460,8 @@
       <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月19日</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>3066</v>
-      </c>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -34012,14 +33483,8 @@
       <c r="U19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月20日</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="n">
-        <v>2845</v>
-      </c>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="20" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -34041,14 +33506,8 @@
       <c r="U20" s="18" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月21日</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>3188</v>
-      </c>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -34070,14 +33529,8 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月22日</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>3080</v>
-      </c>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="20" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -34099,14 +33552,8 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>3506</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -34128,14 +33575,8 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月24日</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>4639</v>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="20" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34157,14 +33598,8 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月25日</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>4546</v>
-      </c>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="20" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34186,14 +33621,8 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月26日</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
-        <v>4370</v>
-      </c>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="20" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34215,14 +33644,8 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月27日</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>3834</v>
-      </c>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="20" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34244,14 +33667,8 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月28日</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>3669</v>
-      </c>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="20" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34273,14 +33690,8 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月29日</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>3709</v>
-      </c>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="20" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34302,14 +33713,8 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月30日</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>12066</v>
-      </c>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -34331,14 +33736,8 @@
       <c r="U30" s="18" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>2025年5月31日</t>
-        </is>
-      </c>
-      <c r="B31" s="20" t="n">
-        <v>9878</v>
-      </c>
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="20" t="n"/>
       <c r="C31" s="15" t="n"/>
       <c r="D31" s="15" t="n"/>
       <c r="E31" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-02 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5024,7 +5024,7 @@
         <v>46174</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
@@ -5034,8 +5034,12 @@
       <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n"/>
-      <c r="B3" s="21" t="n"/>
+      <c r="A3" s="23" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B3" s="21" t="n">
+        <v>1457</v>
+      </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -13746,8 +13750,12 @@
       <c r="G2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n"/>
-      <c r="B3" s="21" t="n"/>
+      <c r="A3" s="23" t="n">
+        <v>45810</v>
+      </c>
+      <c r="B3" s="21" t="n">
+        <v>2163</v>
+      </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -17824,8 +17832,8 @@
           <t>2026年6月1日</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n">
-        <v>1023</v>
+      <c r="B1" s="24" t="n">
+        <v>1043</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17852,8 +17860,14 @@
       <c r="Y1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月2日</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="n">
+        <v>879</v>
+      </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -33045,7 +33059,7 @@
           <t>2025年6月1日</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n">
+      <c r="B1" s="24" t="n">
         <v>5322</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33069,8 +33083,14 @@
       <c r="U1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月2日</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="n">
+        <v>4961</v>
+      </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-03 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5051,8 +5051,12 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
-      <c r="B4" s="21" t="n"/>
+      <c r="A4" s="23" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>1493</v>
+      </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -13763,8 +13767,12 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
-      <c r="B4" s="21" t="n"/>
+      <c r="A4" s="23" t="n">
+        <v>45811</v>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>1249</v>
+      </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -17833,7 +17841,7 @@
         </is>
       </c>
       <c r="B1" s="24" t="n">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17866,7 +17874,7 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>879</v>
+        <v>891</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17893,8 +17901,14 @@
       <c r="Y2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月3日</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n">
+        <v>982</v>
+      </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -33059,7 +33073,7 @@
           <t>2025年6月1日</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n">
+      <c r="B1" s="20" t="n">
         <v>5322</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33088,7 +33102,7 @@
           <t>2025年6月2日</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="20" t="n">
         <v>4961</v>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -33112,8 +33126,14 @@
       <c r="U2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月3日</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="n">
+        <v>2882</v>
+      </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>

</xml_diff>

<commit_message>
Rebuild dashboard with latest June data
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5068,8 +5068,12 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="21" t="n"/>
+      <c r="A5" s="23" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1612</v>
+      </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -13780,8 +13784,12 @@
       <c r="G4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="21" t="n"/>
+      <c r="A5" s="23" t="n">
+        <v>45812</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1280</v>
+      </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -17874,7 +17882,7 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17907,7 +17915,7 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>982</v>
+        <v>993</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17934,8 +17942,14 @@
       <c r="Y3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月4日</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>940</v>
+      </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -33155,8 +33169,14 @@
       <c r="U3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月4日</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="n">
+        <v>3007</v>
+      </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-05 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5085,8 +5085,12 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="21" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1739</v>
+      </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -13797,8 +13801,12 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="21" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>45813</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1259</v>
+      </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -17915,7 +17923,7 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17948,7 +17956,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -17975,8 +17983,14 @@
       <c r="Y4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月5日</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>1042</v>
+      </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -33198,8 +33212,14 @@
       <c r="U4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月5日</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>2476</v>
+      </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-06 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5102,8 +5102,12 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="21" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>2577</v>
+      </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -13814,8 +13818,12 @@
       <c r="G6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="21" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>45814</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>1347</v>
+      </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -17956,7 +17964,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>946</v>
+        <v>951</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -17989,7 +17997,7 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>1042</v>
+        <v>1047</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18016,8 +18024,14 @@
       <c r="Y5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月6日</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>1588</v>
+      </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -33241,8 +33255,14 @@
       <c r="U5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月6日</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>2902</v>
+      </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-07 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5072,7 +5072,7 @@
         <v>46177</v>
       </c>
       <c r="B5" s="21" t="n">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
@@ -5119,8 +5119,12 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="21" t="n"/>
+      <c r="A8" s="23" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>2775</v>
+      </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -13831,8 +13835,12 @@
       <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="21" t="n"/>
+      <c r="A8" s="23" t="n">
+        <v>45815</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>2374</v>
+      </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -17864,7 +17872,7 @@
           <t>2026年6月1日</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n">
+      <c r="B1" s="20" t="n">
         <v>1046</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -17897,7 +17905,7 @@
           <t>2026年6月2日</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="20" t="n">
         <v>893</v>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -17930,7 +17938,7 @@
           <t>2026年6月3日</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="20" t="n">
         <v>995</v>
       </c>
       <c r="C3" s="17" t="n"/>
@@ -17963,7 +17971,7 @@
           <t>2026年6月4日</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="20" t="n">
         <v>951</v>
       </c>
       <c r="C4" s="15" t="n"/>
@@ -17996,8 +18004,8 @@
           <t>2026年6月5日</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
-        <v>1047</v>
+      <c r="B5" s="20" t="n">
+        <v>1051</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18029,8 +18037,8 @@
           <t>2026年6月6日</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
-        <v>1588</v>
+      <c r="B6" s="20" t="n">
+        <v>1608</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18057,8 +18065,14 @@
       <c r="Y6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月7日</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>1983</v>
+      </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -33284,8 +33298,14 @@
       <c r="U6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月7日</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>3826</v>
+      </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-08 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5136,8 +5136,12 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="21" t="n"/>
+      <c r="A9" s="23" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>1610</v>
+      </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -13848,8 +13852,12 @@
       <c r="G8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="21" t="n"/>
+      <c r="A9" s="23" t="n">
+        <v>45816</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>2440</v>
+      </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -18038,7 +18046,7 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>1608</v>
+        <v>1619</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18071,7 +18079,7 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>1983</v>
+        <v>2004</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -18098,8 +18106,14 @@
       <c r="Y7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月8日</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>1336</v>
+      </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -33327,8 +33341,14 @@
       <c r="U7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月8日</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>4737</v>
+      </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-09 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5140,7 +5140,7 @@
         <v>46181</v>
       </c>
       <c r="B9" s="21" t="n">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
@@ -5153,8 +5153,12 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>1538</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -13865,8 +13869,12 @@
       <c r="G9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>45817</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>1373</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -18079,7 +18087,7 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>2004</v>
+        <v>2017</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -18112,7 +18120,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>1336</v>
+        <v>1345</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18139,8 +18147,14 @@
       <c r="Y8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月9日</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>1170</v>
+      </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -33370,8 +33384,14 @@
       <c r="U8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月9日</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>3199</v>
+      </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-10 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5024,7 +5024,7 @@
         <v>46174</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
@@ -5123,7 +5123,7 @@
         <v>46180</v>
       </c>
       <c r="B8" s="21" t="n">
-        <v>2775</v>
+        <v>2773</v>
       </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
@@ -5170,8 +5170,12 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>1512</v>
+      </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -13882,8 +13886,12 @@
       <c r="G10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>45818</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>1271</v>
+      </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -18120,7 +18128,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>1345</v>
+        <v>1349</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18153,7 +18161,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>1170</v>
+        <v>1186</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18180,8 +18188,14 @@
       <c r="Y9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月10日</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>1144</v>
+      </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -33413,8 +33427,14 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月10日</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>2759</v>
+      </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-11 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5140,7 +5140,7 @@
         <v>46181</v>
       </c>
       <c r="B9" s="21" t="n">
-        <v>1609</v>
+        <v>1607</v>
       </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
@@ -5174,7 +5174,7 @@
         <v>46183</v>
       </c>
       <c r="B11" s="21" t="n">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
@@ -5187,8 +5187,12 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="21" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>1555</v>
+      </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -13899,8 +13903,12 @@
       <c r="G11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="21" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>45819</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>1401</v>
+      </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -18161,7 +18169,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>1186</v>
+        <v>1191</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18194,7 +18202,7 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>1144</v>
+        <v>1152</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -18221,8 +18229,14 @@
       <c r="Y10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月11日</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>1088</v>
+      </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -33456,8 +33470,14 @@
       <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月11日</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>2863</v>
+      </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-12 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5204,8 +5204,12 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>1684</v>
+      </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -13916,8 +13920,12 @@
       <c r="G12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>45820</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>1408</v>
+      </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -18037,7 +18045,7 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18202,7 +18210,7 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -18235,7 +18243,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1088</v>
+        <v>1097</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18262,8 +18270,14 @@
       <c r="Y11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月12日</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>1308</v>
+      </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -33499,8 +33513,14 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月12日</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>2804</v>
+      </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-13 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5038,7 +5038,7 @@
         <v>46175</v>
       </c>
       <c r="B3" s="21" t="n">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
@@ -5208,7 +5208,7 @@
         <v>46185</v>
       </c>
       <c r="B13" s="21" t="n">
-        <v>1684</v>
+        <v>1683</v>
       </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
@@ -5221,8 +5221,12 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>2636</v>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -13933,8 +13937,12 @@
       <c r="G13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>45821</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>1435</v>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -18243,7 +18251,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1097</v>
+        <v>1104</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18276,7 +18284,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1308</v>
+        <v>1324</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18303,8 +18311,14 @@
       <c r="Y12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月13日</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>1724</v>
+      </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -33542,8 +33556,14 @@
       <c r="U12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月13日</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>3244</v>
+      </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-14 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5225,7 +5225,7 @@
         <v>46186</v>
       </c>
       <c r="B14" s="21" t="n">
-        <v>2636</v>
+        <v>2635</v>
       </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
@@ -5238,8 +5238,12 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
+      <c r="A15" s="23" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>2626</v>
+      </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -13950,8 +13954,12 @@
       <c r="G14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
+      <c r="A15" s="23" t="n">
+        <v>45822</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>2291</v>
+      </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -17921,7 +17929,7 @@
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>1046</v>
+        <v>1043</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17954,7 +17962,7 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17987,7 +17995,7 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>995</v>
+        <v>991</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -18020,7 +18028,7 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -18053,7 +18061,7 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>1052</v>
+        <v>1019</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18086,7 +18094,7 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>1619</v>
+        <v>1584</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18152,7 +18160,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>1349</v>
+        <v>1314</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18185,7 +18193,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18251,7 +18259,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1104</v>
+        <v>1101</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18284,7 +18292,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1324</v>
+        <v>1297</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18317,7 +18325,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1724</v>
+        <v>1737</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -18344,8 +18352,14 @@
       <c r="Y13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月14日</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>2050</v>
+      </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -33214,7 +33228,7 @@
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>5322</v>
+        <v>5301</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -33243,7 +33257,7 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>4961</v>
+        <v>4945</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -33272,7 +33286,7 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>2882</v>
+        <v>2874</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -33301,7 +33315,7 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>3007</v>
+        <v>3005</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -33330,7 +33344,7 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>2476</v>
+        <v>2460</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -33388,7 +33402,7 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>3826</v>
+        <v>3812</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -33417,7 +33431,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>4737</v>
+        <v>4728</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -33446,7 +33460,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>3199</v>
+        <v>3162</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -33475,7 +33489,7 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>2759</v>
+        <v>2744</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -33504,7 +33518,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>2863</v>
+        <v>2857</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -33533,7 +33547,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>2804</v>
+        <v>2758</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -33562,7 +33576,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>3244</v>
+        <v>3230</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -33585,8 +33599,14 @@
       <c r="U13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月14日</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>6416</v>
+      </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-15 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5255,8 +5255,12 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="21" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1344</v>
+      </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -13967,8 +13971,12 @@
       <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="21" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>45823</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>2285</v>
+      </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -17929,7 +17937,7 @@
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17962,7 +17970,7 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17995,7 +18003,7 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -18028,7 +18036,7 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -18061,7 +18069,7 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>1019</v>
+        <v>1052</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18094,7 +18102,7 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>1584</v>
+        <v>1619</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18160,7 +18168,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>1314</v>
+        <v>1349</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18193,7 +18201,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>1189</v>
+        <v>1191</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18259,7 +18267,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18292,7 +18300,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1297</v>
+        <v>1328</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18325,7 +18333,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>1737</v>
+        <v>1743</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -18358,7 +18366,7 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>2050</v>
+        <v>2064</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18385,8 +18393,14 @@
       <c r="Y14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月15日</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>1376</v>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -33228,7 +33242,7 @@
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>5301</v>
+        <v>5322</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -33257,7 +33271,7 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>4945</v>
+        <v>4961</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -33286,7 +33300,7 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>2874</v>
+        <v>2882</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -33315,7 +33329,7 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>3005</v>
+        <v>3007</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -33344,7 +33358,7 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>2460</v>
+        <v>2476</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -33402,7 +33416,7 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>3812</v>
+        <v>3826</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -33431,7 +33445,7 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>4728</v>
+        <v>4737</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -33460,7 +33474,7 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>3162</v>
+        <v>3199</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -33489,7 +33503,7 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>2744</v>
+        <v>2759</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -33518,7 +33532,7 @@
         </is>
       </c>
       <c r="B11" s="20" t="n">
-        <v>2857</v>
+        <v>2863</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -33547,7 +33561,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>2758</v>
+        <v>2804</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -33576,7 +33590,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>3230</v>
+        <v>3244</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -33605,7 +33619,7 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>6416</v>
+        <v>6450</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -33628,8 +33642,14 @@
       <c r="U14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月15日</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>6176</v>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-16 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5191,7 +5191,7 @@
         <v>46184</v>
       </c>
       <c r="B12" s="21" t="n">
-        <v>1555</v>
+        <v>1554</v>
       </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
@@ -5259,7 +5259,7 @@
         <v>46188</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
@@ -5272,8 +5272,12 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="21" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>1415</v>
+      </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -13984,8 +13988,12 @@
       <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="21" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>45824</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>1355</v>
+      </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -18366,7 +18374,7 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>2064</v>
+        <v>2065</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18399,7 +18407,7 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>1376</v>
+        <v>1383</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18426,8 +18434,14 @@
       <c r="Y15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月16日</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>1392</v>
+      </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -33671,8 +33685,14 @@
       <c r="U15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月16日</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>5140</v>
+      </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-17 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5289,8 +5289,12 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="21" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>1420</v>
+      </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -14001,8 +14005,12 @@
       <c r="G17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="21" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>45825</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>1306</v>
+      </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -18407,7 +18415,7 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18440,7 +18448,7 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1392</v>
+        <v>1404</v>
       </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -18467,8 +18475,14 @@
       <c r="Y16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月17日</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>1369</v>
+      </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -33714,8 +33728,14 @@
       <c r="U16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月17日</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>4742</v>
+      </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-18 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5259,7 +5259,7 @@
         <v>46188</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
@@ -5306,8 +5306,12 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="21" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>1414</v>
+      </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -14018,8 +14022,12 @@
       <c r="G18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="21" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>45826</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>1466</v>
+      </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -18316,7 +18324,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18415,7 +18423,7 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18448,7 +18456,7 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>1404</v>
+        <v>1408</v>
       </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -18481,7 +18489,7 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>1369</v>
+        <v>1377</v>
       </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -18508,8 +18516,14 @@
       <c r="Y17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月18日</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>1418</v>
+      </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -33757,8 +33771,14 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月18日</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>4734</v>
+      </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-19 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5323,8 +5323,12 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="21" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>2184</v>
+      </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -14035,8 +14039,12 @@
       <c r="G19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="21" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>45827</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>1430</v>
+      </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -18489,7 +18497,7 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>1377</v>
+        <v>1385</v>
       </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -18522,7 +18530,7 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1418</v>
+        <v>1426</v>
       </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
@@ -18549,8 +18557,14 @@
       <c r="Y18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月19日</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>2132</v>
+      </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -33800,8 +33814,14 @@
       <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月19日</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>4369</v>
+      </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-20 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5340,8 +5340,12 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="21" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>2608</v>
+      </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -14052,8 +14056,12 @@
       <c r="G20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="21" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>45828</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>1440</v>
+      </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -18530,7 +18538,7 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
@@ -18563,7 +18571,7 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>2132</v>
+        <v>2143</v>
       </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
@@ -18590,8 +18598,14 @@
       <c r="Y19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月20日</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>2331</v>
+      </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -33843,8 +33857,14 @@
       <c r="U19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月20日</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>4822</v>
+      </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-21 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5357,8 +5357,12 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="21" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>2173</v>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -14069,8 +14073,12 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="21" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>45829</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>2313</v>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -18571,7 +18579,7 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>2143</v>
+        <v>2146</v>
       </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
@@ -18604,7 +18612,7 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>2331</v>
+        <v>2350</v>
       </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
@@ -18631,8 +18639,14 @@
       <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月21日</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>2090</v>
+      </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -33886,8 +33900,14 @@
       <c r="U20" s="18" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月21日</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>6238</v>
+      </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-22 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5374,8 +5374,12 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="21" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>1334</v>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -14086,8 +14090,12 @@
       <c r="G22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="21" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>45830</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>2412</v>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -18612,7 +18620,7 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>2350</v>
+        <v>2373</v>
       </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
@@ -18645,7 +18653,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>2090</v>
+        <v>2111</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18672,8 +18680,14 @@
       <c r="Y21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月22日</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>1949</v>
+      </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -33929,8 +33943,14 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月22日</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>9576</v>
+      </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-23 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5174,7 +5174,7 @@
         <v>46183</v>
       </c>
       <c r="B11" s="21" t="n">
-        <v>1511</v>
+        <v>1510</v>
       </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
@@ -5391,8 +5391,12 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="21" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>1206</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14103,8 +14107,12 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="21" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>45831</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>1457</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -18653,7 +18661,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>2111</v>
+        <v>2128</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18686,7 +18694,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>1949</v>
+        <v>1956</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18713,8 +18721,14 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>2042</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -33972,8 +33986,14 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>6451</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-24 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5344,7 +5344,7 @@
         <v>46193</v>
       </c>
       <c r="B21" s="21" t="n">
-        <v>2608</v>
+        <v>2609</v>
       </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
@@ -5395,7 +5395,7 @@
         <v>46196</v>
       </c>
       <c r="B24" s="21" t="n">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
@@ -5408,8 +5408,12 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="21" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>1392</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14120,8 +14124,12 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="21" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>45832</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>1502</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -18694,7 +18702,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>1956</v>
+        <v>1960</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18727,7 +18735,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>2042</v>
+        <v>2048</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18754,8 +18762,14 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>1875</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34015,8 +34029,14 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>5592</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-25 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5425,8 +5425,12 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="21" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>1523</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14137,8 +14141,12 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="21" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>45833</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>1552</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -18735,7 +18743,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>2048</v>
+        <v>2053</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18768,7 +18776,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1875</v>
+        <v>1884</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18795,8 +18803,14 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>1926</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34058,8 +34072,14 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>3735</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-26 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5242,7 +5242,7 @@
         <v>46187</v>
       </c>
       <c r="B15" s="21" t="n">
-        <v>2626</v>
+        <v>2625</v>
       </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
@@ -5442,8 +5442,12 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="21" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>1513</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14154,8 +14158,12 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="21" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>45834</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>1451</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -18776,7 +18784,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1884</v>
+        <v>1886</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18809,7 +18817,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1926</v>
+        <v>1931</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18836,8 +18844,14 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>1949</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34101,8 +34115,14 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>3579</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-27 (silent)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5459,8 +5459,12 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="21" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>46200</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>2349</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14171,8 +14175,12 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="21" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>45835</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>1688</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -18817,7 +18825,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1931</v>
+        <v>1934</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18850,7 +18858,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1949</v>
+        <v>1967</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18877,8 +18885,14 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>2263</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34144,8 +34158,14 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>4723</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-28 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5106,7 +5106,7 @@
         <v>46179</v>
       </c>
       <c r="B7" s="21" t="n">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
@@ -5429,7 +5429,7 @@
         <v>46198</v>
       </c>
       <c r="B26" s="21" t="n">
-        <v>1523</v>
+        <v>1522</v>
       </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
@@ -5476,8 +5476,12 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="21" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>46201</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>2306</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14188,8 +14192,12 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="21" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>45836</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>2363</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -18858,7 +18866,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1967</v>
+        <v>1971</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18891,7 +18899,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>2263</v>
+        <v>2278</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18918,8 +18926,14 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>2533</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34187,8 +34201,14 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>5827</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-29 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5446,7 +5446,7 @@
         <v>46199</v>
       </c>
       <c r="B27" s="21" t="n">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
@@ -5463,7 +5463,7 @@
         <v>46200</v>
       </c>
       <c r="B28" s="21" t="n">
-        <v>2349</v>
+        <v>2347</v>
       </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
@@ -5493,8 +5493,12 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="21" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>1355</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14205,8 +14209,12 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="21" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>45837</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>2424</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -18899,7 +18907,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>2278</v>
+        <v>2277</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18932,7 +18940,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>2533</v>
+        <v>2550</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18959,8 +18967,14 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>3463</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34230,8 +34244,14 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>8688</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-06-30 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5480,7 +5480,7 @@
         <v>46201</v>
       </c>
       <c r="B29" s="21" t="n">
-        <v>2306</v>
+        <v>2305</v>
       </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
@@ -5497,7 +5497,7 @@
         <v>46202</v>
       </c>
       <c r="B30" s="21" t="n">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
@@ -5510,8 +5510,12 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="21" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1456</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -14222,8 +14226,12 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="21" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1779</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -18478,7 +18486,7 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>2065</v>
+        <v>2064</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18940,7 +18948,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>2550</v>
+        <v>2556</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18973,7 +18981,7 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>3463</v>
+        <v>3480</v>
       </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
@@ -19000,8 +19008,14 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2026年6月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>5711</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -34221,7 +34235,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>5827</v>
+        <v>5826</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -34273,8 +34287,14 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2025年6月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>7120</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-01 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5021,10 +5021,10 @@
     </row>
     <row r="2">
       <c r="A2" s="23" t="n">
-        <v>46174</v>
+        <v>46204</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>1260</v>
+        <v>703</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
@@ -5034,12 +5034,8 @@
       <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>46175</v>
-      </c>
-      <c r="B3" s="21" t="n">
-        <v>1456</v>
-      </c>
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="21" t="n"/>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -5051,12 +5047,8 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>46176</v>
-      </c>
-      <c r="B4" s="21" t="n">
-        <v>1493</v>
-      </c>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -5068,12 +5060,8 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>46177</v>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>1611</v>
-      </c>
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -5085,12 +5073,8 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>46178</v>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>1739</v>
-      </c>
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="21" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -5102,12 +5086,8 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>46179</v>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>2576</v>
-      </c>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -5119,12 +5099,8 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>46180</v>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>2773</v>
-      </c>
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="21" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -5136,12 +5112,8 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>46181</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>1607</v>
-      </c>
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -5153,12 +5125,8 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>46182</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>1538</v>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -5170,12 +5138,8 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>46183</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>1510</v>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -5187,12 +5151,8 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>46184</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>1554</v>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -5204,12 +5164,8 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>1683</v>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -5221,12 +5177,8 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>46186</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>2635</v>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -5238,12 +5190,8 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>2625</v>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -5255,12 +5203,8 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>46188</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <v>1344</v>
-      </c>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="21" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -5272,12 +5216,8 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>46189</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <v>1415</v>
-      </c>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -5289,12 +5229,8 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>46190</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>1420</v>
-      </c>
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="21" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -5306,12 +5242,8 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <v>1414</v>
-      </c>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -5323,12 +5255,8 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>46192</v>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>2184</v>
-      </c>
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="21" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -5340,12 +5268,8 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>2609</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -5357,12 +5281,8 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>46194</v>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>2173</v>
-      </c>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="21" t="n"/>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -5374,12 +5294,8 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>46195</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <v>1334</v>
-      </c>
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -5391,12 +5307,8 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>46196</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>1205</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -5408,12 +5320,8 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
-        <v>46197</v>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>1392</v>
-      </c>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -5425,12 +5333,8 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
-        <v>46198</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>1522</v>
-      </c>
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="21" t="n"/>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -5442,12 +5346,8 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n">
-        <v>46199</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>1512</v>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -5459,12 +5359,8 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>2347</v>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="21" t="n"/>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -5476,12 +5372,8 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
-        <v>46201</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>2305</v>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -5493,12 +5385,8 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
-        <v>46202</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>1354</v>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="21" t="n"/>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -5510,12 +5398,8 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>1456</v>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -13853,21 +13737,17 @@
     </row>
     <row r="2">
       <c r="A2" s="23" t="n">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B2" s="21" t="n">
-        <v>2129</v>
+        <v>1021</v>
       </c>
       <c r="F2" s="12" t="n"/>
       <c r="G2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n">
-        <v>45810</v>
-      </c>
-      <c r="B3" s="21" t="n">
-        <v>2163</v>
-      </c>
+      <c r="A3" s="23" t="n"/>
+      <c r="B3" s="21" t="n"/>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -13875,12 +13755,8 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n">
-        <v>45811</v>
-      </c>
-      <c r="B4" s="21" t="n">
-        <v>1249</v>
-      </c>
+      <c r="A4" s="23" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -13888,12 +13764,8 @@
       <c r="G4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
-        <v>45812</v>
-      </c>
-      <c r="B5" s="21" t="n">
-        <v>1280</v>
-      </c>
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="21" t="n"/>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -13901,12 +13773,8 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
-        <v>45813</v>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>1259</v>
-      </c>
+      <c r="A6" s="23" t="n"/>
+      <c r="B6" s="21" t="n"/>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -13914,12 +13782,8 @@
       <c r="G6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
-        <v>45814</v>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>1347</v>
-      </c>
+      <c r="A7" s="23" t="n"/>
+      <c r="B7" s="21" t="n"/>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -13927,12 +13791,8 @@
       <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
-        <v>45815</v>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>2374</v>
-      </c>
+      <c r="A8" s="23" t="n"/>
+      <c r="B8" s="21" t="n"/>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -13940,12 +13800,8 @@
       <c r="G8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
-        <v>45816</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>2440</v>
-      </c>
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="21" t="n"/>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -13953,12 +13809,8 @@
       <c r="G9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
-        <v>45817</v>
-      </c>
-      <c r="B10" s="21" t="n">
-        <v>1373</v>
-      </c>
+      <c r="A10" s="23" t="n"/>
+      <c r="B10" s="21" t="n"/>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -13966,12 +13818,8 @@
       <c r="G10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
-        <v>45818</v>
-      </c>
-      <c r="B11" s="21" t="n">
-        <v>1271</v>
-      </c>
+      <c r="A11" s="23" t="n"/>
+      <c r="B11" s="21" t="n"/>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -13979,12 +13827,8 @@
       <c r="G11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
-        <v>45819</v>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>1401</v>
-      </c>
+      <c r="A12" s="23" t="n"/>
+      <c r="B12" s="21" t="n"/>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -13992,12 +13836,8 @@
       <c r="G12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
-        <v>45820</v>
-      </c>
-      <c r="B13" s="21" t="n">
-        <v>1408</v>
-      </c>
+      <c r="A13" s="23" t="n"/>
+      <c r="B13" s="21" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -14005,12 +13845,8 @@
       <c r="G13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
-        <v>45821</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>1435</v>
-      </c>
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="21" t="n"/>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -14018,12 +13854,8 @@
       <c r="G14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>45822</v>
-      </c>
-      <c r="B15" s="21" t="n">
-        <v>2291</v>
-      </c>
+      <c r="A15" s="23" t="n"/>
+      <c r="B15" s="21" t="n"/>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -14031,12 +13863,8 @@
       <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>45823</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <v>2285</v>
-      </c>
+      <c r="A16" s="23" t="n"/>
+      <c r="B16" s="21" t="n"/>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -14044,12 +13872,8 @@
       <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>45824</v>
-      </c>
-      <c r="B17" s="21" t="n">
-        <v>1355</v>
-      </c>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="21" t="n"/>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -14057,12 +13881,8 @@
       <c r="G17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>45825</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>1306</v>
-      </c>
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="21" t="n"/>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -14070,12 +13890,8 @@
       <c r="G18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>45826</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <v>1466</v>
-      </c>
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="21" t="n"/>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -14083,12 +13899,8 @@
       <c r="G19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n">
-        <v>45827</v>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>1430</v>
-      </c>
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="21" t="n"/>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -14096,12 +13908,8 @@
       <c r="G20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n">
-        <v>45828</v>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>1440</v>
-      </c>
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="21" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -14109,12 +13917,8 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n">
-        <v>45829</v>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>2313</v>
-      </c>
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="21" t="n"/>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -14122,12 +13926,8 @@
       <c r="G22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n">
-        <v>45830</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <v>2412</v>
-      </c>
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="21" t="n"/>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -14135,12 +13935,8 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n">
-        <v>45831</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <v>1457</v>
-      </c>
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="21" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14148,12 +13944,8 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n">
-        <v>45832</v>
-      </c>
-      <c r="B25" s="21" t="n">
-        <v>1502</v>
-      </c>
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="21" t="n"/>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14161,12 +13953,8 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n">
-        <v>45833</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <v>1552</v>
-      </c>
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="21" t="n"/>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14174,12 +13962,8 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n">
-        <v>45834</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <v>1451</v>
-      </c>
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="21" t="n"/>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14187,12 +13971,8 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n">
-        <v>45835</v>
-      </c>
-      <c r="B28" s="21" t="n">
-        <v>1688</v>
-      </c>
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="21" t="n"/>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14200,12 +13980,8 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n">
-        <v>45836</v>
-      </c>
-      <c r="B29" s="21" t="n">
-        <v>2363</v>
-      </c>
+      <c r="A29" s="23" t="n"/>
+      <c r="B29" s="21" t="n"/>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14213,12 +13989,8 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n">
-        <v>45837</v>
-      </c>
-      <c r="B30" s="21" t="n">
-        <v>2424</v>
-      </c>
+      <c r="A30" s="23" t="n"/>
+      <c r="B30" s="21" t="n"/>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14226,12 +13998,8 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n">
-        <v>45838</v>
-      </c>
-      <c r="B31" s="21" t="n">
-        <v>1779</v>
-      </c>
+      <c r="A31" s="23" t="n"/>
+      <c r="B31" s="21" t="n"/>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -18053,11 +17821,11 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>2026年6月1日</t>
+          <t>2026年7月1日</t>
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>1046</v>
+        <v>1112</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -18084,14 +17852,8 @@
       <c r="Y1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月2日</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>893</v>
-      </c>
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="20" t="n"/>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -18117,14 +17879,8 @@
       <c r="Y2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月3日</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>995</v>
-      </c>
+      <c r="A3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -18150,14 +17906,8 @@
       <c r="Y3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月4日</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>951</v>
-      </c>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -18183,14 +17933,8 @@
       <c r="Y4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月5日</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>1052</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="20" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -18216,14 +17960,8 @@
       <c r="Y5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月6日</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>1619</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -18249,14 +17987,8 @@
       <c r="Y6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月7日</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>2017</v>
-      </c>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -18282,14 +18014,8 @@
       <c r="Y7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月8日</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>1349</v>
-      </c>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -18315,14 +18041,8 @@
       <c r="Y8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月9日</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>1191</v>
-      </c>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -18348,14 +18068,8 @@
       <c r="Y9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月10日</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n">
-        <v>1151</v>
-      </c>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -18381,14 +18095,8 @@
       <c r="Y10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月11日</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>1104</v>
-      </c>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -18414,14 +18122,8 @@
       <c r="Y11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月12日</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>1329</v>
-      </c>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -18447,14 +18149,8 @@
       <c r="Y12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月13日</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>1743</v>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -18480,14 +18176,8 @@
       <c r="Y13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月14日</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>2064</v>
-      </c>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -18513,14 +18203,8 @@
       <c r="Y14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月15日</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>1385</v>
-      </c>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -18546,14 +18230,8 @@
       <c r="Y15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月16日</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>1408</v>
-      </c>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -18579,14 +18257,8 @@
       <c r="Y16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月17日</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>1385</v>
-      </c>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -18612,14 +18284,8 @@
       <c r="Y17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月18日</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="n">
-        <v>1427</v>
-      </c>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="20" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -18645,14 +18311,8 @@
       <c r="Y18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月19日</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>2146</v>
-      </c>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -18678,14 +18338,8 @@
       <c r="Y19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月20日</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="n">
-        <v>2373</v>
-      </c>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="20" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -18711,14 +18365,8 @@
       <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月21日</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>2128</v>
-      </c>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -18744,14 +18392,8 @@
       <c r="Y21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月22日</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>1960</v>
-      </c>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="20" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -18777,14 +18419,8 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>2053</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -18810,14 +18446,8 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月24日</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>1886</v>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="20" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -18843,14 +18473,8 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月25日</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>1934</v>
-      </c>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="20" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -18876,14 +18500,8 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月26日</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
-        <v>1971</v>
-      </c>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="20" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -18909,14 +18527,8 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月27日</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>2277</v>
-      </c>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="20" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -18942,14 +18554,8 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月28日</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>2556</v>
-      </c>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="20" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -18975,14 +18581,8 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月29日</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>3480</v>
-      </c>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="20" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -19008,14 +18608,8 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>2026年6月30日</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>5711</v>
-      </c>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -33448,11 +33042,11 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>2025年6月1日</t>
+          <t>2025年7月1日</t>
         </is>
       </c>
       <c r="B1" s="20" t="n">
-        <v>5322</v>
+        <v>2137</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -33475,14 +33069,8 @@
       <c r="U1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月2日</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>4961</v>
-      </c>
+      <c r="A2" s="19" t="n"/>
+      <c r="B2" s="20" t="n"/>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -33504,14 +33092,8 @@
       <c r="U2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月3日</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>2882</v>
-      </c>
+      <c r="A3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -33533,14 +33115,8 @@
       <c r="U3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月4日</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>3007</v>
-      </c>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -33562,14 +33138,8 @@
       <c r="U4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月5日</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="n">
-        <v>2476</v>
-      </c>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="20" t="n"/>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -33591,14 +33161,8 @@
       <c r="U5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月6日</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>2902</v>
-      </c>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="n"/>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -33620,14 +33184,8 @@
       <c r="U6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月7日</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="n">
-        <v>3826</v>
-      </c>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -33649,14 +33207,8 @@
       <c r="U7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月8日</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n">
-        <v>4737</v>
-      </c>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -33678,14 +33230,8 @@
       <c r="U8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月9日</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n">
-        <v>3199</v>
-      </c>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="20" t="n"/>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -33707,14 +33253,8 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月10日</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n">
-        <v>2759</v>
-      </c>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="n"/>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -33736,14 +33276,8 @@
       <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月11日</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>2863</v>
-      </c>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="20" t="n"/>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -33765,14 +33299,8 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月12日</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="n">
-        <v>2804</v>
-      </c>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -33794,14 +33322,8 @@
       <c r="U12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月13日</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>3244</v>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -33823,14 +33345,8 @@
       <c r="U13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月14日</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>6450</v>
-      </c>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="20" t="n"/>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -33852,14 +33368,8 @@
       <c r="U14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月15日</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="n">
-        <v>6176</v>
-      </c>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -33881,14 +33391,8 @@
       <c r="U15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月16日</t>
-        </is>
-      </c>
-      <c r="B16" s="20" t="n">
-        <v>5140</v>
-      </c>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="20" t="n"/>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -33910,14 +33414,8 @@
       <c r="U16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月17日</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>4742</v>
-      </c>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -33939,14 +33437,8 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月18日</t>
-        </is>
-      </c>
-      <c r="B18" s="20" t="n">
-        <v>4734</v>
-      </c>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="20" t="n"/>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -33968,14 +33460,8 @@
       <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月19日</t>
-        </is>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>4369</v>
-      </c>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -33997,14 +33483,8 @@
       <c r="U19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月20日</t>
-        </is>
-      </c>
-      <c r="B20" s="20" t="n">
-        <v>4822</v>
-      </c>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="20" t="n"/>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -34026,14 +33506,8 @@
       <c r="U20" s="18" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月21日</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>6238</v>
-      </c>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -34055,14 +33529,8 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月22日</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="n">
-        <v>9576</v>
-      </c>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="20" t="n"/>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -34084,14 +33552,8 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月23日</t>
-        </is>
-      </c>
-      <c r="B23" s="20" t="n">
-        <v>6451</v>
-      </c>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="20" t="n"/>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -34113,14 +33575,8 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月24日</t>
-        </is>
-      </c>
-      <c r="B24" s="20" t="n">
-        <v>5592</v>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="20" t="n"/>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34142,14 +33598,8 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月25日</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
-        <v>3735</v>
-      </c>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="20" t="n"/>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34171,14 +33621,8 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月26日</t>
-        </is>
-      </c>
-      <c r="B26" s="20" t="n">
-        <v>3579</v>
-      </c>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="20" t="n"/>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34200,14 +33644,8 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月27日</t>
-        </is>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>4723</v>
-      </c>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="20" t="n"/>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34229,14 +33667,8 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月28日</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="n">
-        <v>5826</v>
-      </c>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="20" t="n"/>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34258,14 +33690,8 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月29日</t>
-        </is>
-      </c>
-      <c r="B29" s="20" t="n">
-        <v>8688</v>
-      </c>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="20" t="n"/>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34287,14 +33713,8 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
-        <is>
-          <t>2025年6月30日</t>
-        </is>
-      </c>
-      <c r="B30" s="20" t="n">
-        <v>7120</v>
-      </c>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-02 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -220,7 +220,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -280,6 +280,9 @@
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5034,8 +5037,12 @@
       <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n"/>
-      <c r="B3" s="21" t="n"/>
+      <c r="A3" s="23" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B3" s="21" t="n">
+        <v>688</v>
+      </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -13746,8 +13753,12 @@
       <c r="G2" s="12" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="n"/>
-      <c r="B3" s="21" t="n"/>
+      <c r="A3" s="23" t="n">
+        <v>45840</v>
+      </c>
+      <c r="B3" s="21" t="n">
+        <v>781</v>
+      </c>
       <c r="C3" s="13" t="n"/>
       <c r="D3" s="13" t="n"/>
       <c r="E3" s="13" t="n"/>
@@ -17824,8 +17835,8 @@
           <t>2026年7月1日</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n">
-        <v>1112</v>
+      <c r="B1" s="24" t="n">
+        <v>1130</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17852,8 +17863,14 @@
       <c r="Y1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月2日</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="n">
+        <v>871</v>
+      </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>
@@ -33045,7 +33062,7 @@
           <t>2025年7月1日</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n">
+      <c r="B1" s="25" t="n">
         <v>2137</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33069,8 +33086,14 @@
       <c r="U1" s="16" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="n"/>
-      <c r="B2" s="20" t="n"/>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月2日</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="n">
+        <v>2059</v>
+      </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
       <c r="E2" s="15" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-03 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5054,8 +5054,12 @@
       <c r="K3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
-      <c r="B4" s="21" t="n"/>
+      <c r="A4" s="23" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>683</v>
+      </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -13766,8 +13770,12 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="n"/>
-      <c r="B4" s="21" t="n"/>
+      <c r="A4" s="23" t="n">
+        <v>45841</v>
+      </c>
+      <c r="B4" s="21" t="n">
+        <v>951</v>
+      </c>
       <c r="C4" s="13" t="n"/>
       <c r="D4" s="13" t="n"/>
       <c r="E4" s="13" t="n"/>
@@ -17836,7 +17844,7 @@
         </is>
       </c>
       <c r="B1" s="24" t="n">
-        <v>1130</v>
+        <v>1132</v>
       </c>
       <c r="C1" s="14" t="n"/>
       <c r="D1" s="14" t="n"/>
@@ -17869,7 +17877,7 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17896,8 +17904,14 @@
       <c r="Y2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月3日</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n">
+        <v>949</v>
+      </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>
@@ -33062,7 +33076,7 @@
           <t>2025年7月1日</t>
         </is>
       </c>
-      <c r="B1" s="25" t="n">
+      <c r="B1" s="24" t="n">
         <v>2137</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33091,7 +33105,7 @@
           <t>2025年7月2日</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n">
+      <c r="B2" s="24" t="n">
         <v>2059</v>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -33115,8 +33129,14 @@
       <c r="U2" s="18" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="n"/>
-      <c r="B3" s="20" t="n"/>
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月3日</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n">
+        <v>2253</v>
+      </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
       <c r="E3" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-04 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5071,8 +5071,12 @@
       <c r="K4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="21" t="n"/>
+      <c r="A5" s="23" t="n">
+        <v>46207</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1360</v>
+      </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -13783,8 +13787,12 @@
       <c r="G4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n"/>
-      <c r="B5" s="21" t="n"/>
+      <c r="A5" s="23" t="n">
+        <v>45842</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>972</v>
+      </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
@@ -17877,7 +17885,7 @@
         </is>
       </c>
       <c r="B2" s="24" t="n">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="C2" s="15" t="n"/>
       <c r="D2" s="15" t="n"/>
@@ -17910,7 +17918,7 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>949</v>
+        <v>957</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17937,8 +17945,14 @@
       <c r="Y3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月4日</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>1328</v>
+      </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>
@@ -33158,8 +33172,14 @@
       <c r="U3" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="n"/>
-      <c r="B4" s="20" t="n"/>
+      <c r="A4" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月4日</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>2439</v>
+      </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
       <c r="E4" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-05 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5075,7 +5075,7 @@
         <v>46207</v>
       </c>
       <c r="B5" s="21" t="n">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="C5" s="13" t="n"/>
       <c r="D5" s="13" t="n"/>
@@ -5088,8 +5088,12 @@
       <c r="K5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="21" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1562</v>
+      </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -13800,8 +13804,12 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n"/>
-      <c r="B6" s="21" t="n"/>
+      <c r="A6" s="23" t="n">
+        <v>45843</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1785</v>
+      </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
       <c r="E6" s="13" t="n"/>
@@ -17918,7 +17926,7 @@
         </is>
       </c>
       <c r="B3" s="24" t="n">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="C3" s="17" t="n"/>
       <c r="D3" s="17" t="n"/>
@@ -17951,7 +17959,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>1328</v>
+        <v>1338</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -17978,8 +17986,14 @@
       <c r="Y4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月5日</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>1733</v>
+      </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>
@@ -33090,7 +33104,7 @@
           <t>2025年7月1日</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n">
+      <c r="B1" s="20" t="n">
         <v>2137</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -33119,7 +33133,7 @@
           <t>2025年7月2日</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="20" t="n">
         <v>2059</v>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -33148,7 +33162,7 @@
           <t>2025年7月3日</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="20" t="n">
         <v>2253</v>
       </c>
       <c r="C3" s="17" t="n"/>
@@ -33177,7 +33191,7 @@
           <t>2025年7月4日</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="20" t="n">
         <v>2439</v>
       </c>
       <c r="C4" s="15" t="n"/>
@@ -33201,8 +33215,14 @@
       <c r="U4" s="18" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n"/>
-      <c r="B5" s="20" t="n"/>
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月5日</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>4074</v>
+      </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-06 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5092,7 +5092,7 @@
         <v>46208</v>
       </c>
       <c r="B6" s="21" t="n">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="C6" s="13" t="n"/>
       <c r="D6" s="13" t="n"/>
@@ -5105,8 +5105,12 @@
       <c r="K6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="21" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>769</v>
+      </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -13817,8 +13821,12 @@
       <c r="G6" s="13" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n"/>
-      <c r="B7" s="21" t="n"/>
+      <c r="A7" s="23" t="n">
+        <v>45844</v>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>1874</v>
+      </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
       <c r="E7" s="13" t="n"/>
@@ -17959,7 +17967,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="C4" s="15" t="n"/>
       <c r="D4" s="15" t="n"/>
@@ -17992,7 +18000,7 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>1733</v>
+        <v>1753</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18019,8 +18027,14 @@
       <c r="Y5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月6日</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>1058</v>
+      </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>
@@ -33244,8 +33258,14 @@
       <c r="U5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月6日</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>4725</v>
+      </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
       <c r="E6" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-07 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5109,7 +5109,7 @@
         <v>46209</v>
       </c>
       <c r="B7" s="21" t="n">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C7" s="13" t="n"/>
       <c r="D7" s="13" t="n"/>
@@ -5122,8 +5122,12 @@
       <c r="K7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="21" t="n"/>
+      <c r="A8" s="23" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>794</v>
+      </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -13834,8 +13838,12 @@
       <c r="G7" s="13" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n"/>
-      <c r="B8" s="21" t="n"/>
+      <c r="A8" s="23" t="n">
+        <v>45845</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>981</v>
+      </c>
       <c r="C8" s="13" t="n"/>
       <c r="D8" s="13" t="n"/>
       <c r="E8" s="13" t="n"/>
@@ -18000,7 +18008,7 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="C5" s="15" t="n"/>
       <c r="D5" s="15" t="n"/>
@@ -18033,7 +18041,7 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>1058</v>
+        <v>1065</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18060,8 +18068,14 @@
       <c r="Y6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月7日</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>1026</v>
+      </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>
@@ -33287,8 +33301,14 @@
       <c r="U6" s="18" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n"/>
-      <c r="B7" s="20" t="n"/>
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月7日</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>3101</v>
+      </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
       <c r="E7" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-08 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5139,8 +5139,12 @@
       <c r="K8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="21" t="n"/>
+      <c r="A9" s="23" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>769</v>
+      </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -13851,8 +13855,12 @@
       <c r="G8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="21" t="n"/>
+      <c r="A9" s="23" t="n">
+        <v>45846</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>1025</v>
+      </c>
       <c r="C9" s="13" t="n"/>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
@@ -18041,7 +18049,7 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>1065</v>
+        <v>1067</v>
       </c>
       <c r="C6" s="15" t="n"/>
       <c r="D6" s="15" t="n"/>
@@ -18074,7 +18082,7 @@
         </is>
       </c>
       <c r="B7" s="24" t="n">
-        <v>1026</v>
+        <v>1033</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -18101,8 +18109,14 @@
       <c r="Y7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月8日</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>1024</v>
+      </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>
@@ -33330,8 +33344,14 @@
       <c r="U7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n"/>
-      <c r="B8" s="20" t="n"/>
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月8日</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="n">
+        <v>2912</v>
+      </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-09 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5156,8 +5156,12 @@
       <c r="K9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>764</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -13868,8 +13872,12 @@
       <c r="G9" s="13" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="21" t="n"/>
+      <c r="A10" s="23" t="n">
+        <v>45847</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>1076</v>
+      </c>
       <c r="C10" s="13" t="n"/>
       <c r="D10" s="13" t="n"/>
       <c r="E10" s="13" t="n"/>
@@ -18082,7 +18090,7 @@
         </is>
       </c>
       <c r="B7" s="24" t="n">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="15" t="n"/>
@@ -18115,7 +18123,7 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18142,8 +18150,14 @@
       <c r="Y8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月9日</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>1079</v>
+      </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>
@@ -33373,8 +33387,14 @@
       <c r="U8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="n"/>
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月9日</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>3139</v>
+      </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
       <c r="E9" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-10 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5173,8 +5173,12 @@
       <c r="K10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>860</v>
+      </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -13885,8 +13889,12 @@
       <c r="G10" s="13" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="21" t="n"/>
+      <c r="A11" s="23" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>1234</v>
+      </c>
       <c r="C11" s="13" t="n"/>
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
@@ -18123,7 +18131,7 @@
         </is>
       </c>
       <c r="B8" s="24" t="n">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
@@ -18156,7 +18164,7 @@
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>1079</v>
+        <v>1088</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18183,8 +18191,14 @@
       <c r="Y9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月10日</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>1044</v>
+      </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>
@@ -33416,8 +33430,14 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="n"/>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月10日</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>2796</v>
+      </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-11 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5190,8 +5190,12 @@
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="21" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>1599</v>
+      </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -13902,8 +13906,12 @@
       <c r="G11" s="13" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="21" t="n"/>
+      <c r="A12" s="23" t="n">
+        <v>45849</v>
+      </c>
+      <c r="B12" s="21" t="n">
+        <v>1153</v>
+      </c>
       <c r="C12" s="13" t="n"/>
       <c r="D12" s="13" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -18164,7 +18172,7 @@
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>1088</v>
+        <v>1092</v>
       </c>
       <c r="C9" s="15" t="n"/>
       <c r="D9" s="15" t="n"/>
@@ -18197,7 +18205,7 @@
         </is>
       </c>
       <c r="B10" s="24" t="n">
-        <v>1044</v>
+        <v>1047</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -18224,8 +18232,14 @@
       <c r="Y10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月11日</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>1441</v>
+      </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>
@@ -33459,8 +33473,14 @@
       <c r="U10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月11日</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>3348</v>
+      </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-12 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5207,8 +5207,12 @@
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>1552</v>
+      </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -13919,8 +13923,12 @@
       <c r="G12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="21" t="n"/>
+      <c r="A13" s="23" t="n">
+        <v>45850</v>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>1922</v>
+      </c>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="13" t="n"/>
@@ -18205,7 +18213,7 @@
         </is>
       </c>
       <c r="B10" s="24" t="n">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="C10" s="15" t="n"/>
       <c r="D10" s="15" t="n"/>
@@ -18238,7 +18246,7 @@
         </is>
       </c>
       <c r="B11" s="24" t="n">
-        <v>1441</v>
+        <v>1446</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18265,8 +18273,14 @@
       <c r="Y11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月12日</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>1692</v>
+      </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>
@@ -33502,8 +33516,14 @@
       <c r="U11" s="18" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月12日</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="n">
+        <v>4607</v>
+      </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-13 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5224,8 +5224,12 @@
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>902</v>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -13936,8 +13940,12 @@
       <c r="G13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="21" t="n"/>
+      <c r="A14" s="23" t="n">
+        <v>45851</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>1999</v>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -18246,7 +18254,7 @@
         </is>
       </c>
       <c r="B11" s="24" t="n">
-        <v>1446</v>
+        <v>1451</v>
       </c>
       <c r="C11" s="15" t="n"/>
       <c r="D11" s="15" t="n"/>
@@ -18279,7 +18287,7 @@
         </is>
       </c>
       <c r="B12" s="24" t="n">
-        <v>1692</v>
+        <v>1709</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18306,8 +18314,14 @@
       <c r="Y12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月13日</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>1296</v>
+      </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -33545,8 +33559,14 @@
       <c r="U12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="20" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月13日</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>5586</v>
+      </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
       <c r="E13" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-14 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5241,8 +5241,12 @@
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
+      <c r="A15" s="23" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>916</v>
+      </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -13953,8 +13957,12 @@
       <c r="G14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="21" t="n"/>
+      <c r="A15" s="23" t="n">
+        <v>45852</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1112</v>
+      </c>
       <c r="C15" s="13" t="n"/>
       <c r="D15" s="13" t="n"/>
       <c r="E15" s="13" t="n"/>
@@ -18287,7 +18295,7 @@
         </is>
       </c>
       <c r="B12" s="24" t="n">
-        <v>1709</v>
+        <v>1713</v>
       </c>
       <c r="C12" s="15" t="n"/>
       <c r="D12" s="15" t="n"/>
@@ -18320,7 +18328,7 @@
         </is>
       </c>
       <c r="B13" s="24" t="n">
-        <v>1296</v>
+        <v>1308</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -18347,8 +18355,14 @@
       <c r="Y13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月14日</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>1029</v>
+      </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>
@@ -33588,8 +33602,14 @@
       <c r="U13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n"/>
-      <c r="B14" s="20" t="n"/>
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月14日</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n">
+        <v>3749</v>
+      </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-15 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5258,8 +5258,12 @@
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="21" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1033</v>
+      </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -13970,8 +13974,12 @@
       <c r="G15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="21" t="n"/>
+      <c r="A16" s="23" t="n">
+        <v>45853</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>1052</v>
+      </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -18328,7 +18336,7 @@
         </is>
       </c>
       <c r="B13" s="24" t="n">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="15" t="n"/>
@@ -18361,7 +18369,7 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18388,8 +18396,14 @@
       <c r="Y14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月15日</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>1073</v>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -33631,8 +33645,14 @@
       <c r="U14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n"/>
-      <c r="B15" s="20" t="n"/>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月15日</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>3292</v>
+      </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
       <c r="E15" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-16 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5228,7 +5228,7 @@
         <v>46216</v>
       </c>
       <c r="B14" s="21" t="n">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
@@ -5262,7 +5262,7 @@
         <v>46218</v>
       </c>
       <c r="B16" s="21" t="n">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="C16" s="13" t="n"/>
       <c r="D16" s="13" t="n"/>
@@ -5275,8 +5275,12 @@
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="21" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>921</v>
+      </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -13987,8 +13991,12 @@
       <c r="G16" s="13" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="21" t="n"/>
+      <c r="A17" s="23" t="n">
+        <v>45854</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>1187</v>
+      </c>
       <c r="C17" s="13" t="n"/>
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="13" t="n"/>
@@ -18369,7 +18377,7 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="C14" s="15" t="n"/>
       <c r="D14" s="15" t="n"/>
@@ -18402,7 +18410,7 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18429,8 +18437,14 @@
       <c r="Y15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月16日</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>1141</v>
+      </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>
@@ -33674,8 +33688,14 @@
       <c r="U15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="20" t="n"/>
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月16日</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="n">
+        <v>3277</v>
+      </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
       <c r="E16" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-17 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5292,8 +5292,12 @@
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="21" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>1185</v>
+      </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -14004,8 +14008,12 @@
       <c r="G17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="21" t="n"/>
+      <c r="A18" s="23" t="n">
+        <v>45855</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>1182</v>
+      </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -18410,7 +18418,7 @@
         </is>
       </c>
       <c r="B15" s="24" t="n">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="C15" s="15" t="n"/>
       <c r="D15" s="15" t="n"/>
@@ -18443,7 +18451,7 @@
         </is>
       </c>
       <c r="B16" s="24" t="n">
-        <v>1141</v>
+        <v>1149</v>
       </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -18470,8 +18478,14 @@
       <c r="Y16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月17日</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="n">
+        <v>1412</v>
+      </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -33717,8 +33731,14 @@
       <c r="U16" s="18" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n"/>
-      <c r="B17" s="20" t="n"/>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月17日</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>3374</v>
+      </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-18 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5309,8 +5309,12 @@
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="21" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>1787</v>
+      </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -14021,8 +14025,12 @@
       <c r="G18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="21" t="n"/>
+      <c r="A19" s="23" t="n">
+        <v>45856</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>1221</v>
+      </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
       <c r="E19" s="13" t="n"/>
@@ -18451,7 +18459,7 @@
         </is>
       </c>
       <c r="B16" s="24" t="n">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="C16" s="15" t="n"/>
       <c r="D16" s="15" t="n"/>
@@ -18484,7 +18492,7 @@
         </is>
       </c>
       <c r="B17" s="24" t="n">
-        <v>1412</v>
+        <v>1418</v>
       </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -18511,8 +18519,14 @@
       <c r="Y17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月18日</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="n">
+        <v>1588</v>
+      </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>
@@ -33760,8 +33774,14 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n"/>
-      <c r="B18" s="20" t="n"/>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月18日</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="n">
+        <v>3305</v>
+      </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
       <c r="E18" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-20 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5326,8 +5326,12 @@
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="21" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>1783</v>
+      </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -5339,8 +5343,12 @@
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="21" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>935</v>
+      </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -14038,8 +14046,12 @@
       <c r="G19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="21" t="n"/>
+      <c r="A20" s="23" t="n">
+        <v>45857</v>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>1928</v>
+      </c>
       <c r="C20" s="13" t="n"/>
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -14047,8 +14059,12 @@
       <c r="G20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="21" t="n"/>
+      <c r="A21" s="23" t="n">
+        <v>45858</v>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>1795</v>
+      </c>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="13" t="n"/>
@@ -17963,7 +17979,7 @@
           <t>2026年7月1日</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n">
+      <c r="B1" s="20" t="n">
         <v>1132</v>
       </c>
       <c r="C1" s="14" t="n"/>
@@ -17996,7 +18012,7 @@
           <t>2026年7月2日</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="20" t="n">
         <v>884</v>
       </c>
       <c r="C2" s="15" t="n"/>
@@ -18029,7 +18045,7 @@
           <t>2026年7月3日</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="20" t="n">
         <v>963</v>
       </c>
       <c r="C3" s="17" t="n"/>
@@ -18062,7 +18078,7 @@
           <t>2026年7月4日</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="20" t="n">
         <v>1339</v>
       </c>
       <c r="C4" s="15" t="n"/>
@@ -18095,7 +18111,7 @@
           <t>2026年7月5日</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="20" t="n">
         <v>1754</v>
       </c>
       <c r="C5" s="15" t="n"/>
@@ -18128,7 +18144,7 @@
           <t>2026年7月6日</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="20" t="n">
         <v>1067</v>
       </c>
       <c r="C6" s="15" t="n"/>
@@ -18161,7 +18177,7 @@
           <t>2026年7月7日</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="20" t="n">
         <v>1034</v>
       </c>
       <c r="C7" s="15" t="n"/>
@@ -18194,7 +18210,7 @@
           <t>2026年7月8日</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="20" t="n">
         <v>1034</v>
       </c>
       <c r="C8" s="15" t="n"/>
@@ -18227,7 +18243,7 @@
           <t>2026年7月9日</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="20" t="n">
         <v>1092</v>
       </c>
       <c r="C9" s="15" t="n"/>
@@ -18260,7 +18276,7 @@
           <t>2026年7月10日</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n">
+      <c r="B10" s="20" t="n">
         <v>1048</v>
       </c>
       <c r="C10" s="15" t="n"/>
@@ -18293,7 +18309,7 @@
           <t>2026年7月11日</t>
         </is>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="20" t="n">
         <v>1451</v>
       </c>
       <c r="C11" s="15" t="n"/>
@@ -18326,7 +18342,7 @@
           <t>2026年7月12日</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="20" t="n">
         <v>1713</v>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -18359,7 +18375,7 @@
           <t>2026年7月13日</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="20" t="n">
         <v>1309</v>
       </c>
       <c r="C13" s="15" t="n"/>
@@ -18392,7 +18408,7 @@
           <t>2026年7月14日</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="20" t="n">
         <v>1035</v>
       </c>
       <c r="C14" s="15" t="n"/>
@@ -18425,7 +18441,7 @@
           <t>2026年7月15日</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="20" t="n">
         <v>1081</v>
       </c>
       <c r="C15" s="15" t="n"/>
@@ -18458,7 +18474,7 @@
           <t>2026年7月16日</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="20" t="n">
         <v>1151</v>
       </c>
       <c r="C16" s="15" t="n"/>
@@ -18491,8 +18507,8 @@
           <t>2026年7月17日</t>
         </is>
       </c>
-      <c r="B17" s="24" t="n">
-        <v>1418</v>
+      <c r="B17" s="20" t="n">
+        <v>1430</v>
       </c>
       <c r="C17" s="15" t="n"/>
       <c r="D17" s="15" t="n"/>
@@ -18524,8 +18540,8 @@
           <t>2026年7月18日</t>
         </is>
       </c>
-      <c r="B18" s="24" t="n">
-        <v>1588</v>
+      <c r="B18" s="20" t="n">
+        <v>1606</v>
       </c>
       <c r="C18" s="15" t="n"/>
       <c r="D18" s="15" t="n"/>
@@ -18552,8 +18568,14 @@
       <c r="Y18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月19日</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>1910</v>
+      </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -18579,8 +18601,14 @@
       <c r="Y19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月20日</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>1342</v>
+      </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>
@@ -33803,8 +33831,14 @@
       <c r="U18" s="15" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="20" t="n"/>
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月19日</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>6804</v>
+      </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -33826,8 +33860,14 @@
       <c r="U19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="n"/>
-      <c r="B20" s="20" t="n"/>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月20日</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>6135</v>
+      </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-21 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5360,8 +5360,12 @@
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="21" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>970</v>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -14072,8 +14076,12 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="21" t="n"/>
+      <c r="A22" s="23" t="n">
+        <v>45859</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>1150</v>
+      </c>
       <c r="C22" s="13" t="n"/>
       <c r="D22" s="13" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -18574,7 +18582,7 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>1910</v>
+        <v>1913</v>
       </c>
       <c r="C19" s="15" t="n"/>
       <c r="D19" s="17" t="n"/>
@@ -18607,7 +18615,7 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>1342</v>
+        <v>1357</v>
       </c>
       <c r="C20" s="15" t="n"/>
       <c r="D20" s="15" t="n"/>
@@ -18634,8 +18642,14 @@
       <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月21日</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>1317</v>
+      </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -33889,8 +33903,14 @@
       <c r="U20" s="18" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="20" t="n"/>
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月21日</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>5229</v>
+      </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-22 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5377,8 +5377,12 @@
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="21" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>1050</v>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -14089,8 +14093,12 @@
       <c r="G22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="21" t="n"/>
+      <c r="A23" s="23" t="n">
+        <v>45860</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>1159</v>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
@@ -18648,7 +18656,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>1317</v>
+        <v>1326</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18675,8 +18683,14 @@
       <c r="Y21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月22日</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>1365</v>
+      </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>
@@ -33932,8 +33946,14 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="n"/>
-      <c r="B22" s="20" t="n"/>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月22日</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>4810</v>
+      </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
       <c r="E22" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-23 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5394,8 +5394,12 @@
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="21" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>1103</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -14106,8 +14110,12 @@
       <c r="G23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="21" t="n"/>
+      <c r="A24" s="23" t="n">
+        <v>45861</v>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>1249</v>
+      </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -18656,7 +18664,7 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>1326</v>
+        <v>1328</v>
       </c>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="15" t="n"/>
@@ -18689,7 +18697,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>1365</v>
+        <v>1377</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18716,8 +18724,14 @@
       <c r="Y22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>1354</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -33975,8 +33989,14 @@
       <c r="U22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="n"/>
-      <c r="B23" s="20" t="n"/>
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月23日</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>5576</v>
+      </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
       <c r="E23" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-24 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5398,7 +5398,7 @@
         <v>46226</v>
       </c>
       <c r="B24" s="21" t="n">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
@@ -5411,8 +5411,12 @@
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="21" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>1288</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -14123,8 +14127,12 @@
       <c r="G24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="21" t="n"/>
+      <c r="A25" s="23" t="n">
+        <v>45862</v>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>1237</v>
+      </c>
       <c r="C25" s="13" t="n"/>
       <c r="D25" s="13" t="n"/>
       <c r="E25" s="13" t="n"/>
@@ -18697,7 +18705,7 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>1377</v>
+        <v>1380</v>
       </c>
       <c r="C22" s="15" t="n"/>
       <c r="D22" s="15" t="n"/>
@@ -18730,7 +18738,7 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>1354</v>
+        <v>1360</v>
       </c>
       <c r="C23" s="15" t="n"/>
       <c r="D23" s="15" t="n"/>
@@ -18757,8 +18765,14 @@
       <c r="Y23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>1430</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -34018,8 +34032,14 @@
       <c r="U23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="20" t="n"/>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月24日</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="n">
+        <v>4655</v>
+      </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
       <c r="E24" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-25 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5428,8 +5428,12 @@
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="21" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>2036</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -14140,8 +14144,12 @@
       <c r="G25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="21" t="n"/>
+      <c r="A26" s="23" t="n">
+        <v>45863</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>1383</v>
+      </c>
       <c r="C26" s="13" t="n"/>
       <c r="D26" s="13" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -18771,7 +18779,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18798,8 +18806,14 @@
       <c r="Y24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>1631</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -34061,8 +34075,14 @@
       <c r="U24" s="18" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="20" t="n"/>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月25日</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>5348</v>
+      </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
       <c r="E25" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-26 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5445,8 +5445,12 @@
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="21" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>1829</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -14157,8 +14161,12 @@
       <c r="G26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="21" t="n"/>
+      <c r="A27" s="23" t="n">
+        <v>45864</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>2049</v>
+      </c>
       <c r="C27" s="13" t="n"/>
       <c r="D27" s="13" t="n"/>
       <c r="E27" s="13" t="n"/>
@@ -18779,7 +18787,7 @@
         </is>
       </c>
       <c r="B24" s="20" t="n">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="15" t="n"/>
@@ -18812,7 +18820,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1631</v>
+        <v>1642</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18839,8 +18847,14 @@
       <c r="Y25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>1964</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>
@@ -34104,8 +34118,14 @@
       <c r="U25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="20" t="n"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月26日</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>6680</v>
+      </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
       <c r="E26" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-27 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5462,8 +5462,12 @@
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="21" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>1228</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -14174,8 +14178,12 @@
       <c r="G27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="21" t="n"/>
+      <c r="A28" s="23" t="n">
+        <v>45865</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>1952</v>
+      </c>
       <c r="C28" s="13" t="n"/>
       <c r="D28" s="13" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -18820,7 +18828,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1642</v>
+        <v>1655</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18853,7 +18861,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1964</v>
+        <v>1987</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18880,8 +18888,14 @@
       <c r="Y26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>1847</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -34147,8 +34161,14 @@
       <c r="U26" s="18" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="20" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月27日</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>8753</v>
+      </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="15" t="n"/>
       <c r="E27" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-28 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5313,7 +5313,7 @@
         <v>46221</v>
       </c>
       <c r="B19" s="21" t="n">
-        <v>1787</v>
+        <v>1786</v>
       </c>
       <c r="C19" s="13" t="n"/>
       <c r="D19" s="13" t="n"/>
@@ -5479,8 +5479,12 @@
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="21" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>1672</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -14191,8 +14195,12 @@
       <c r="G28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="21" t="n"/>
+      <c r="A29" s="23" t="n">
+        <v>45866</v>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>1259</v>
+      </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
@@ -18861,7 +18869,7 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>1987</v>
+        <v>1988</v>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="15" t="n"/>
@@ -18894,7 +18902,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>1847</v>
+        <v>1854</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18921,8 +18929,14 @@
       <c r="Y27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>2112</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>
@@ -34190,8 +34204,14 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="20" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月28日</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>5133</v>
+      </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
       <c r="E28" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-29 (manual-workbench)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5483,7 +5483,7 @@
         <v>46231</v>
       </c>
       <c r="B29" s="21" t="n">
-        <v>1672</v>
+        <v>1670</v>
       </c>
       <c r="C29" s="13" t="n"/>
       <c r="D29" s="13" t="n"/>
@@ -5496,8 +5496,12 @@
       <c r="K29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="21" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>1369</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -14208,8 +14212,12 @@
       <c r="G29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="21" t="n"/>
+      <c r="A30" s="23" t="n">
+        <v>45867</v>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>1340</v>
+      </c>
       <c r="C30" s="13" t="n"/>
       <c r="D30" s="13" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -18836,7 +18844,7 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>1655</v>
+        <v>1653</v>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="15" t="n"/>
@@ -18902,7 +18910,7 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>1854</v>
+        <v>1855</v>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="17" t="n"/>
@@ -18935,7 +18943,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>2112</v>
+        <v>2120</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18962,8 +18970,14 @@
       <c r="Y28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>2342</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -34233,8 +34247,14 @@
       <c r="U28" s="18" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="20" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月29日</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>5700</v>
+      </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="17" t="n"/>

</xml_diff>

<commit_message>
Auto publish dashboard data 2026-07-30 (interactive)
</commit_message>
<xml_diff>
--- a/data/source/NEV+ICE_ldai.xlsx
+++ b/data/source/NEV+ICE_ldai.xlsx
@@ -5513,8 +5513,12 @@
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="21" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1642</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -14225,8 +14229,12 @@
       <c r="G30" s="13" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="21" t="n"/>
+      <c r="A31" s="23" t="n">
+        <v>45868</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>1311</v>
+      </c>
       <c r="C31" s="13" t="n"/>
       <c r="D31" s="13" t="n"/>
       <c r="E31" s="13" t="n"/>
@@ -18943,7 +18951,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>2120</v>
+        <v>2123</v>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="15" t="n"/>
@@ -18976,7 +18984,7 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>2342</v>
+        <v>2359</v>
       </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="15" t="n"/>
@@ -19003,8 +19011,14 @@
       <c r="Y29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2026年7月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>3193</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>
@@ -34276,8 +34290,14 @@
       <c r="U29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="20" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>2025年7月30日</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>6791</v>
+      </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="15" t="n"/>
       <c r="E30" s="17" t="n"/>

</xml_diff>